<commit_message>
Frise et Tableau des courants, courant Mésopotamie antique, 4 boutons d'accueil, cartouches Frise/Tableau (histoires, recherche)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-courant-pensee-oriental.xlsx
+++ b/data/frise-courant-pensee-oriental.xlsx
@@ -2312,12 +2312,14 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="132.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="14" t="n">
-        <v>-1400</v>
+      <c r="A7" s="14">
+        <v>1090</v>
       </c>
       <c r="B7" s="14"/>
-      <c r="C7" s="14" t="s">
-        <v>32</v>
+      <c r="C7" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1090</t>
+        </is>
       </c>
       <c r="D7" s="15" t="s">
         <v>33</v>
@@ -2346,7 +2348,7 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t xml:space="preserve">orient-ancien;islam-juif;russe</t>
+          <t xml:space="preserve">islam-juif;russe</t>
         </is>
       </c>
     </row>
@@ -4511,18 +4513,49 @@
       </c>
     </row>
     <row r="73" customFormat="false" ht="316.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A73" s="0"/>
+      <c r="A73" s="0">
+        <v>-2600</v>
+      </c>
       <c r="B73" s="0"/>
-      <c r="C73" s="0"/>
-      <c r="D73" s="0"/>
-      <c r="E73" s="0"/>
+      <c r="C73" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2600 av. J.-C.</t>
+        </is>
+      </c>
+      <c r="D73" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mésopotamie antique</t>
+        </is>
+      </c>
+      <c r="E73" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/M%C3%A9sopotamie"  title=" Wikipedia"&gt;La pensée de la Mésopotamie antique&lt;/a&gt; est née entre le Tigre et l'Euphrate, chez les Sumériens puis les Akkadiens, les Babyloniens et les Assyriens, du IIIe millénaire avant J.-C. jusqu'à l'époque hellénistique. Elle ne s'exprime pas en traités mais dans des textes de sagesse, des hymnes, des épopées et des recueils de lois, écrits en cunéiforme sur des tablettes d'argile.&lt;/p&gt; &lt;p&gt;Les &lt;em&gt;Instructions de Shuruppak&lt;/em&gt;, parmi les plus anciens textes connus, donnent des conseils de prudence et de justice. Les hymnes d'Enheduanna, première autrice connue de l'histoire, font de la relation au divin une expérience personnelle. L'&lt;em&gt;Épopée de Gilgamesh&lt;/em&gt; médite sur l'amitié, la mort et la vanité de la quête d'immortalité, et le &lt;em&gt;Code de Hammurabi&lt;/em&gt; pense la justice royale et l'ordre de la cité.&lt;/p&gt; &lt;p&gt;D'autres textes posent déjà la question du mal : le &lt;em&gt;Ludlul bēl nēmeqi&lt;/em&gt; fait parler un juste éprouvé qui ne comprend pas pourquoi les dieux le frappent, et le &lt;em&gt;Dialogue du pessimisme&lt;/em&gt; met en scène, avec une ironie grinçante, un maître qui doute de toute action. La &lt;em&gt;Sagesse d'Ahiqar&lt;/em&gt; circulera ensuite dans tout le Proche-Orient, et Bérose transmettra au monde grec l'histoire et le savoir de Babylone.&lt;/p&gt; &lt;p&gt;Cette pensée, centrée sur l'ordre du monde, la justice, le destin et la condition humaine face aux dieux, a nourri les sagesses de la Bible et de la Grèce : elle est l'une des sources les plus anciennes de la réflexion philosophique.&lt;/p&gt;</t>
+        </is>
+      </c>
       <c r="F73" s="0"/>
       <c r="G73" s="0"/>
       <c r="H73" s="0"/>
       <c r="I73" s="0"/>
-      <c r="J73" s="0"/>
-      <c r="K73" s="0"/>
-      <c r="L73" s="0"/>
+      <c r="J73" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sagesses de Sumer et de Babylone sur la justice, le destin et la condition humaine.</t>
+        </is>
+      </c>
+      <c r="K73" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Théologie et spiritualité;Éthique;Philosophie politique</t>
+        </is>
+      </c>
+      <c r="L73" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ENHEDUANNA;GILGAMESH;HAMMURABI;SHURUPPAK</t>
+        </is>
+      </c>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">orient-ancien</t>
+        </is>
+      </c>
     </row>
     <row r="74" customFormat="false" ht="271.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="0"/>

</xml_diff>

<commit_message>
Accueil : nouveau sous-titre, « Ressource mise à jour 2026 » dans le footer ; Bienvenue : étape Philosophes d'aujourd'hui ; /frises/ : jalons limités à la tradition principale ; branche « langage » d'Apel, crédit Mésopotamie antique, date de Zarathoustra
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-courant-pensee-oriental.xlsx
+++ b/data/frise-courant-pensee-oriental.xlsx
@@ -2327,8 +2327,10 @@
       <c r="F5" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="G5" s="2" t="s">
-        <v>28</v>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mésopotamie : la 1ʳᵉ civilisation par les mondes de l’histoire</t>
+        </is>
       </c>
       <c r="J5" s="2" t="s">
         <v>29</v>

</xml_diff>

<commit_message>
Corée et Chine : 35 penseurs coréens intégrés à « orientaux » (textes enrichis), Jaegwon Kim aux Américains, 15 penseurs chinois modernes (Wang Fuzhi, Dai Zhen, Kang Youwei, Liang Qichao, Feng Youlan, Mou Zongsan…) ; courants Donghak, Minjung, Kaozheng, Nouveau confucianisme ; /frises/ : frises Indiens, Chinois, Coréens, Japonais ; époque moderne en 9 zones (Europe du Nord & centrale, Europe du Sud, Asie, Islam & pensées du Sud, Monde entier), époques des contemporains vers l'Antiquité ; traditions Occident (voie de la frise du monde), Pensée russe, Proche-Orient ancien ; courants : carte double Occident | Reste du monde ; accueil : devise en citation ; build-data ignore les vignettes absentes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-courant-pensee-oriental.xlsx
+++ b/data/frise-courant-pensee-oriental.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="606" uniqueCount="467">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="630" uniqueCount="485">
   <si>
     <t xml:space="preserve">FRISE DES COURANTS DE PENSÉE ORIENTALE — Données source</t>
   </si>
@@ -112,7 +112,7 @@
     <t xml:space="preserve">lrjRbKXjjeI</t>
   </si>
   <si>
-    <t xml:space="preserve">Mésopotamie : le 1ere civilisation par les mondes de l’histoire</t>
+    <t xml:space="preserve">Mésopotamie : la 1ʳᵉ civilisation par les mondes de l’histoire</t>
   </si>
   <si>
     <t xml:space="preserve">sagesses de Sumer et de Babylone sur la justice, le destin et la condition humaine.</t>
@@ -1382,6 +1382,60 @@
   </si>
   <si>
     <t xml:space="preserve">philosophie andine du bien-vivre en harmonie avec la nature, intégrée aux constitutions équatorienne et bolivienne.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Donghak</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Donghak" title=" Wikipedia"&gt; Le Donghak&lt;/a&gt; (« savoir de l’Orient ») est un mouvement de pensée religieuse et sociale fondé en 1860 par Choe Je-u, en réaction à la fois contre la pénétration du « savoir de l’Occident » (seohak, le catholicisme) et contre la crise d’une société Joseon minée par l’injustice et la misère paysanne.&lt;/p&gt;&lt;p&gt;Sa doctrine puise dans le confucianisme, le bouddhisme, le taoïsme et le chamanisme coréen. Son idée centrale, « l’être humain porte en lui le Ciel » (si cheonju), puis « l’être humain est le Ciel » (in nae cheon), fonde une égalité radicale entre tous, sans distinction de rang, de sexe ni de fortune.&lt;/p&gt;&lt;p&gt;Choe Je-u est exécuté en 1864 pour hérésie, mais le mouvement se diffuse dans les campagnes et inspire la grande révolte paysanne de 1894, dont la répression sert de prétexte à l’intervention chinoise et japonaise en Corée.&lt;/p&gt;&lt;p&gt;Renommé Cheondogyo (« religion de la Voie céleste ») en 1905, le Donghak joue un rôle majeur dans le mouvement d’indépendance du 1er mars 1919 et reste l’une des premières expressions d’une pensée moderne proprement coréenne.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mouvement religieux et social coréen fondé par Choe Je-u, affirmant que le Ciel réside en chaque être humain.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Minjung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;&lt;a href="https://en.wikipedia.org/wiki/Minjung_theology" title=" Wikipedia (en)"&gt; La pensée Minjung&lt;/a&gt; (« le peuple », au sens des masses opprimées) est un courant théologique et philosophique sud-coréen qui prend forme dans les années 1970, sous la dictature de Park Chung-hee, au sein des chrétiens engagés dans la lutte pour la démocratie et les droits des travailleurs.&lt;/p&gt;&lt;p&gt;Le minjung désigne ceux qui sont opprimés politiquement, exploités économiquement et tenus à l’écart de la culture. Pour Ahn Byung-mu et Suh Nam-dong, ce peuple souffrant n’est pas seulement l’objet de la compassion : il est le véritable sujet de l’histoire, et c’est dans ses luttes que se révèle le sens des Écritures.&lt;/p&gt;&lt;p&gt;La pensée Minjung s’appuie sur l’expérience coréenne du han, ce sentiment collectif de souffrance et de ressentiment accumulés, et sur les formes populaires comme le théâtre masqué. Elle trouve un précurseur dans la philosophie de la « graine » (ssial) de Ham Seok-heon, qui voyait dans le peuple le germe vivant de l’histoire.&lt;/p&gt;&lt;p&gt;Proche des théologies de la libération d’Amérique latine, elle a nourri le mouvement démocratique coréen des années 1980 et reste une référence majeure de la pensée sociale en Asie.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">courant théologique sud-coréen des années 1970 faisant du peuple opprimé le sujet de l’histoire.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Théologie et spiritualité ; Philosophie politique</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1650</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kaozheng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;&lt;a href="https://en.wikipedia.org/wiki/Kaozheng"  title=" Wikipedia (en)"&gt;Le Kaozheng&lt;/a&gt; (« recherche des preuves ») désigne le grand mouvement d’érudition qui domine la vie intellectuelle chinoise sous la dynastie Qing, du XVIIe au début du XIXe siècle. Né du traumatisme de la chute des Ming en 1644, il reproche au néoconfucianisme, et surtout à l’école de Wang Yangming, de s’être perdu dans des spéculations creuses sur l’esprit et le principe.&lt;/p&gt; &lt;p&gt;Contre ces « paroles vides », ses lettrés prônent une « étude solide » : retrouver le sens originel des classiques confucéens en les débarrassant des commentaires des Song, grâce à la philologie, à la phonétique ancienne, à l’épigraphie, à l’astronomie et aux mathématiques. Chaque affirmation doit reposer sur des preuves vérifiables, selon une méthode que les historiens ont souvent comparée à la critique historique européenne.&lt;/p&gt; &lt;p&gt;Fondé par Gu Yanwu, le mouvement atteint son apogée au XVIIIe siècle avec Dai Zhen et les savants des écoles de Suzhou et de l’Anhui, portés par les grands chantiers éditoriaux de l’empereur Qianlong. Mais la critique des textes conduit aussi à une critique des idées : Dai Zhen s’en sert pour contester une morale du principe opposée aux désirs.&lt;/p&gt; &lt;p&gt;Au début du XXe siècle, Liang Qichao et Hu Shi virent dans le Kaozheng une « renaissance » chinoise et une préfiguration de l’esprit scientifique moderne.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">école philologique des Qing, qui veut retrouver le sens originel des classiques par la critique des textes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GU Yanwu;DAI Zhen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1921</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nouveau confucianisme</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Nouveau_confucianisme"  title=" Wikipedia"&gt;Le nouveau confucianisme&lt;/a&gt; est un courant philosophique né dans les années 1920, en réaction au mouvement du 4 Mai 1919, qui rejetait la tradition confucéenne comme responsable du retard de la Chine. Ses penseurs veulent au contraire montrer que le confucianisme, repensé, peut répondre aux défis de la modernité.&lt;/p&gt; &lt;p&gt;Le livre de Liang Shuming sur les cultures d’Orient et d’Occident (1921) en marque le point de départ. Xiong Shili lui donne ensuite une métaphysique, inspirée du &lt;em&gt;Livre des mutations&lt;/em&gt; et d’une critique du bouddhisme, tandis que Feng Youlan relit Zhu Xi à l’aide de la logique moderne. Tous cherchent à concilier la sagesse morale chinoise avec la science et la démocratie venues d’Occident.&lt;/p&gt; &lt;p&gt;Après 1949, le courant se poursuit surtout à Hong Kong et à Taïwan, autour de Mou Zongsan, Tang Junyi et Xu Fuguan, qui publient en 1958 un &lt;em&gt;Manifeste pour une réévaluation de la culture chinoise&lt;/em&gt;. Mou Zongsan y engage un dialogue approfondi avec Kant pour fonder une « métaphysique morale ».&lt;/p&gt; &lt;p&gt;Une troisième génération, avec Tu Weiming ou Liu Shu-hsien, a porté ce courant dans les universités américaines, et il connaît depuis les années 1980 un important renouveau en Chine continentale.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">courant du XXe siècle qui renouvelle la pensée confucéenne pour répondre à la science et à la démocratie modernes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Métaphysique;Éthique</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LIANG Shuming;XIONG Shili;FENG Youlan;MOU Zongsan;TANG Junyi</t>
   </si>
   <si>
     <t xml:space="preserve">📖 MODE D'EMPLOI</t>
@@ -1809,7 +1863,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="31">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1819,10 +1873,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2190,7 +2240,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:XFD78"/>
+  <dimension ref="A1:N78"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6.53"/>
@@ -2205,68 +2255,68 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="2" width="19.61"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="2" width="25.04"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="2" width="10.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="3" width="10.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="2" width="10.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16383" style="1" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="4"/>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="I1" s="3"/>
     </row>
     <row r="2" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
-      <c r="I2" s="5"/>
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="4"/>
     </row>
     <row r="3" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="7" t="s">
+      <c r="G3" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="H3" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="I3" s="8" t="s">
+      <c r="I3" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="J3" s="9" t="s">
+      <c r="J3" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="K3" s="7" t="s">
+      <c r="K3" s="6" t="s">
         <v>12</v>
       </c>
       <c r="L3" s="2" t="s">
@@ -2280,34 +2330,34 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="174" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="10" t="n">
+      <c r="A4" s="9" t="n">
         <v>-2500</v>
       </c>
-      <c r="B4" s="10"/>
-      <c r="C4" s="10" t="s">
+      <c r="B4" s="9"/>
+      <c r="C4" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="D4" s="11" t="s">
+      <c r="D4" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="E4" s="12" t="s">
+      <c r="E4" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="F4" s="10" t="s">
+      <c r="F4" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="G4" s="12" t="s">
+      <c r="G4" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="H4" s="10"/>
-      <c r="I4" s="10"/>
+      <c r="H4" s="9"/>
+      <c r="I4" s="9"/>
       <c r="J4" s="2" t="s">
         <v>21</v>
       </c>
       <c r="K4" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M4" s="3" t="s">
+      <c r="M4" s="2" t="s">
         <v>23</v>
       </c>
     </row>
@@ -2318,7 +2368,7 @@
       <c r="C5" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D5" s="13" t="s">
+      <c r="D5" s="12" t="s">
         <v>25</v>
       </c>
       <c r="E5" s="2" t="s">
@@ -2327,10 +2377,8 @@
       <c r="F5" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Mésopotamie : la 1ʳᵉ civilisation par les mondes de l’histoire</t>
-        </is>
+      <c r="G5" s="2" t="s">
+        <v>28</v>
       </c>
       <c r="J5" s="2" t="s">
         <v>29</v>
@@ -2341,11 +2389,9 @@
       <c r="L5" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="M5" s="3" t="s">
+      <c r="M5" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="XFC5" s="0"/>
-      <c r="XFD5" s="0"/>
     </row>
     <row r="6" customFormat="false" ht="226.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="n">
@@ -2354,7 +2400,7 @@
       <c r="C6" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D6" s="14" t="s">
+      <c r="D6" s="13" t="s">
         <v>33</v>
       </c>
       <c r="E6" s="2" t="s">
@@ -2372,7 +2418,7 @@
       <c r="K6" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M6" s="3" t="s">
+      <c r="M6" s="2" t="s">
         <v>23</v>
       </c>
     </row>
@@ -2383,10 +2429,10 @@
       <c r="C7" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D7" s="14" t="s">
+      <c r="D7" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="E7" s="15" t="s">
+      <c r="E7" s="14" t="s">
         <v>39</v>
       </c>
       <c r="F7" s="1" t="s">
@@ -2395,48 +2441,48 @@
       <c r="G7" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="J7" s="15" t="s">
+      <c r="J7" s="14" t="s">
         <v>42</v>
       </c>
       <c r="K7" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M7" s="3" t="s">
+      <c r="M7" s="2" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="132.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="16" t="n">
+      <c r="A8" s="15" t="n">
         <v>1090</v>
       </c>
-      <c r="B8" s="16"/>
-      <c r="C8" s="16" t="s">
+      <c r="B8" s="15"/>
+      <c r="C8" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="D8" s="17" t="s">
+      <c r="D8" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="E8" s="18" t="s">
+      <c r="E8" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="F8" s="16" t="s">
+      <c r="F8" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="G8" s="18" t="s">
+      <c r="G8" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="H8" s="16"/>
-      <c r="I8" s="16"/>
+      <c r="H8" s="15"/>
+      <c r="I8" s="15"/>
       <c r="J8" s="2" t="s">
         <v>49</v>
       </c>
       <c r="K8" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M8" s="3" t="s">
+      <c r="M8" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="N8" s="0" t="s">
+      <c r="N8" s="1" t="s">
         <v>51</v>
       </c>
     </row>
@@ -2465,10 +2511,10 @@
       <c r="K9" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M9" s="3" t="s">
+      <c r="M9" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="N9" s="0" t="s">
+      <c r="N9" s="1" t="s">
         <v>23</v>
       </c>
     </row>
@@ -2497,42 +2543,42 @@
       <c r="K10" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M10" s="3" t="s">
+      <c r="M10" s="2" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="144.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="10" t="n">
+      <c r="A11" s="9" t="n">
         <v>-700</v>
       </c>
-      <c r="B11" s="10"/>
-      <c r="C11" s="10" t="s">
+      <c r="B11" s="9"/>
+      <c r="C11" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="D11" s="11" t="s">
+      <c r="D11" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="E11" s="12" t="s">
+      <c r="E11" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="F11" s="10" t="s">
+      <c r="F11" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="G11" s="12" t="s">
+      <c r="G11" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="H11" s="10"/>
-      <c r="I11" s="10"/>
+      <c r="H11" s="9"/>
+      <c r="I11" s="9"/>
       <c r="J11" s="2" t="s">
         <v>70</v>
       </c>
       <c r="K11" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M11" s="3" t="s">
+      <c r="M11" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="N11" s="0" t="s">
+      <c r="N11" s="1" t="s">
         <v>58</v>
       </c>
     </row>
@@ -2561,42 +2607,42 @@
       <c r="K12" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M12" s="3" t="s">
+      <c r="M12" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="N12" s="0" t="s">
+      <c r="N12" s="1" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="111.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="16" t="n">
+      <c r="A13" s="15" t="n">
         <v>-600</v>
       </c>
-      <c r="B13" s="16"/>
-      <c r="C13" s="16" t="s">
+      <c r="B13" s="15"/>
+      <c r="C13" s="15" t="s">
         <v>77</v>
       </c>
-      <c r="D13" s="17" t="s">
+      <c r="D13" s="16" t="s">
         <v>78</v>
       </c>
-      <c r="E13" s="18" t="s">
+      <c r="E13" s="17" t="s">
         <v>79</v>
       </c>
-      <c r="F13" s="16" t="s">
+      <c r="F13" s="15" t="s">
         <v>80</v>
       </c>
-      <c r="G13" s="18" t="s">
+      <c r="G13" s="17" t="s">
         <v>81</v>
       </c>
-      <c r="H13" s="16"/>
-      <c r="I13" s="16"/>
+      <c r="H13" s="15"/>
+      <c r="I13" s="15"/>
       <c r="J13" s="2" t="s">
         <v>82</v>
       </c>
       <c r="K13" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M13" s="3" t="s">
+      <c r="M13" s="2" t="s">
         <v>43</v>
       </c>
     </row>
@@ -2607,7 +2653,7 @@
       <c r="C14" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="D14" s="14" t="s">
+      <c r="D14" s="13" t="s">
         <v>83</v>
       </c>
       <c r="E14" s="2" t="s">
@@ -2625,7 +2671,7 @@
       <c r="K14" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="M14" s="3" t="s">
+      <c r="M14" s="2" t="s">
         <v>43</v>
       </c>
     </row>
@@ -2633,13 +2679,13 @@
       <c r="A15" s="1" t="n">
         <v>-550</v>
       </c>
-      <c r="C15" s="19" t="s">
+      <c r="C15" s="18" t="s">
         <v>89</v>
       </c>
-      <c r="D15" s="14" t="s">
+      <c r="D15" s="13" t="s">
         <v>90</v>
       </c>
-      <c r="E15" s="15" t="s">
+      <c r="E15" s="14" t="s">
         <v>91</v>
       </c>
       <c r="F15" s="1" t="s">
@@ -2648,77 +2694,77 @@
       <c r="G15" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="J15" s="15" t="s">
+      <c r="J15" s="14" t="s">
         <v>94</v>
       </c>
       <c r="K15" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M15" s="3" t="s">
+      <c r="M15" s="2" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="174" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="10" t="n">
+      <c r="A16" s="9" t="n">
         <v>-520</v>
       </c>
-      <c r="B16" s="10"/>
-      <c r="C16" s="10" t="s">
+      <c r="B16" s="9"/>
+      <c r="C16" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="D16" s="11" t="s">
+      <c r="D16" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="E16" s="12" t="s">
+      <c r="E16" s="11" t="s">
         <v>97</v>
       </c>
-      <c r="F16" s="10" t="s">
+      <c r="F16" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="G16" s="12" t="s">
+      <c r="G16" s="11" t="s">
         <v>99</v>
       </c>
-      <c r="H16" s="10"/>
-      <c r="I16" s="10"/>
+      <c r="H16" s="9"/>
+      <c r="I16" s="9"/>
       <c r="J16" s="2" t="s">
         <v>100</v>
       </c>
       <c r="K16" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M16" s="3" t="s">
+      <c r="M16" s="2" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="16" t="n">
+      <c r="A17" s="15" t="n">
         <v>-510</v>
       </c>
-      <c r="B17" s="16"/>
-      <c r="C17" s="16" t="s">
+      <c r="B17" s="15"/>
+      <c r="C17" s="15" t="s">
         <v>102</v>
       </c>
-      <c r="D17" s="17" t="s">
+      <c r="D17" s="16" t="s">
         <v>103</v>
       </c>
-      <c r="E17" s="18" t="s">
+      <c r="E17" s="17" t="s">
         <v>104</v>
       </c>
-      <c r="F17" s="16" t="s">
+      <c r="F17" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="G17" s="18" t="s">
+      <c r="G17" s="17" t="s">
         <v>106</v>
       </c>
-      <c r="H17" s="16"/>
-      <c r="I17" s="16"/>
+      <c r="H17" s="15"/>
+      <c r="I17" s="15"/>
       <c r="J17" s="2" t="s">
         <v>107</v>
       </c>
       <c r="K17" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="M17" s="3" t="s">
+      <c r="M17" s="2" t="s">
         <v>64</v>
       </c>
     </row>
@@ -2729,7 +2775,7 @@
       <c r="C18" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="D18" s="14" t="s">
+      <c r="D18" s="13" t="s">
         <v>110</v>
       </c>
       <c r="E18" s="2" t="s">
@@ -2747,7 +2793,7 @@
       <c r="K18" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M18" s="3" t="s">
+      <c r="M18" s="2" t="s">
         <v>43</v>
       </c>
     </row>
@@ -2758,7 +2804,7 @@
       <c r="C19" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="D19" s="14" t="s">
+      <c r="D19" s="13" t="s">
         <v>115</v>
       </c>
       <c r="E19" s="2" t="s">
@@ -2776,170 +2822,170 @@
       <c r="K19" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="M19" s="3" t="s">
+      <c r="M19" s="2" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="138.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="10" t="n">
+      <c r="A20" s="9" t="n">
         <v>-500</v>
       </c>
-      <c r="B20" s="10"/>
-      <c r="C20" s="10" t="s">
+      <c r="B20" s="9"/>
+      <c r="C20" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="D20" s="11" t="s">
+      <c r="D20" s="10" t="s">
         <v>121</v>
       </c>
-      <c r="E20" s="12" t="s">
+      <c r="E20" s="11" t="s">
         <v>122</v>
       </c>
-      <c r="F20" s="10" t="s">
+      <c r="F20" s="9" t="s">
         <v>123</v>
       </c>
-      <c r="G20" s="12" t="s">
+      <c r="G20" s="11" t="s">
         <v>124</v>
       </c>
-      <c r="H20" s="10"/>
-      <c r="I20" s="10"/>
+      <c r="H20" s="9"/>
+      <c r="I20" s="9"/>
       <c r="J20" s="2" t="s">
         <v>125</v>
       </c>
       <c r="K20" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M20" s="3" t="s">
+      <c r="M20" s="2" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="10" t="n">
+      <c r="A21" s="9" t="n">
         <v>-470</v>
       </c>
-      <c r="B21" s="10"/>
-      <c r="C21" s="10" t="s">
+      <c r="B21" s="9"/>
+      <c r="C21" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="D21" s="11" t="s">
+      <c r="D21" s="10" t="s">
         <v>127</v>
       </c>
-      <c r="E21" s="12" t="s">
+      <c r="E21" s="11" t="s">
         <v>128</v>
       </c>
-      <c r="F21" s="10" t="s">
+      <c r="F21" s="9" t="s">
         <v>129</v>
       </c>
-      <c r="G21" s="12" t="s">
+      <c r="G21" s="11" t="s">
         <v>130</v>
       </c>
-      <c r="H21" s="10"/>
-      <c r="I21" s="10"/>
+      <c r="H21" s="9"/>
+      <c r="I21" s="9"/>
       <c r="J21" s="2" t="s">
         <v>131</v>
       </c>
       <c r="K21" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M21" s="3" t="s">
+      <c r="M21" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="N21" s="0" t="s">
+      <c r="N21" s="1" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="16" t="n">
+      <c r="A22" s="15" t="n">
         <v>-450</v>
       </c>
-      <c r="B22" s="16"/>
-      <c r="C22" s="16" t="s">
+      <c r="B22" s="15"/>
+      <c r="C22" s="15" t="s">
         <v>132</v>
       </c>
-      <c r="D22" s="17" t="s">
+      <c r="D22" s="16" t="s">
         <v>133</v>
       </c>
-      <c r="E22" s="18" t="s">
+      <c r="E22" s="17" t="s">
         <v>134</v>
       </c>
-      <c r="F22" s="16" t="s">
+      <c r="F22" s="15" t="s">
         <v>135</v>
       </c>
-      <c r="G22" s="18" t="s">
+      <c r="G22" s="17" t="s">
         <v>136</v>
       </c>
-      <c r="H22" s="16"/>
-      <c r="I22" s="16"/>
+      <c r="H22" s="15"/>
+      <c r="I22" s="15"/>
       <c r="J22" s="2" t="s">
         <v>137</v>
       </c>
       <c r="K22" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="M22" s="3" t="s">
+      <c r="M22" s="2" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="10" t="n">
+      <c r="A23" s="9" t="n">
         <v>-410</v>
       </c>
-      <c r="B23" s="10"/>
-      <c r="C23" s="10" t="s">
+      <c r="B23" s="9"/>
+      <c r="C23" s="9" t="s">
         <v>138</v>
       </c>
-      <c r="D23" s="11" t="s">
+      <c r="D23" s="10" t="s">
         <v>139</v>
       </c>
-      <c r="E23" s="12" t="s">
+      <c r="E23" s="11" t="s">
         <v>140</v>
       </c>
-      <c r="F23" s="10" t="s">
+      <c r="F23" s="9" t="s">
         <v>141</v>
       </c>
-      <c r="G23" s="12" t="s">
+      <c r="G23" s="11" t="s">
         <v>142</v>
       </c>
-      <c r="H23" s="10"/>
-      <c r="I23" s="10"/>
+      <c r="H23" s="9"/>
+      <c r="I23" s="9"/>
       <c r="J23" s="2" t="s">
         <v>143</v>
       </c>
       <c r="K23" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M23" s="3" t="s">
+      <c r="M23" s="2" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="16" t="n">
+      <c r="A24" s="15" t="n">
         <v>-400</v>
       </c>
-      <c r="B24" s="16"/>
-      <c r="C24" s="16" t="s">
+      <c r="B24" s="15"/>
+      <c r="C24" s="15" t="s">
         <v>144</v>
       </c>
-      <c r="D24" s="17" t="s">
+      <c r="D24" s="16" t="s">
         <v>145</v>
       </c>
-      <c r="E24" s="18" t="s">
+      <c r="E24" s="17" t="s">
         <v>146</v>
       </c>
-      <c r="F24" s="16" t="s">
+      <c r="F24" s="15" t="s">
         <v>147</v>
       </c>
-      <c r="G24" s="18" t="s">
+      <c r="G24" s="17" t="s">
         <v>148</v>
       </c>
-      <c r="H24" s="16"/>
-      <c r="I24" s="16"/>
+      <c r="H24" s="15"/>
+      <c r="I24" s="15"/>
       <c r="J24" s="2" t="s">
         <v>149</v>
       </c>
       <c r="K24" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M24" s="3" t="s">
+      <c r="M24" s="2" t="s">
         <v>101</v>
       </c>
     </row>
@@ -2950,7 +2996,7 @@
       <c r="C25" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="D25" s="14" t="s">
+      <c r="D25" s="13" t="s">
         <v>150</v>
       </c>
       <c r="E25" s="2" t="s">
@@ -2968,39 +3014,39 @@
       <c r="K25" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="M25" s="3" t="s">
+      <c r="M25" s="2" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="10" t="n">
+      <c r="A26" s="9" t="n">
         <v>-350</v>
       </c>
-      <c r="B26" s="10"/>
-      <c r="C26" s="10" t="s">
+      <c r="B26" s="9"/>
+      <c r="C26" s="9" t="s">
         <v>156</v>
       </c>
-      <c r="D26" s="11" t="s">
+      <c r="D26" s="10" t="s">
         <v>157</v>
       </c>
-      <c r="E26" s="20" t="s">
+      <c r="E26" s="19" t="s">
         <v>158</v>
       </c>
-      <c r="F26" s="10" t="s">
+      <c r="F26" s="9" t="s">
         <v>159</v>
       </c>
-      <c r="G26" s="12" t="s">
+      <c r="G26" s="11" t="s">
         <v>160</v>
       </c>
-      <c r="H26" s="10"/>
-      <c r="I26" s="10"/>
+      <c r="H26" s="9"/>
+      <c r="I26" s="9"/>
       <c r="J26" s="2" t="s">
         <v>161</v>
       </c>
       <c r="K26" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="M26" s="3" t="s">
+      <c r="M26" s="2" t="s">
         <v>43</v>
       </c>
     </row>
@@ -3011,7 +3057,7 @@
       <c r="C27" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="D27" s="14" t="s">
+      <c r="D27" s="13" t="s">
         <v>162</v>
       </c>
       <c r="E27" s="2" t="s">
@@ -3029,7 +3075,7 @@
       <c r="K27" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="M27" s="3" t="s">
+      <c r="M27" s="2" t="s">
         <v>101</v>
       </c>
     </row>
@@ -3040,7 +3086,7 @@
       <c r="C28" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="D28" s="14" t="s">
+      <c r="D28" s="13" t="s">
         <v>168</v>
       </c>
       <c r="E28" s="2" t="s">
@@ -3058,71 +3104,71 @@
       <c r="K28" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M28" s="3" t="s">
+      <c r="M28" s="2" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="16" t="n">
+      <c r="A29" s="15" t="n">
         <v>-150</v>
       </c>
-      <c r="B29" s="16"/>
-      <c r="C29" s="16" t="s">
+      <c r="B29" s="15"/>
+      <c r="C29" s="15" t="s">
         <v>173</v>
       </c>
-      <c r="D29" s="17" t="s">
+      <c r="D29" s="16" t="s">
         <v>174</v>
       </c>
-      <c r="E29" s="21" t="s">
+      <c r="E29" s="20" t="s">
         <v>175</v>
       </c>
-      <c r="F29" s="16" t="s">
+      <c r="F29" s="15" t="s">
         <v>176</v>
       </c>
-      <c r="G29" s="18" t="s">
+      <c r="G29" s="17" t="s">
         <v>177</v>
       </c>
-      <c r="H29" s="16"/>
-      <c r="I29" s="16"/>
+      <c r="H29" s="15"/>
+      <c r="I29" s="15"/>
       <c r="J29" s="2" t="s">
         <v>178</v>
       </c>
       <c r="K29" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="M29" s="3" t="s">
+      <c r="M29" s="2" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="10" t="n">
+      <c r="A30" s="9" t="n">
         <v>-100</v>
       </c>
-      <c r="B30" s="10"/>
-      <c r="C30" s="10" t="s">
+      <c r="B30" s="9"/>
+      <c r="C30" s="9" t="s">
         <v>179</v>
       </c>
-      <c r="D30" s="11" t="s">
+      <c r="D30" s="10" t="s">
         <v>180</v>
       </c>
-      <c r="E30" s="20" t="s">
+      <c r="E30" s="19" t="s">
         <v>181</v>
       </c>
-      <c r="F30" s="10" t="s">
+      <c r="F30" s="9" t="s">
         <v>182</v>
       </c>
-      <c r="G30" s="12" t="s">
+      <c r="G30" s="11" t="s">
         <v>183</v>
       </c>
-      <c r="H30" s="10"/>
-      <c r="I30" s="10"/>
+      <c r="H30" s="9"/>
+      <c r="I30" s="9"/>
       <c r="J30" s="2" t="s">
         <v>184</v>
       </c>
       <c r="K30" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="M30" s="3" t="s">
+      <c r="M30" s="2" t="s">
         <v>43</v>
       </c>
     </row>
@@ -3133,7 +3179,7 @@
       <c r="C31" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="D31" s="14" t="s">
+      <c r="D31" s="13" t="s">
         <v>185</v>
       </c>
       <c r="E31" s="2" t="s">
@@ -3151,74 +3197,74 @@
       <c r="K31" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M31" s="3" t="s">
+      <c r="M31" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="N31" s="0" t="s">
+      <c r="N31" s="1" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="16" t="n">
+      <c r="A32" s="15" t="n">
         <v>250</v>
       </c>
-      <c r="B32" s="16"/>
-      <c r="C32" s="16" t="s">
+      <c r="B32" s="15"/>
+      <c r="C32" s="15" t="s">
         <v>190</v>
       </c>
-      <c r="D32" s="17" t="s">
+      <c r="D32" s="16" t="s">
         <v>191</v>
       </c>
-      <c r="E32" s="21" t="s">
+      <c r="E32" s="20" t="s">
         <v>192</v>
       </c>
-      <c r="F32" s="16" t="s">
+      <c r="F32" s="15" t="s">
         <v>193</v>
       </c>
-      <c r="G32" s="18" t="s">
+      <c r="G32" s="17" t="s">
         <v>194</v>
       </c>
-      <c r="H32" s="16"/>
-      <c r="I32" s="16"/>
+      <c r="H32" s="15"/>
+      <c r="I32" s="15"/>
       <c r="J32" s="2" t="s">
         <v>195</v>
       </c>
       <c r="K32" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="M32" s="3" t="s">
+      <c r="M32" s="2" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="108.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="16" t="n">
+      <c r="A33" s="15" t="n">
         <v>450</v>
       </c>
-      <c r="B33" s="16"/>
-      <c r="C33" s="16" t="n">
+      <c r="B33" s="15"/>
+      <c r="C33" s="15" t="n">
         <v>450</v>
       </c>
-      <c r="D33" s="17" t="s">
+      <c r="D33" s="16" t="s">
         <v>197</v>
       </c>
-      <c r="E33" s="22" t="s">
+      <c r="E33" s="21" t="s">
         <v>198</v>
       </c>
-      <c r="F33" s="16" t="s">
+      <c r="F33" s="15" t="s">
         <v>199</v>
       </c>
-      <c r="G33" s="18" t="s">
+      <c r="G33" s="17" t="s">
         <v>200</v>
       </c>
-      <c r="H33" s="16"/>
-      <c r="I33" s="16"/>
+      <c r="H33" s="15"/>
+      <c r="I33" s="15"/>
       <c r="J33" s="2" t="s">
         <v>201</v>
       </c>
       <c r="K33" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M33" s="3" t="s">
+      <c r="M33" s="2" t="s">
         <v>23</v>
       </c>
     </row>
@@ -3229,7 +3275,7 @@
       <c r="C34" s="1" t="n">
         <v>500</v>
       </c>
-      <c r="D34" s="14" t="s">
+      <c r="D34" s="13" t="s">
         <v>202</v>
       </c>
       <c r="E34" s="2" t="s">
@@ -3247,7 +3293,7 @@
       <c r="K34" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M34" s="3" t="s">
+      <c r="M34" s="2" t="s">
         <v>101</v>
       </c>
     </row>
@@ -3258,7 +3304,7 @@
       <c r="C35" s="1" t="n">
         <v>700</v>
       </c>
-      <c r="D35" s="14" t="s">
+      <c r="D35" s="13" t="s">
         <v>207</v>
       </c>
       <c r="E35" s="2" t="s">
@@ -3276,10 +3322,10 @@
       <c r="K35" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M35" s="3" t="s">
+      <c r="M35" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="N35" s="0" t="s">
+      <c r="N35" s="1" t="s">
         <v>101</v>
       </c>
     </row>
@@ -3290,10 +3336,10 @@
       <c r="C36" s="1" t="n">
         <v>720</v>
       </c>
-      <c r="D36" s="14" t="s">
+      <c r="D36" s="13" t="s">
         <v>212</v>
       </c>
-      <c r="E36" s="23" t="s">
+      <c r="E36" s="22" t="s">
         <v>213</v>
       </c>
       <c r="F36" s="1" t="s">
@@ -3302,77 +3348,77 @@
       <c r="G36" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="J36" s="23" t="s">
+      <c r="J36" s="22" t="s">
         <v>216</v>
       </c>
       <c r="K36" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M36" s="3" t="s">
+      <c r="M36" s="2" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="306.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="10" t="n">
+      <c r="A37" s="9" t="n">
         <v>750</v>
       </c>
-      <c r="B37" s="10"/>
-      <c r="C37" s="10" t="s">
+      <c r="B37" s="9"/>
+      <c r="C37" s="9" t="s">
         <v>217</v>
       </c>
-      <c r="D37" s="11" t="s">
+      <c r="D37" s="10" t="s">
         <v>218</v>
       </c>
-      <c r="E37" s="12" t="s">
+      <c r="E37" s="11" t="s">
         <v>219</v>
       </c>
-      <c r="F37" s="10" t="s">
+      <c r="F37" s="9" t="s">
         <v>220</v>
       </c>
-      <c r="G37" s="12" t="s">
+      <c r="G37" s="11" t="s">
         <v>221</v>
       </c>
-      <c r="H37" s="10"/>
-      <c r="I37" s="10"/>
+      <c r="H37" s="9"/>
+      <c r="I37" s="9"/>
       <c r="J37" s="2" t="s">
         <v>222</v>
       </c>
       <c r="K37" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M37" s="3" t="s">
+      <c r="M37" s="2" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="115.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="16" t="n">
+      <c r="A38" s="15" t="n">
         <v>750</v>
       </c>
-      <c r="B38" s="16"/>
-      <c r="C38" s="16" t="s">
+      <c r="B38" s="15"/>
+      <c r="C38" s="15" t="s">
         <v>217</v>
       </c>
-      <c r="D38" s="17" t="s">
+      <c r="D38" s="16" t="s">
         <v>223</v>
       </c>
-      <c r="E38" s="21" t="s">
+      <c r="E38" s="20" t="s">
         <v>224</v>
       </c>
-      <c r="F38" s="16" t="s">
+      <c r="F38" s="15" t="s">
         <v>225</v>
       </c>
-      <c r="G38" s="18" t="s">
+      <c r="G38" s="17" t="s">
         <v>226</v>
       </c>
-      <c r="H38" s="16"/>
-      <c r="I38" s="16"/>
+      <c r="H38" s="15"/>
+      <c r="I38" s="15"/>
       <c r="J38" s="2" t="s">
         <v>227</v>
       </c>
       <c r="K38" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="M38" s="3" t="s">
+      <c r="M38" s="2" t="s">
         <v>43</v>
       </c>
     </row>
@@ -3383,7 +3429,7 @@
       <c r="C39" s="1" t="n">
         <v>800</v>
       </c>
-      <c r="D39" s="14" t="s">
+      <c r="D39" s="13" t="s">
         <v>228</v>
       </c>
       <c r="E39" s="2" t="s">
@@ -3401,42 +3447,42 @@
       <c r="K39" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="M39" s="3" t="s">
+      <c r="M39" s="2" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="10" t="n">
+      <c r="A40" s="9" t="n">
         <v>820</v>
       </c>
-      <c r="B40" s="10"/>
-      <c r="C40" s="10" t="s">
+      <c r="B40" s="9"/>
+      <c r="C40" s="9" t="s">
         <v>233</v>
       </c>
-      <c r="D40" s="11" t="s">
+      <c r="D40" s="10" t="s">
         <v>234</v>
       </c>
-      <c r="E40" s="12" t="s">
+      <c r="E40" s="11" t="s">
         <v>235</v>
       </c>
-      <c r="F40" s="10" t="s">
+      <c r="F40" s="9" t="s">
         <v>236</v>
       </c>
-      <c r="G40" s="12" t="s">
+      <c r="G40" s="11" t="s">
         <v>237</v>
       </c>
-      <c r="H40" s="10"/>
-      <c r="I40" s="10"/>
+      <c r="H40" s="9"/>
+      <c r="I40" s="9"/>
       <c r="J40" s="2" t="s">
         <v>238</v>
       </c>
       <c r="K40" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M40" s="3" t="s">
+      <c r="M40" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="N40" s="0" t="s">
+      <c r="N40" s="1" t="s">
         <v>239</v>
       </c>
     </row>
@@ -3447,7 +3493,7 @@
       <c r="C41" s="1" t="n">
         <v>850</v>
       </c>
-      <c r="D41" s="14" t="s">
+      <c r="D41" s="13" t="s">
         <v>240</v>
       </c>
       <c r="E41" s="2" t="s">
@@ -3465,39 +3511,39 @@
       <c r="K41" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M41" s="3" t="s">
+      <c r="M41" s="2" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="290.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="16" t="n">
+      <c r="A42" s="15" t="n">
         <v>890</v>
       </c>
-      <c r="B42" s="16"/>
-      <c r="C42" s="16" t="s">
+      <c r="B42" s="15"/>
+      <c r="C42" s="15" t="s">
         <v>245</v>
       </c>
-      <c r="D42" s="17" t="s">
+      <c r="D42" s="16" t="s">
         <v>246</v>
       </c>
-      <c r="E42" s="18" t="s">
+      <c r="E42" s="17" t="s">
         <v>247</v>
       </c>
-      <c r="F42" s="16" t="s">
+      <c r="F42" s="15" t="s">
         <v>248</v>
       </c>
-      <c r="G42" s="18" t="s">
+      <c r="G42" s="17" t="s">
         <v>249</v>
       </c>
-      <c r="H42" s="16"/>
-      <c r="I42" s="16"/>
+      <c r="H42" s="15"/>
+      <c r="I42" s="15"/>
       <c r="J42" s="2" t="s">
         <v>250</v>
       </c>
       <c r="K42" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M42" s="3" t="s">
+      <c r="M42" s="2" t="s">
         <v>58</v>
       </c>
     </row>
@@ -3508,7 +3554,7 @@
       <c r="C43" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="D43" s="14" t="s">
+      <c r="D43" s="13" t="s">
         <v>252</v>
       </c>
       <c r="E43" s="2" t="s">
@@ -3540,7 +3586,7 @@
       <c r="C44" s="1" t="n">
         <v>1000</v>
       </c>
-      <c r="D44" s="14" t="s">
+      <c r="D44" s="13" t="s">
         <v>259</v>
       </c>
       <c r="E44" s="2" t="s">
@@ -3558,7 +3604,7 @@
       <c r="K44" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M44" s="3" t="s">
+      <c r="M44" s="2" t="s">
         <v>101</v>
       </c>
     </row>
@@ -3569,7 +3615,7 @@
       <c r="C45" s="1" t="n">
         <v>1000</v>
       </c>
-      <c r="D45" s="14" t="s">
+      <c r="D45" s="13" t="s">
         <v>264</v>
       </c>
       <c r="E45" s="2" t="s">
@@ -3587,7 +3633,7 @@
       <c r="K45" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M45" s="3" t="s">
+      <c r="M45" s="2" t="s">
         <v>64</v>
       </c>
     </row>
@@ -3598,7 +3644,7 @@
       <c r="C46" s="1" t="n">
         <v>1150</v>
       </c>
-      <c r="D46" s="14" t="s">
+      <c r="D46" s="13" t="s">
         <v>269</v>
       </c>
       <c r="E46" s="2" t="s">
@@ -3616,42 +3662,42 @@
       <c r="K46" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M46" s="3" t="s">
+      <c r="M46" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="N46" s="0" t="s">
+      <c r="N46" s="1" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="219" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="10" t="n">
+      <c r="A47" s="9" t="n">
         <v>1150</v>
       </c>
-      <c r="B47" s="10"/>
-      <c r="C47" s="10" t="s">
+      <c r="B47" s="9"/>
+      <c r="C47" s="9" t="s">
         <v>274</v>
       </c>
-      <c r="D47" s="11" t="s">
+      <c r="D47" s="10" t="s">
         <v>275</v>
       </c>
-      <c r="E47" s="24" t="s">
+      <c r="E47" s="23" t="s">
         <v>276</v>
       </c>
-      <c r="F47" s="10" t="s">
+      <c r="F47" s="9" t="s">
         <v>277</v>
       </c>
-      <c r="G47" s="12" t="s">
+      <c r="G47" s="11" t="s">
         <v>278</v>
       </c>
-      <c r="H47" s="10"/>
-      <c r="I47" s="10"/>
+      <c r="H47" s="9"/>
+      <c r="I47" s="9"/>
       <c r="J47" s="2" t="s">
         <v>279</v>
       </c>
       <c r="K47" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M47" s="3" t="s">
+      <c r="M47" s="2" t="s">
         <v>101</v>
       </c>
     </row>
@@ -3662,7 +3708,7 @@
       <c r="C48" s="1" t="n">
         <v>1200</v>
       </c>
-      <c r="D48" s="14" t="s">
+      <c r="D48" s="13" t="s">
         <v>280</v>
       </c>
       <c r="E48" s="2" t="s">
@@ -3680,7 +3726,7 @@
       <c r="K48" s="2" t="s">
         <v>285</v>
       </c>
-      <c r="M48" s="3" t="s">
+      <c r="M48" s="2" t="s">
         <v>101</v>
       </c>
     </row>
@@ -3691,7 +3737,7 @@
       <c r="C49" s="1" t="n">
         <v>1300</v>
       </c>
-      <c r="D49" s="14" t="s">
+      <c r="D49" s="13" t="s">
         <v>286</v>
       </c>
       <c r="E49" s="2" t="s">
@@ -3709,7 +3755,7 @@
       <c r="K49" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M49" s="3" t="s">
+      <c r="M49" s="2" t="s">
         <v>101</v>
       </c>
     </row>
@@ -3720,10 +3766,10 @@
       <c r="C50" s="1" t="n">
         <v>1650</v>
       </c>
-      <c r="D50" s="14" t="s">
+      <c r="D50" s="13" t="s">
         <v>291</v>
       </c>
-      <c r="E50" s="25" t="s">
+      <c r="E50" s="24" t="s">
         <v>292</v>
       </c>
       <c r="F50" s="1" t="s">
@@ -3732,77 +3778,77 @@
       <c r="G50" s="2" t="s">
         <v>294</v>
       </c>
-      <c r="J50" s="25" t="s">
+      <c r="J50" s="24" t="s">
         <v>295</v>
       </c>
       <c r="K50" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M50" s="3" t="s">
+      <c r="M50" s="2" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="293.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="16" t="n">
+      <c r="A51" s="15" t="n">
         <v>1680</v>
       </c>
-      <c r="B51" s="16"/>
-      <c r="C51" s="16" t="s">
+      <c r="B51" s="15"/>
+      <c r="C51" s="15" t="s">
         <v>296</v>
       </c>
-      <c r="D51" s="17" t="s">
+      <c r="D51" s="16" t="s">
         <v>297</v>
       </c>
-      <c r="E51" s="18" t="s">
+      <c r="E51" s="17" t="s">
         <v>298</v>
       </c>
-      <c r="F51" s="16" t="s">
+      <c r="F51" s="15" t="s">
         <v>299</v>
       </c>
-      <c r="G51" s="18" t="s">
+      <c r="G51" s="17" t="s">
         <v>300</v>
       </c>
-      <c r="H51" s="16"/>
-      <c r="I51" s="16"/>
+      <c r="H51" s="15"/>
+      <c r="I51" s="15"/>
       <c r="J51" s="2" t="s">
         <v>301</v>
       </c>
       <c r="K51" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M51" s="3" t="s">
+      <c r="M51" s="2" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="395.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="16" t="n">
+      <c r="A52" s="15" t="n">
         <v>1720</v>
       </c>
-      <c r="B52" s="16"/>
-      <c r="C52" s="16" t="n">
+      <c r="B52" s="15"/>
+      <c r="C52" s="15" t="n">
         <v>1720</v>
       </c>
-      <c r="D52" s="17" t="s">
+      <c r="D52" s="16" t="s">
         <v>302</v>
       </c>
-      <c r="E52" s="21" t="s">
+      <c r="E52" s="20" t="s">
         <v>303</v>
       </c>
-      <c r="F52" s="16" t="s">
+      <c r="F52" s="15" t="s">
         <v>304</v>
       </c>
-      <c r="G52" s="18" t="s">
+      <c r="G52" s="17" t="s">
         <v>305</v>
       </c>
-      <c r="H52" s="16"/>
-      <c r="I52" s="16"/>
-      <c r="J52" s="25" t="s">
+      <c r="H52" s="15"/>
+      <c r="I52" s="15"/>
+      <c r="J52" s="24" t="s">
         <v>306</v>
       </c>
       <c r="K52" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M52" s="3" t="s">
+      <c r="M52" s="2" t="s">
         <v>58</v>
       </c>
     </row>
@@ -3813,7 +3859,7 @@
       <c r="C53" s="1" t="n">
         <v>1750</v>
       </c>
-      <c r="D53" s="14" t="s">
+      <c r="D53" s="13" t="s">
         <v>307</v>
       </c>
       <c r="E53" s="2" t="s">
@@ -3831,71 +3877,71 @@
       <c r="K53" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M53" s="3" t="s">
+      <c r="M53" s="2" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="249.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="10" t="n">
+      <c r="A54" s="9" t="n">
         <v>1760</v>
       </c>
-      <c r="B54" s="10"/>
-      <c r="C54" s="10" t="s">
+      <c r="B54" s="9"/>
+      <c r="C54" s="9" t="s">
         <v>312</v>
       </c>
-      <c r="D54" s="11" t="s">
+      <c r="D54" s="10" t="s">
         <v>313</v>
       </c>
-      <c r="E54" s="12" t="s">
+      <c r="E54" s="11" t="s">
         <v>314</v>
       </c>
-      <c r="F54" s="10" t="s">
+      <c r="F54" s="9" t="s">
         <v>315</v>
       </c>
-      <c r="G54" s="12" t="s">
+      <c r="G54" s="11" t="s">
         <v>316</v>
       </c>
-      <c r="H54" s="10"/>
-      <c r="I54" s="10"/>
+      <c r="H54" s="9"/>
+      <c r="I54" s="9"/>
       <c r="J54" s="2" t="s">
         <v>317</v>
       </c>
       <c r="K54" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M54" s="3" t="s">
+      <c r="M54" s="2" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="304.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="16" t="n">
+      <c r="A55" s="15" t="n">
         <v>1820</v>
       </c>
-      <c r="B55" s="16"/>
-      <c r="C55" s="16" t="n">
+      <c r="B55" s="15"/>
+      <c r="C55" s="15" t="n">
         <v>1820</v>
       </c>
-      <c r="D55" s="17" t="s">
+      <c r="D55" s="16" t="s">
         <v>318</v>
       </c>
-      <c r="E55" s="18" t="s">
+      <c r="E55" s="17" t="s">
         <v>319</v>
       </c>
-      <c r="F55" s="16" t="s">
+      <c r="F55" s="15" t="s">
         <v>320</v>
       </c>
-      <c r="G55" s="18" t="s">
+      <c r="G55" s="17" t="s">
         <v>321</v>
       </c>
-      <c r="H55" s="16"/>
-      <c r="I55" s="18"/>
+      <c r="H55" s="15"/>
+      <c r="I55" s="17"/>
       <c r="J55" s="2" t="s">
         <v>322</v>
       </c>
       <c r="K55" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="M55" s="3" t="s">
+      <c r="M55" s="2" t="s">
         <v>76</v>
       </c>
     </row>
@@ -3906,7 +3952,7 @@
       <c r="C56" s="1" t="s">
         <v>323</v>
       </c>
-      <c r="D56" s="14" t="s">
+      <c r="D56" s="13" t="s">
         <v>324</v>
       </c>
       <c r="E56" s="2" t="s">
@@ -3938,7 +3984,7 @@
       <c r="C57" s="1" t="s">
         <v>331</v>
       </c>
-      <c r="D57" s="14" t="s">
+      <c r="D57" s="13" t="s">
         <v>332</v>
       </c>
       <c r="E57" s="2" t="s">
@@ -3956,106 +4002,106 @@
       <c r="K57" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M57" s="3" t="s">
+      <c r="M57" s="2" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="151.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="16" t="n">
+      <c r="A58" s="15" t="n">
         <v>1845</v>
       </c>
-      <c r="B58" s="16"/>
-      <c r="C58" s="16" t="n">
+      <c r="B58" s="15"/>
+      <c r="C58" s="15" t="n">
         <v>1845</v>
       </c>
-      <c r="D58" s="17" t="s">
+      <c r="D58" s="16" t="s">
         <v>337</v>
       </c>
-      <c r="E58" s="18" t="s">
+      <c r="E58" s="17" t="s">
         <v>338</v>
       </c>
-      <c r="F58" s="16" t="s">
+      <c r="F58" s="15" t="s">
         <v>339</v>
       </c>
-      <c r="G58" s="18" t="s">
+      <c r="G58" s="17" t="s">
         <v>340</v>
       </c>
-      <c r="H58" s="16"/>
-      <c r="I58" s="18"/>
+      <c r="H58" s="15"/>
+      <c r="I58" s="17"/>
       <c r="J58" s="2" t="s">
         <v>341</v>
       </c>
       <c r="K58" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="M58" s="3" t="s">
+      <c r="M58" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="N58" s="0" t="s">
+      <c r="N58" s="1" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="329.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="16" t="n">
+      <c r="A59" s="15" t="n">
         <v>1850</v>
       </c>
-      <c r="B59" s="16"/>
-      <c r="C59" s="16" t="n">
+      <c r="B59" s="15"/>
+      <c r="C59" s="15" t="n">
         <v>1850</v>
       </c>
-      <c r="D59" s="26" t="s">
+      <c r="D59" s="25" t="s">
         <v>342</v>
       </c>
-      <c r="E59" s="27" t="s">
+      <c r="E59" s="26" t="s">
         <v>343</v>
       </c>
-      <c r="F59" s="16" t="s">
+      <c r="F59" s="15" t="s">
         <v>344</v>
       </c>
-      <c r="G59" s="18" t="s">
+      <c r="G59" s="17" t="s">
         <v>345</v>
       </c>
-      <c r="H59" s="16"/>
-      <c r="I59" s="18"/>
+      <c r="H59" s="15"/>
+      <c r="I59" s="17"/>
       <c r="J59" s="2" t="s">
         <v>346</v>
       </c>
       <c r="K59" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M59" s="3" t="s">
+      <c r="M59" s="2" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="267" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="16" t="n">
+      <c r="A60" s="15" t="n">
         <v>1850</v>
       </c>
-      <c r="B60" s="16"/>
-      <c r="C60" s="16" t="n">
+      <c r="B60" s="15"/>
+      <c r="C60" s="15" t="n">
         <v>1850</v>
       </c>
-      <c r="D60" s="17" t="s">
+      <c r="D60" s="16" t="s">
         <v>347</v>
       </c>
-      <c r="E60" s="18" t="s">
+      <c r="E60" s="17" t="s">
         <v>348</v>
       </c>
-      <c r="F60" s="16" t="s">
+      <c r="F60" s="15" t="s">
         <v>349</v>
       </c>
-      <c r="G60" s="18" t="s">
+      <c r="G60" s="17" t="s">
         <v>350</v>
       </c>
-      <c r="H60" s="16"/>
-      <c r="I60" s="18"/>
+      <c r="H60" s="15"/>
+      <c r="I60" s="17"/>
       <c r="J60" s="2" t="s">
         <v>351</v>
       </c>
       <c r="K60" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="M60" s="3" t="s">
+      <c r="M60" s="2" t="s">
         <v>76</v>
       </c>
     </row>
@@ -4084,71 +4130,71 @@
       <c r="K61" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M61" s="3" t="s">
+      <c r="M61" s="2" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="169.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A62" s="10" t="n">
+      <c r="A62" s="9" t="n">
         <v>1870</v>
       </c>
-      <c r="B62" s="10"/>
-      <c r="C62" s="10" t="n">
+      <c r="B62" s="9"/>
+      <c r="C62" s="9" t="n">
         <v>1870</v>
       </c>
-      <c r="D62" s="11" t="s">
+      <c r="D62" s="10" t="s">
         <v>358</v>
       </c>
-      <c r="E62" s="28" t="s">
+      <c r="E62" s="27" t="s">
         <v>359</v>
       </c>
-      <c r="F62" s="10" t="s">
+      <c r="F62" s="9" t="s">
         <v>360</v>
       </c>
-      <c r="G62" s="12" t="s">
+      <c r="G62" s="11" t="s">
         <v>361</v>
       </c>
-      <c r="H62" s="10"/>
-      <c r="I62" s="10"/>
+      <c r="H62" s="9"/>
+      <c r="I62" s="9"/>
       <c r="J62" s="2" t="s">
         <v>362</v>
       </c>
       <c r="K62" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="M62" s="3" t="s">
+      <c r="M62" s="2" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="138" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A63" s="16" t="n">
+      <c r="A63" s="15" t="n">
         <v>1878</v>
       </c>
-      <c r="B63" s="16"/>
-      <c r="C63" s="16" t="n">
+      <c r="B63" s="15"/>
+      <c r="C63" s="15" t="n">
         <v>1878</v>
       </c>
-      <c r="D63" s="17" t="s">
+      <c r="D63" s="16" t="s">
         <v>363</v>
       </c>
-      <c r="E63" s="18" t="s">
+      <c r="E63" s="17" t="s">
         <v>364</v>
       </c>
-      <c r="F63" s="16" t="s">
+      <c r="F63" s="15" t="s">
         <v>365</v>
       </c>
-      <c r="G63" s="18" t="s">
+      <c r="G63" s="17" t="s">
         <v>366</v>
       </c>
-      <c r="H63" s="16"/>
-      <c r="I63" s="18"/>
+      <c r="H63" s="15"/>
+      <c r="I63" s="17"/>
       <c r="J63" s="2" t="s">
         <v>367</v>
       </c>
       <c r="K63" s="2" t="s">
         <v>368</v>
       </c>
-      <c r="M63" s="3" t="s">
+      <c r="M63" s="2" t="s">
         <v>76</v>
       </c>
     </row>
@@ -4159,7 +4205,7 @@
       <c r="C64" s="1" t="n">
         <v>1900</v>
       </c>
-      <c r="D64" s="14" t="s">
+      <c r="D64" s="13" t="s">
         <v>369</v>
       </c>
       <c r="E64" s="2" t="s">
@@ -4177,10 +4223,10 @@
       <c r="K64" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="M64" s="3" t="s">
+      <c r="M64" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="N64" s="0" t="s">
+      <c r="N64" s="1" t="s">
         <v>50</v>
       </c>
     </row>
@@ -4191,7 +4237,7 @@
       <c r="C65" s="1" t="n">
         <v>1905</v>
       </c>
-      <c r="D65" s="14" t="s">
+      <c r="D65" s="13" t="s">
         <v>374</v>
       </c>
       <c r="E65" s="2" t="s">
@@ -4209,7 +4255,7 @@
       <c r="K65" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="M65" s="3" t="s">
+      <c r="M65" s="2" t="s">
         <v>43</v>
       </c>
     </row>
@@ -4220,10 +4266,10 @@
       <c r="C66" s="1" t="n">
         <v>1905</v>
       </c>
-      <c r="D66" s="14" t="s">
+      <c r="D66" s="13" t="s">
         <v>379</v>
       </c>
-      <c r="E66" s="23" t="s">
+      <c r="E66" s="22" t="s">
         <v>380</v>
       </c>
       <c r="F66" s="1" t="s">
@@ -4232,13 +4278,13 @@
       <c r="G66" s="2" t="s">
         <v>382</v>
       </c>
-      <c r="J66" s="23" t="s">
+      <c r="J66" s="22" t="s">
         <v>383</v>
       </c>
       <c r="K66" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="M66" s="3" t="s">
+      <c r="M66" s="2" t="s">
         <v>76</v>
       </c>
     </row>
@@ -4249,7 +4295,7 @@
       <c r="C67" s="1" t="n">
         <v>1920</v>
       </c>
-      <c r="D67" s="14" t="s">
+      <c r="D67" s="13" t="s">
         <v>384</v>
       </c>
       <c r="E67" s="2" t="s">
@@ -4267,7 +4313,7 @@
       <c r="K67" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="M67" s="3" t="s">
+      <c r="M67" s="2" t="s">
         <v>43</v>
       </c>
     </row>
@@ -4296,39 +4342,39 @@
       <c r="K68" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="M68" s="3" t="s">
+      <c r="M68" s="2" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="77.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A69" s="16" t="n">
+      <c r="A69" s="15" t="n">
         <v>1935</v>
       </c>
-      <c r="B69" s="16"/>
-      <c r="C69" s="16" t="s">
+      <c r="B69" s="15"/>
+      <c r="C69" s="15" t="s">
         <v>395</v>
       </c>
-      <c r="D69" s="17" t="s">
+      <c r="D69" s="16" t="s">
         <v>396</v>
       </c>
-      <c r="E69" s="18" t="s">
+      <c r="E69" s="17" t="s">
         <v>397</v>
       </c>
-      <c r="F69" s="16" t="s">
+      <c r="F69" s="15" t="s">
         <v>398</v>
       </c>
-      <c r="G69" s="18" t="s">
+      <c r="G69" s="17" t="s">
         <v>399</v>
       </c>
-      <c r="H69" s="16"/>
-      <c r="I69" s="16"/>
+      <c r="H69" s="15"/>
+      <c r="I69" s="15"/>
       <c r="J69" s="2" t="s">
         <v>400</v>
       </c>
       <c r="K69" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="M69" s="3" t="s">
+      <c r="M69" s="2" t="s">
         <v>64</v>
       </c>
     </row>
@@ -4339,10 +4385,10 @@
       <c r="C70" s="1" t="n">
         <v>1940</v>
       </c>
-      <c r="D70" s="14" t="s">
+      <c r="D70" s="13" t="s">
         <v>401</v>
       </c>
-      <c r="E70" s="25" t="s">
+      <c r="E70" s="24" t="s">
         <v>402</v>
       </c>
       <c r="F70" s="1" t="s">
@@ -4351,13 +4397,13 @@
       <c r="G70" s="2" t="s">
         <v>404</v>
       </c>
-      <c r="J70" s="25" t="s">
+      <c r="J70" s="24" t="s">
         <v>405</v>
       </c>
       <c r="K70" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="M70" s="3" t="s">
+      <c r="M70" s="2" t="s">
         <v>76</v>
       </c>
     </row>
@@ -4368,7 +4414,7 @@
       <c r="C71" s="1" t="n">
         <v>1945</v>
       </c>
-      <c r="D71" s="14" t="s">
+      <c r="D71" s="13" t="s">
         <v>406</v>
       </c>
       <c r="E71" s="2" t="s">
@@ -4386,7 +4432,7 @@
       <c r="K71" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="M71" s="3" t="s">
+      <c r="M71" s="2" t="s">
         <v>64</v>
       </c>
     </row>
@@ -4397,7 +4443,7 @@
       <c r="C72" s="1" t="n">
         <v>1964</v>
       </c>
-      <c r="D72" s="14" t="s">
+      <c r="D72" s="13" t="s">
         <v>411</v>
       </c>
       <c r="E72" s="2" t="s">
@@ -4415,18 +4461,18 @@
       <c r="K72" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="M72" s="3" t="s">
+      <c r="M72" s="2" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="73" customFormat="false" ht="249.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="73" customFormat="false" ht="201.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="1" t="n">
         <v>1990</v>
       </c>
       <c r="C73" s="1" t="n">
         <v>1990</v>
       </c>
-      <c r="D73" s="14" t="s">
+      <c r="D73" s="13" t="s">
         <v>416</v>
       </c>
       <c r="E73" s="2" t="s">
@@ -4444,31 +4490,111 @@
       <c r="K73" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M73" s="3" t="s">
+      <c r="M73" s="2" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="74" customFormat="false" ht="316.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A74" s="0"/>
-      <c r="B74" s="0"/>
-      <c r="C74" s="0"/>
-      <c r="D74" s="0"/>
-      <c r="E74" s="0"/>
-      <c r="F74" s="0"/>
-      <c r="G74" s="0"/>
-      <c r="H74" s="0"/>
-      <c r="I74" s="0"/>
-      <c r="J74" s="0"/>
-      <c r="K74" s="0"/>
-      <c r="L74" s="0"/>
-      <c r="M74" s="0"/>
-    </row>
-    <row r="75" customFormat="false" ht="271.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D75" s="1"/>
+    <row r="74" customFormat="false" ht="273.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A74" s="1" t="n">
+        <v>1860</v>
+      </c>
+      <c r="C74" s="1" t="n">
+        <v>1860</v>
+      </c>
+      <c r="D74" s="1" t="s">
+        <v>421</v>
+      </c>
+      <c r="E74" s="2" t="s">
+        <v>422</v>
+      </c>
+      <c r="G74" s="1"/>
+      <c r="J74" s="1" t="s">
+        <v>423</v>
+      </c>
+      <c r="K74" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="L74" s="1"/>
+      <c r="M74" s="1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="218.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A75" s="1" t="n">
+        <v>1970</v>
+      </c>
+      <c r="C75" s="1" t="n">
+        <v>1970</v>
+      </c>
+      <c r="D75" s="1" t="s">
+        <v>424</v>
+      </c>
+      <c r="E75" s="2" t="s">
+        <v>425</v>
+      </c>
+      <c r="J75" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="K75" s="2" t="s">
+        <v>427</v>
+      </c>
       <c r="L75" s="1"/>
-    </row>
-    <row r="76" customFormat="false" ht="180" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+      <c r="M75" s="2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="238.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A76" s="1" t="n">
+        <v>1650</v>
+      </c>
+      <c r="C76" s="1" t="s">
+        <v>428</v>
+      </c>
+      <c r="D76" s="1" t="s">
+        <v>429</v>
+      </c>
+      <c r="E76" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="J76" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="K76" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="L76" s="1" t="s">
+        <v>432</v>
+      </c>
+      <c r="M76" s="2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="226.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A77" s="1" t="n">
+        <v>1921</v>
+      </c>
+      <c r="C77" s="1" t="s">
+        <v>433</v>
+      </c>
+      <c r="D77" s="1" t="s">
+        <v>434</v>
+      </c>
+      <c r="E77" s="2" t="s">
+        <v>435</v>
+      </c>
+      <c r="J77" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="K77" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="L77" s="1" t="s">
+        <v>438</v>
+      </c>
+      <c r="M77" s="2" t="s">
+        <v>101</v>
+      </c>
+    </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="2">
@@ -4519,193 +4645,193 @@
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B3" s="29" t="s">
-        <v>421</v>
+      <c r="B3" s="28" t="s">
+        <v>439</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B5" s="29" t="s">
-        <v>422</v>
+      <c r="B5" s="28" t="s">
+        <v>440</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="53.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="30" t="s">
-        <v>423</v>
-      </c>
-      <c r="C6" s="31" t="s">
-        <v>424</v>
+      <c r="B6" s="29" t="s">
+        <v>441</v>
+      </c>
+      <c r="C6" s="30" t="s">
+        <v>442</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="32.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="30" t="s">
-        <v>425</v>
-      </c>
-      <c r="C7" s="31" t="s">
-        <v>426</v>
+      <c r="B7" s="29" t="s">
+        <v>443</v>
+      </c>
+      <c r="C7" s="30" t="s">
+        <v>444</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="84.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="30" t="s">
-        <v>427</v>
-      </c>
-      <c r="C8" s="31" t="s">
-        <v>428</v>
+      <c r="B8" s="29" t="s">
+        <v>445</v>
+      </c>
+      <c r="C8" s="30" t="s">
+        <v>446</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="30" t="s">
-        <v>429</v>
-      </c>
-      <c r="C9" s="31" t="s">
-        <v>430</v>
+      <c r="B9" s="29" t="s">
+        <v>447</v>
+      </c>
+      <c r="C9" s="30" t="s">
+        <v>448</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="199.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B10" s="30" t="s">
-        <v>431</v>
-      </c>
-      <c r="C10" s="31" t="s">
-        <v>432</v>
+      <c r="B10" s="29" t="s">
+        <v>449</v>
+      </c>
+      <c r="C10" s="30" t="s">
+        <v>450</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="157.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B11" s="30" t="s">
-        <v>433</v>
-      </c>
-      <c r="C11" s="31" t="s">
-        <v>434</v>
+      <c r="B11" s="29" t="s">
+        <v>451</v>
+      </c>
+      <c r="C11" s="30" t="s">
+        <v>452</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="157.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B12" s="30" t="s">
-        <v>435</v>
-      </c>
-      <c r="C12" s="31" t="s">
-        <v>436</v>
+      <c r="B12" s="29" t="s">
+        <v>453</v>
+      </c>
+      <c r="C12" s="30" t="s">
+        <v>454</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B13" s="30" t="s">
-        <v>437</v>
-      </c>
-      <c r="C13" s="31" t="s">
-        <v>438</v>
+      <c r="B13" s="29" t="s">
+        <v>455</v>
+      </c>
+      <c r="C13" s="30" t="s">
+        <v>456</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="30" t="s">
-        <v>439</v>
-      </c>
-      <c r="C14" s="31" t="s">
-        <v>440</v>
+      <c r="B14" s="29" t="s">
+        <v>457</v>
+      </c>
+      <c r="C14" s="30" t="s">
+        <v>458</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B16" s="29" t="s">
-        <v>441</v>
+      <c r="B16" s="28" t="s">
+        <v>459</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="53.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B17" s="30" t="s">
-        <v>442</v>
-      </c>
-      <c r="C17" s="31" t="s">
-        <v>443</v>
+      <c r="B17" s="29" t="s">
+        <v>460</v>
+      </c>
+      <c r="C17" s="30" t="s">
+        <v>461</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="105.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B18" s="30" t="s">
-        <v>444</v>
-      </c>
-      <c r="C18" s="31" t="s">
-        <v>445</v>
+      <c r="B18" s="29" t="s">
+        <v>462</v>
+      </c>
+      <c r="C18" s="30" t="s">
+        <v>463</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B19" s="30" t="s">
-        <v>446</v>
-      </c>
-      <c r="C19" s="31" t="s">
-        <v>447</v>
+      <c r="B19" s="29" t="s">
+        <v>464</v>
+      </c>
+      <c r="C19" s="30" t="s">
+        <v>465</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B21" s="29" t="s">
-        <v>448</v>
+      <c r="B21" s="28" t="s">
+        <v>466</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B22" s="30" t="s">
-        <v>449</v>
-      </c>
-      <c r="C22" s="31" t="s">
-        <v>450</v>
+      <c r="B22" s="29" t="s">
+        <v>467</v>
+      </c>
+      <c r="C22" s="30" t="s">
+        <v>468</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B23" s="30" t="s">
-        <v>451</v>
-      </c>
-      <c r="C23" s="31" t="s">
-        <v>452</v>
+      <c r="B23" s="29" t="s">
+        <v>469</v>
+      </c>
+      <c r="C23" s="30" t="s">
+        <v>470</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B25" s="29" t="s">
-        <v>453</v>
+      <c r="B25" s="28" t="s">
+        <v>471</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="32.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B26" s="30" t="s">
-        <v>454</v>
-      </c>
-      <c r="C26" s="31" t="s">
-        <v>455</v>
+      <c r="B26" s="29" t="s">
+        <v>472</v>
+      </c>
+      <c r="C26" s="30" t="s">
+        <v>473</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="84.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B27" s="30" t="s">
-        <v>456</v>
-      </c>
-      <c r="C27" s="31" t="s">
-        <v>457</v>
+      <c r="B27" s="29" t="s">
+        <v>474</v>
+      </c>
+      <c r="C27" s="30" t="s">
+        <v>475</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="95.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B28" s="30" t="s">
-        <v>458</v>
-      </c>
-      <c r="C28" s="31" t="s">
-        <v>459</v>
+      <c r="B28" s="29" t="s">
+        <v>476</v>
+      </c>
+      <c r="C28" s="30" t="s">
+        <v>477</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B29" s="30" t="s">
-        <v>460</v>
-      </c>
-      <c r="C29" s="31" t="s">
-        <v>461</v>
+      <c r="B29" s="29" t="s">
+        <v>478</v>
+      </c>
+      <c r="C29" s="30" t="s">
+        <v>479</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B31" s="29" t="s">
-        <v>462</v>
+      <c r="B31" s="28" t="s">
+        <v>480</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="84.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B32" s="30" t="s">
-        <v>463</v>
-      </c>
-      <c r="C32" s="31" t="s">
-        <v>464</v>
+      <c r="B32" s="29" t="s">
+        <v>481</v>
+      </c>
+      <c r="C32" s="30" t="s">
+        <v>482</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="53.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B33" s="30" t="s">
-        <v>465</v>
-      </c>
-      <c r="C33" s="31" t="s">
-        <v>466</v>
+      <c r="B33" s="29" t="s">
+        <v>483</v>
+      </c>
+      <c r="C33" s="30" t="s">
+        <v>484</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Japon : 15 nouveaux penseurs (Saichō, Hōnen, Nichiren, Zeami, Itō Jinsai, Hakuin, Andō Shōeki, Nishi Amane, Fukuzawa Yukichi, Okakura Kakuzō, D. T. Suzuki, Tanabe Hajime, Hiratsuka Raichō, Kuki Shūzō, Watsuji Tetsurō) et courant « École de Kyōto » ; Nishitani daté 1900-1990
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-courant-pensee-oriental.xlsx
+++ b/data/frise-courant-pensee-oriental.xlsx
@@ -4595,7 +4595,46 @@
         <v>101</v>
       </c>
     </row>
-    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A78" s="1">
+        <v>1911</v>
+      </c>
+      <c r="C78" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1911</t>
+        </is>
+      </c>
+      <c r="D78" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">École de Kyōto</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/%C3%89cole_de_Ky%C5%8Dto"  title=" Wikipedia"&gt;L’école de Kyōto&lt;/a&gt; désigne le premier grand courant de philosophie moderne né au Japon, autour de Kitarō Nishida et de ses successeurs à l’université impériale de Kyōto. Son point de départ est souvent fixé à 1911, date de la &lt;em&gt;Recherche sur le bien&lt;/em&gt; de Nishida.&lt;/p&gt; &lt;p&gt;Ses penseurs, formés à la philosophie allemande, de Kant et Hegel à Husserl et Heidegger, veulent exprimer dans le langage de la philosophie occidentale l’expérience spirituelle de l’Asie, en particulier celle du bouddhisme zen et de la Terre pure. Au centre de leur réflexion se trouve la notion de « néant absolu » : non pas un simple manque, mais le fond ouvert d’où tout surgit, que Nishida pense comme le « lieu » de toute réalité.&lt;/p&gt; &lt;p&gt;Tanabe Hajime, Nishitani Keiji, puis Ueda Shizuteru développèrent cette pensée, tandis que Watsuji Tetsurō et Kuki Shūzō, proches du groupe, l’ouvrirent à l’éthique et à l’esthétique. Plusieurs de ses membres furent compromis dans la justification idéologique de la guerre du Pacifique, ce qui a longtemps pesé sur sa réception.&lt;/p&gt; &lt;p&gt;Depuis les années 1980, l’école de Kyōto est étudiée dans le monde entier comme le lieu d’un dialogue majeur entre la philosophie occidentale et les traditions spirituelles d’Asie.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J78" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">premier grand courant de philosophie moderne né au Japon, autour de Nishida, Tanabe et Nishitani.</t>
+        </is>
+      </c>
+      <c r="K78" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Métaphysique;Théologie et spiritualité</t>
+        </is>
+      </c>
+      <c r="L78" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kitaro NISHIDA;Hajime TANABE;Keiji NISHITANI;Tetsurō WATSUJI;Shūzō KUKI</t>
+        </is>
+      </c>
+      <c r="M78" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">asie-est</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
Grands absents (lots 5 et 6, 29 fiches) : Unamuno, Huineng, Zhiyi, Shantideva, Guru Nanak, Heschel, Leibowitz, Vasconcelos, Paz, Dignaga, Padmasambhava, Fazang, Linji, Atisha, dalaï-lama, Radhakrishnan, Baal Shem Tov, Sanches, Vieira, Lourenço, Bolívar, Rodó, Kusch, Salazar Bondy, Sobukwe, Tutu, Mazrui, Ngũgĩ, Gyekye ; courant Sikhisme ; lien du Brahmoïsme corrigé ; 4 portraits
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-courant-pensee-oriental.xlsx
+++ b/data/frise-courant-pensee-oriental.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="647" uniqueCount="500">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="654" uniqueCount="506">
   <si>
     <t xml:space="preserve">FRISE DES COURANTS DE PENSÉE ORIENTALE — Données source</t>
   </si>
@@ -1161,7 +1161,7 @@
     <t xml:space="preserve">Brahmoïsme</t>
   </si>
   <si>
-    <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Marxisme"  title=" Wikipedia"&gt; Le Brahmoïsme &lt;/a&gt; est un mouvement religieux et philosophique hindou réformiste qui est né au milieu du XIXe siècle lors de la Renaissance bengalie, fondé en 1828 à Calcutta par Raja Ram Mohan Roy. Ce mouvement considère Dieu comme un principe divin unique, infini et illimité, et ses adeptes, appelés Brahmos, se déclarent « ni hindous, ni musulmans, ni chrétiens », mais adhérents à une nouvelle religion de l'Inde.  &lt;/p&gt; &lt;p&gt; La philosophie brahmo repose sur le monothéisme absolu et le rejet total des traditions hindoues conventionnelles : elle ne reconnaît pas l'autorité des Vedas, ne croit pas aux avatars (incarnations divines), rejette le karma et le samsara, et abandonne le culte des images et les rituels traditionnels. Debendranath Tagore a codifié cette doctrine en 1848 avec le Brahmo Dharma, faisant de la raison et de l'intuition vertueuse les fondements de la foi plutôt que l'autorité scripturaire. &lt;/p&gt; &lt;p&gt; Au cœur du Brahmoïsme se trouve le concept de Brahman, la réalité ultime impersonnelle et transcendante dont émane toute existence, immanente et présente en tout, du plus petit plant au plus grand chêne. Cette philosophie enseigne que l'âme individuelle (Atman) est identique au Brahman universel, et que Dieu est à la fois immanent dans l'univers et transcendant au-delà de lui, inaccessible à la connaissance directe mais accessible par la méditation. &lt;/p&gt; &lt;p&gt; Au cœur du Brahmoïsme se trouve le concept de Brahman, la réalité ultime impersonnelle et transcendante dont émane toute existence, immanente et présente en tout, du plus petit plant au plus grand chêne. Cette philosophie enseigne que l'âme individuelle (Atman) est identique au Brahman universel, et que Dieu est à la fois immanent dans l'univers et transcendant au-delà de lui, inaccessible à la connaissance directe mais accessible par la méditation. &lt;/p&gt; &lt;p&gt; L'éthique brahmo est fondée sur la droiture comme seul mode de vie, la vérité, la connaissance, le libre arbitre et l'égalité fondamentale entre tous les êtres humains, avec un rejet radical du système des castes. Le mouvement a joué un rôle considérable dans les réformes sociales : il a lutté contre le sati (veuves brûlées sur le bûcher), encouragé l'éducation des femmes, soutenu la tempérance et promu l'indépendance nationale indienne, devenant ainsi un moteur de la modernisation de l'Inde. &lt;/p&gt; 
+    <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Brahmo%C3%AFsme"  title=" Wikipedia"&gt; Le Brahmoïsme &lt;/a&gt; est un mouvement religieux et philosophique hindou réformiste qui est né au milieu du XIXe siècle lors de la Renaissance bengalie, fondé en 1828 à Calcutta par Raja Ram Mohan Roy. Ce mouvement considère Dieu comme un principe divin unique, infini et illimité, et ses adeptes, appelés Brahmos, se déclarent « ni hindous, ni musulmans, ni chrétiens », mais adhérents à une nouvelle religion de l'Inde.  &lt;/p&gt; &lt;p&gt; La philosophie brahmo repose sur le monothéisme absolu et le rejet total des traditions hindoues conventionnelles : elle ne reconnaît pas l'autorité des Vedas, ne croit pas aux avatars (incarnations divines), rejette le karma et le samsara, et abandonne le culte des images et les rituels traditionnels. Debendranath Tagore a codifié cette doctrine en 1848 avec le Brahmo Dharma, faisant de la raison et de l'intuition vertueuse les fondements de la foi plutôt que l'autorité scripturaire. &lt;/p&gt; &lt;p&gt; Au cœur du Brahmoïsme se trouve le concept de Brahman, la réalité ultime impersonnelle et transcendante dont émane toute existence, immanente et présente en tout, du plus petit plant au plus grand chêne. Cette philosophie enseigne que l'âme individuelle (Atman) est identique au Brahman universel, et que Dieu est à la fois immanent dans l'univers et transcendant au-delà de lui, inaccessible à la connaissance directe mais accessible par la méditation. &lt;/p&gt; &lt;p&gt; Au cœur du Brahmoïsme se trouve le concept de Brahman, la réalité ultime impersonnelle et transcendante dont émane toute existence, immanente et présente en tout, du plus petit plant au plus grand chêne. Cette philosophie enseigne que l'âme individuelle (Atman) est identique au Brahman universel, et que Dieu est à la fois immanent dans l'univers et transcendant au-delà de lui, inaccessible à la connaissance directe mais accessible par la méditation. &lt;/p&gt; &lt;p&gt; L'éthique brahmo est fondée sur la droiture comme seul mode de vie, la vérité, la connaissance, le libre arbitre et l'égalité fondamentale entre tous les êtres humains, avec un rejet radical du système des castes. Le mouvement a joué un rôle considérable dans les réformes sociales : il a lutté contre le sati (veuves brûlées sur le bûcher), encouragé l'éducation des femmes, soutenu la tempérance et promu l'indépendance nationale indienne, devenant ainsi un moteur de la modernisation de l'Inde. &lt;/p&gt; 
 </t>
   </si>
   <si>
@@ -1347,6 +1347,7 @@
         <color theme="1"/>
         <rFont val="Arial"/>
         <family val="0"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">&lt;audio controls title="Philosophie japonaise: l’école de Kyôto par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/10467-15.11.2013-ITEMA_20549374-2013C12410E0320-NET_FC_EE7092B3-7D80-40AA-947D-AFAD338FBA01-21.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt; </t>
     </r>
@@ -1520,6 +1521,24 @@
   </si>
   <si>
     <t xml:space="preserve">philosophie andine du bien-vivre en harmonie avec la nature, intégrée aux constitutions équatorienne et bolivienne.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1500</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sikhisme</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Sikhisme" title=" Wikipedia"&gt;Le sikhisme&lt;/a&gt; est une religion et une sagesse nées au Pendjab, au nord de l’Inde, à la fin du XVe siècle, dans l’enseignement de Guru Nanak ; le mot « sikh » signifie « disciple ». Dans une région où se côtoient l’hindouisme, l’islam et les mouvements mystiques de la &lt;em&gt;bhakti&lt;/em&gt; et du soufisme, il affirme qu’il n’y a qu’un seul Dieu, sans forme ni incarnation, présent en toute chose, que l’on rejoint par l’amour, la méditation de son Nom et une vie juste, plutôt que par les rites, les idoles ou l’ascèse.&lt;/p&gt; &lt;p&gt;Dix gurus se succèdent de Nanak à Gobind Singh, qui fonde en 1699 le &lt;em&gt;Khalsa&lt;/em&gt;, la communauté des initiés, reconnaissables à cinq signes dont les cheveux jamais coupés, et décide qu’après lui le seul guru sera le livre saint, le &lt;a href="https://fr.wikipedia.org/wiki/Guru_Granth_Sahib" title=" Wikipedia"&gt;&lt;em&gt;Guru Granth Sahib&lt;/em&gt;&lt;/a&gt;. Celui-ci réunit les hymnes des gurus, mais aussi ceux de saints hindous et musulmans comme Kabir : la vérité n’appartient à aucune religion particulière. Le Temple d’or d’Amritsar, ouvert sur quatre côtés, symbolise cet accueil de tous.&lt;/p&gt; &lt;p&gt;Sa philosophie refuse les castes et affirme l’égalité de tous les êtres humains, hommes et femmes. Elle tient la vie juste en trois préceptes : se souvenir de Dieu, gagner honnêtement sa vie, partager avec les autres. La cuisine commune, le &lt;a href="https://fr.wikipedia.org/wiki/Langar" title=" Wikipedia"&gt;&lt;em&gt;langar&lt;/em&gt;&lt;/a&gt;, où tous mangent assis au même rang, en est l’expression concrète. Le sikhisme ne prône pas la fuite du monde mais la sainteté dans la vie ordinaire, au travail et en famille, unie au service désintéressé des autres. Il compte aujourd’hui près de trente millions de fidèles.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">religion et sagesse du Pendjab fondée par Guru Nanak : un Dieu unique, l’égalité de tous et la sainteté dans la vie ordinaire.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Théologie et spiritualité;Éthique</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GURU NANAK</t>
   </si>
   <si>
     <t xml:space="preserve">📖 MODE D'EMPLOI</t>
@@ -1667,7 +1686,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="25">
+  <fonts count="24">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1818,12 +1837,6 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
       <b val="true"/>
       <sz val="11"/>
       <color rgb="FFD4A843"/>
@@ -1961,7 +1974,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2074,15 +2087,19 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="22" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="23" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="21" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="24" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="22" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2338,7 +2355,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:XFD1048576"/>
+  <dimension ref="A1:N80"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6.53"/>
@@ -4257,15 +4274,13 @@
       <c r="J62" s="1" t="s">
         <v>362</v>
       </c>
-      <c r="K62" s="1" t="s">
+      <c r="K62" s="2" t="s">
         <v>22</v>
       </c>
       <c r="L62" s="1"/>
       <c r="M62" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="XFC62" s="0"/>
-      <c r="XFD62" s="0"/>
     </row>
     <row r="63" customFormat="false" ht="169.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="1" t="n">
@@ -4750,41 +4765,40 @@
         <v>64</v>
       </c>
     </row>
-    <row r="79" customFormat="false" ht="226.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A79" s="0"/>
-      <c r="B79" s="0"/>
-      <c r="C79" s="0"/>
-      <c r="D79" s="0"/>
-      <c r="E79" s="0"/>
-      <c r="F79" s="0"/>
-      <c r="G79" s="0"/>
-      <c r="H79" s="0"/>
-      <c r="I79" s="0"/>
-      <c r="J79" s="0"/>
-      <c r="K79" s="0"/>
-      <c r="L79" s="0"/>
-      <c r="M79" s="0"/>
-      <c r="XFC79" s="0"/>
-      <c r="XFD79" s="0"/>
+    <row r="79" customFormat="false" ht="295.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A79" s="1" t="n">
+        <v>1500</v>
+      </c>
+      <c r="C79" s="1" t="s">
+        <v>454</v>
+      </c>
+      <c r="D79" s="28" t="s">
+        <v>455</v>
+      </c>
+      <c r="E79" s="2" t="s">
+        <v>456</v>
+      </c>
+      <c r="G79" s="1"/>
+      <c r="J79" s="1" t="s">
+        <v>457</v>
+      </c>
+      <c r="K79" s="2" t="s">
+        <v>458</v>
+      </c>
+      <c r="L79" s="1" t="s">
+        <v>459</v>
+      </c>
+      <c r="M79" s="1" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="80" customFormat="false" ht="225.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A80" s="0"/>
-      <c r="B80" s="0"/>
-      <c r="C80" s="0"/>
-      <c r="D80" s="0"/>
-      <c r="E80" s="0"/>
-      <c r="F80" s="0"/>
-      <c r="G80" s="0"/>
-      <c r="H80" s="0"/>
-      <c r="I80" s="0"/>
-      <c r="J80" s="0"/>
-      <c r="K80" s="0"/>
-      <c r="L80" s="0"/>
-      <c r="M80" s="0"/>
-      <c r="XFC80" s="0"/>
-      <c r="XFD80" s="0"/>
-    </row>
-    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+      <c r="D80" s="1"/>
+      <c r="G80" s="1"/>
+      <c r="J80" s="1"/>
+      <c r="L80" s="1"/>
+      <c r="M80" s="1"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:I1"/>
@@ -4834,193 +4848,193 @@
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B3" s="28" t="s">
-        <v>454</v>
+      <c r="B3" s="29" t="s">
+        <v>460</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B5" s="28" t="s">
-        <v>455</v>
+      <c r="B5" s="29" t="s">
+        <v>461</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="53.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="29" t="s">
-        <v>456</v>
-      </c>
-      <c r="C6" s="30" t="s">
-        <v>457</v>
+      <c r="B6" s="30" t="s">
+        <v>462</v>
+      </c>
+      <c r="C6" s="31" t="s">
+        <v>463</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="32.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="29" t="s">
-        <v>458</v>
-      </c>
-      <c r="C7" s="30" t="s">
-        <v>459</v>
+      <c r="B7" s="30" t="s">
+        <v>464</v>
+      </c>
+      <c r="C7" s="31" t="s">
+        <v>465</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="84.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="29" t="s">
-        <v>460</v>
-      </c>
-      <c r="C8" s="30" t="s">
-        <v>461</v>
+      <c r="B8" s="30" t="s">
+        <v>466</v>
+      </c>
+      <c r="C8" s="31" t="s">
+        <v>467</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="29" t="s">
-        <v>462</v>
-      </c>
-      <c r="C9" s="30" t="s">
-        <v>463</v>
+      <c r="B9" s="30" t="s">
+        <v>468</v>
+      </c>
+      <c r="C9" s="31" t="s">
+        <v>469</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="199.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B10" s="29" t="s">
-        <v>464</v>
-      </c>
-      <c r="C10" s="30" t="s">
-        <v>465</v>
+      <c r="B10" s="30" t="s">
+        <v>470</v>
+      </c>
+      <c r="C10" s="31" t="s">
+        <v>471</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="157.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B11" s="29" t="s">
-        <v>466</v>
-      </c>
-      <c r="C11" s="30" t="s">
-        <v>467</v>
+      <c r="B11" s="30" t="s">
+        <v>472</v>
+      </c>
+      <c r="C11" s="31" t="s">
+        <v>473</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="157.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B12" s="29" t="s">
-        <v>468</v>
-      </c>
-      <c r="C12" s="30" t="s">
-        <v>469</v>
+      <c r="B12" s="30" t="s">
+        <v>474</v>
+      </c>
+      <c r="C12" s="31" t="s">
+        <v>475</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B13" s="29" t="s">
-        <v>470</v>
-      </c>
-      <c r="C13" s="30" t="s">
-        <v>471</v>
+      <c r="B13" s="30" t="s">
+        <v>476</v>
+      </c>
+      <c r="C13" s="31" t="s">
+        <v>477</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="29" t="s">
-        <v>472</v>
-      </c>
-      <c r="C14" s="30" t="s">
-        <v>473</v>
+      <c r="B14" s="30" t="s">
+        <v>478</v>
+      </c>
+      <c r="C14" s="31" t="s">
+        <v>479</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B16" s="28" t="s">
-        <v>474</v>
+      <c r="B16" s="29" t="s">
+        <v>480</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="53.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B17" s="29" t="s">
-        <v>475</v>
-      </c>
-      <c r="C17" s="30" t="s">
-        <v>476</v>
+      <c r="B17" s="30" t="s">
+        <v>481</v>
+      </c>
+      <c r="C17" s="31" t="s">
+        <v>482</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="105.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B18" s="29" t="s">
-        <v>477</v>
-      </c>
-      <c r="C18" s="30" t="s">
-        <v>478</v>
+      <c r="B18" s="30" t="s">
+        <v>483</v>
+      </c>
+      <c r="C18" s="31" t="s">
+        <v>484</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B19" s="29" t="s">
-        <v>479</v>
-      </c>
-      <c r="C19" s="30" t="s">
-        <v>480</v>
+      <c r="B19" s="30" t="s">
+        <v>485</v>
+      </c>
+      <c r="C19" s="31" t="s">
+        <v>486</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B21" s="28" t="s">
-        <v>481</v>
+      <c r="B21" s="29" t="s">
+        <v>487</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B22" s="29" t="s">
-        <v>482</v>
-      </c>
-      <c r="C22" s="30" t="s">
-        <v>483</v>
+      <c r="B22" s="30" t="s">
+        <v>488</v>
+      </c>
+      <c r="C22" s="31" t="s">
+        <v>489</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B23" s="29" t="s">
-        <v>484</v>
-      </c>
-      <c r="C23" s="30" t="s">
-        <v>485</v>
+      <c r="B23" s="30" t="s">
+        <v>490</v>
+      </c>
+      <c r="C23" s="31" t="s">
+        <v>491</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B25" s="28" t="s">
-        <v>486</v>
+      <c r="B25" s="29" t="s">
+        <v>492</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="32.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B26" s="29" t="s">
-        <v>487</v>
-      </c>
-      <c r="C26" s="30" t="s">
-        <v>488</v>
+      <c r="B26" s="30" t="s">
+        <v>493</v>
+      </c>
+      <c r="C26" s="31" t="s">
+        <v>494</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="84.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B27" s="29" t="s">
-        <v>489</v>
-      </c>
-      <c r="C27" s="30" t="s">
-        <v>490</v>
+      <c r="B27" s="30" t="s">
+        <v>495</v>
+      </c>
+      <c r="C27" s="31" t="s">
+        <v>496</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="95.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B28" s="29" t="s">
-        <v>491</v>
-      </c>
-      <c r="C28" s="30" t="s">
-        <v>492</v>
+      <c r="B28" s="30" t="s">
+        <v>497</v>
+      </c>
+      <c r="C28" s="31" t="s">
+        <v>498</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B29" s="29" t="s">
-        <v>493</v>
-      </c>
-      <c r="C29" s="30" t="s">
-        <v>494</v>
+      <c r="B29" s="30" t="s">
+        <v>499</v>
+      </c>
+      <c r="C29" s="31" t="s">
+        <v>500</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B31" s="28" t="s">
-        <v>495</v>
+      <c r="B31" s="29" t="s">
+        <v>501</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="84.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B32" s="29" t="s">
-        <v>496</v>
-      </c>
-      <c r="C32" s="30" t="s">
-        <v>497</v>
+      <c r="B32" s="30" t="s">
+        <v>502</v>
+      </c>
+      <c r="C32" s="31" t="s">
+        <v>503</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="53.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B33" s="29" t="s">
-        <v>498</v>
-      </c>
-      <c r="C33" s="30" t="s">
-        <v>499</v>
+      <c r="B33" s="30" t="s">
+        <v>504</v>
+      </c>
+      <c r="C33" s="31" t="s">
+        <v>505</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Courants : 22 nouveaux courants (lots A, B, C) et 11 fiches ; éditeur des courants ; figures clés prises en compte
- Lot A (bouddhisme et Inde) : Madhyamaka, Yogācāra, Terre pure, Tiantai, Huayan, Bhakti, Shivaïsme du Cachemire, Néo-védanta
- Lot B (islam et judaïsme) : Ismaélisme, Maturidisme, Kabbale, Hassidisme, Haskala, École d'Ispahan
- Lot C (Sud et Russie) : Sophiologie, Eurasisme, Ethnophilosophie, Socialisme africain, Théologie et Philosophie de la libération, Créolisation, Pensée décoloniale
- Fiches : Louria, Moïse de León, Aboulafia, al-Kirmani, al-Nasafi, Gutiérrez, Boff, Troubetskoï, Tempels, Quijano, Mignolo
- Philosophes existants rattachés aux nouveaux courants
- content.config.ts : figures_cles n'était pas dans le schéma des courants, les « Principaux représentants » l'ignoraient
- Éditeur : mode « Courants de pensée » (liste, filtres, philosophes rattachés, renommage reporté dans les fiches, nouveau courant)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-courant-pensee-oriental.xlsx
+++ b/data/frise-courant-pensee-oriental.xlsx
@@ -2355,7 +2355,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N80"/>
+  <dimension ref="A1:N101"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6.53"/>
@@ -4793,11 +4793,931 @@
       </c>
     </row>
     <row r="80" customFormat="false" ht="225.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D80" s="1"/>
+      <c r="A80" s="1">
+        <v>150</v>
+      </c>
+      <c r="C80" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">150</t>
+        </is>
+      </c>
+      <c r="D80" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Madhyamaka</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Madhyamaka" title=" Wikipedia"&gt;Le Madhyamaka&lt;/a&gt;, ou « école de la Voie du milieu », est l’une des deux grandes écoles philosophiques du bouddhisme mahāyāna. Il naît en Inde vers le IIe siècle avec Nāgārjuna, dont les &lt;a href="https://fr.wikipedia.org/wiki/Mulamadhyamakakarika" title=" Wikipedia"&gt;&lt;em&gt;Stances de la Voie du milieu&lt;/em&gt;&lt;/a&gt; sont le texte fondateur, et son disciple Āryadeva. Le « milieu » qu’il cherche se tient entre deux extrêmes : croire que les choses existent en elles-mêmes, ou croire qu’elles n’existent pas du tout.&lt;/p&gt; &lt;p&gt;Sa thèse centrale est la &lt;a href="https://fr.wikipedia.org/wiki/%C5%9A%C5%ABnyat%C4%81" title=" Wikipedia"&gt;vacuité&lt;/a&gt; (&lt;em&gt;śūnyatā&lt;/em&gt;) : aucune chose n’a d’existence propre, car toute chose dépend d’autre chose, de ses causes, de ses parties et de l’esprit qui la nomme. La vacuité n’est donc pas le néant, mais l’autre nom de la « production conditionnée » enseignée par le Bouddha. Nāgārjuna procède par réfutation : il montre que toute thèse sur l’être, le mouvement, le temps ou la causalité aboutit à des contradictions dès qu’on la tient pour absolue. Il distingue la vérité conventionnelle, celle du langage et de la vie ordinaire, de la vérité ultime, qui échappe aux concepts ; et la vacuité est elle-même vide : ce n’est pas une nouvelle doctrine à laquelle s’accrocher.&lt;/p&gt; &lt;p&gt;L’école se divise ensuite entre ceux qui admettent des raisonnements autonomes et les « Prāsaṅgika » de Candrakīrti, qui se contentent de montrer l’absurdité des thèses adverses. Śāntideva en tire une éthique de la compassion. Transmis au Tibet par Atiśa et systématisé par Tsongkhapa, le Madhyamaka reste la philosophie de référence du bouddhisme tibétain. On l’a souvent rapproché, au XXe siècle, de la critique du langage chez Wittgenstein.&lt;/p&gt;</t>
+        </is>
+      </c>
       <c r="G80" s="1"/>
-      <c r="J80" s="1"/>
-      <c r="L80" s="1"/>
-      <c r="M80" s="1"/>
+      <c r="J80" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">école bouddhiste de la Voie du milieu fondée par Nāgārjuna : rien n’existe en soi, tout est vide parce qu’interdépendant.</t>
+        </is>
+      </c>
+      <c r="K80" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Métaphysique;Épistémologie</t>
+        </is>
+      </c>
+      <c r="L80" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NAGARJUNA;SHANTIDEVA;Je TSONGKHAPA</t>
+        </is>
+      </c>
+      <c r="M80" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">inde</t>
+        </is>
+      </c>
+      <c r="N80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">asie-est</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="225.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A81" s="1">
+        <v>350</v>
+      </c>
+      <c r="C81" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">350</t>
+        </is>
+      </c>
+      <c r="D81" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yogācāra</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Chittamatra" title=" Wikipedia"&gt;Le Yogācāra&lt;/a&gt;, « pratique du yoga », appelé aussi Cittamātra, « esprit seul », est avec le Madhyamaka l’une des deux grandes écoles philosophiques du bouddhisme mahāyāna. Il se forme en Inde au IVe siècle autour de deux frères, Asaṅga et Vasubandhu, à partir de l’expérience des méditants : ce que l’on observe en méditation montre combien le monde vécu est façonné par l’esprit. On doit à Vasubandhu deux courts traités, les &lt;em&gt;Vingt stances&lt;/em&gt; et les &lt;em&gt;Trente stances&lt;/em&gt;, qui résument la doctrine.&lt;/p&gt; &lt;p&gt;Sa thèse est que nous ne connaissons jamais que des représentations : les objets que nous croyons extérieurs sont des apparitions de la conscience, comme dans un rêve. Pour l’expliquer, il ajoute aux six consciences reconnues par le bouddhisme une conscience souillée, qui produit l’illusion d’un moi, et surtout une &lt;a href="https://fr.wikipedia.org/wiki/%C4%80layavij%C3%B1%C4%81na" title=" Wikipedia"&gt;conscience-réceptacle&lt;/a&gt; (&lt;em&gt;ālayavijñāna&lt;/em&gt;), sorte d’inconscient où les actes passés déposent des traces, comme des graines qui germeront plus tard. Il décrit aussi « trois natures » des choses : imaginaire, dépendante et parfaitement accomplie. L’éveil consiste à transformer ce fond de la conscience, jusqu’à ce que cesse le partage entre un sujet qui saisit et un objet saisi.&lt;/p&gt; &lt;p&gt;Ses logiciens, Dignāga puis Dharmakīrti, fondent la grande épistémologie bouddhique. Le pèlerin chinois &lt;a href="https://fr.wikipedia.org/wiki/Xuanzang" title=" Wikipedia"&gt;Xuanzang&lt;/a&gt; rapporte ses textes d’Inde au VIIe siècle et fonde en Chine l’école de la « conscience seule ». Le Yogācāra a nourri le zen, le bouddhisme tibétain et, aujourd’hui, le dialogue avec la phénoménologie et les sciences cognitives.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J81" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">école bouddhiste de « l’esprit seul » : le monde que nous percevons est une construction de la conscience.</t>
+        </is>
+      </c>
+      <c r="K81" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Philosophie de l'esprit;Métaphysique;Épistémologie</t>
+        </is>
+      </c>
+      <c r="L81" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ASANGA;VASUBANDHU;XUANZANG</t>
+        </is>
+      </c>
+      <c r="M81" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">inde</t>
+        </is>
+      </c>
+      <c r="N81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">asie-est</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="225.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A82" s="1">
+        <v>402</v>
+      </c>
+      <c r="C82" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">402</t>
+        </is>
+      </c>
+      <c r="D82" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bouddhisme de la Terre pure</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;Le bouddhisme de la &lt;a href="https://fr.wikipedia.org/wiki/Terre_pure" title=" Wikipedia"&gt;Terre pure&lt;/a&gt; est le courant du bouddhisme mahāyāna centré sur la dévotion au bouddha Amitābha (Amida en japonais) qui, selon les sūtras, a fait le vœu d’accueillir dans sa « Terre pure », un paradis situé à l’Occident, tous ceux qui l’invoquent avec foi. Né en Chine, il remonte à Huiyuan, qui réunit en 402 au mont Lu une communauté vouée à Amitābha, puis à &lt;a href="https://fr.wikipedia.org/wiki/Tanluan" title=" Wikipedia"&gt;Tanluan&lt;/a&gt; et à Shandao, qui en font une école.&lt;/p&gt; &lt;p&gt;Sa philosophie part d’un constat : en cette époque de « déclin de la Loi », les êtres humains ne peuvent plus atteindre l’éveil par leurs propres forces, par la méditation ou l’ascèse. Il faut s’en remettre à la « force de l’autre », la compassion d’Amitābha. La pratique principale devient la récitation de son nom, le &lt;em&gt;nembutsu&lt;/em&gt; : « Namu Amida Butsu ». Au Japon, Hōnen fonde en 1175 l’école &lt;a href="https://fr.wikipedia.org/wiki/J%C5%8Ddo_sh%C5%AB" title=" Wikipedia"&gt;Jōdo shū&lt;/a&gt; et affirme que cette seule récitation suffit au salut, ce qui ouvre le bouddhisme aux gens simples, aux paysans et aux femmes. Son disciple Shinran va plus loin avec le &lt;a href="https://fr.wikipedia.org/wiki/J%C5%8Ddo_shinsh%C5%AB" title=" Wikipedia"&gt;Jōdo shinshū&lt;/a&gt; : le salut est entièrement un don reçu dans la foi, et c’est le « méchant » conscient de ses fautes, plus encore que le juste, que le Bouddha veut sauver. Shinran se marie, quitte la vie monastique et vit parmi le peuple.&lt;/p&gt; &lt;p&gt;Devenue l’une des formes du bouddhisme les plus pratiquées d’Asie de l’Est, la Terre pure évoque la doctrine chrétienne de la grâce, rapprochement qui a fasciné bien des théologiens occidentaux. Elle compte aujourd’hui des dizaines de millions de fidèles au Japon, en Chine, en Corée et au Viêt Nam.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J82" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bouddhisme de la foi en Amitābha : le salut par la récitation de son nom et la « force de l’autre ».</t>
+        </is>
+      </c>
+      <c r="K82" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Théologie et spiritualité</t>
+        </is>
+      </c>
+      <c r="L82" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HŌNEN;SHINRAN</t>
+        </is>
+      </c>
+      <c r="M82" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">asie-est</t>
+        </is>
+      </c>
+      <c r="N82"/>
+    </row>
+    <row r="83" customFormat="false" ht="225.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A83" s="1">
+        <v>575</v>
+      </c>
+      <c r="C83" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">575</t>
+        </is>
+      </c>
+      <c r="D83" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tiantai</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Tiantai" title=" Wikipedia"&gt;Le Tiantai&lt;/a&gt; est la première grande école du bouddhisme née en Chine plutôt qu’importée d’Inde. Elle tire son nom du mont Tiantai, dans le Zhejiang, où le moine Zhiyi (538-597) s’installe en 575 et élabore sa doctrine. Face à la masse des sūtras traduits en chinois, souvent contradictoires, Zhiyi les classe en périodes et en méthodes d’enseignement : le Bouddha aurait adapté sa parole à ses auditeurs, et le &lt;a href="https://fr.wikipedia.org/wiki/S%C5%ABtra_du_Lotus" title=" Wikipedia"&gt;&lt;em&gt;Sūtra du Lotus&lt;/em&gt;&lt;/a&gt; en serait le sommet, qui révèle que tous les êtres peuvent devenir bouddhas.&lt;/p&gt; &lt;p&gt;Sa philosophie repose sur la doctrine des « trois vérités » : toute chose est vide, car sans existence propre ; elle existe pourtant provisoirement, comme apparence ; et elle est le « milieu », qui unit les deux sans les séparer. Zhiyi en tire l’idée qu’« un instant de pensée contient trois mille mondes » : chaque moment de conscience renferme la totalité des états possibles de l’existence, des enfers jusqu’à l’éveil. Le salut n’est donc pas ailleurs : il se découvre au cœur même du monde ordinaire. Zhiyi va jusqu’à soutenir que la nature de bouddha contient aussi le mal, ce qui fait l’originalité de l’école. Il unit étroitement l’étude des textes et la méditation, qu’il expose dans de grands traités sur « l’arrêt et la contemplation ».&lt;/p&gt; &lt;p&gt;Introduite au Japon en 805 par Saichō sous le nom de &lt;a href="https://fr.wikipedia.org/wiki/Tendai" title=" Wikipedia"&gt;Tendai&lt;/a&gt;, l’école fait du monastère du mont Hiei le grand centre du bouddhisme japonais. Elle y forme la plupart des fondateurs des écoles ultérieures, dont Hōnen, Shinran, Dōgen et Nichiren, qui en reprend la dévotion au Lotus.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J83" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">école bouddhiste chinoise fondée par Zhiyi sur le Sūtra du Lotus : trois vérités et trois mille mondes dans un instant de pensée.</t>
+        </is>
+      </c>
+      <c r="K83" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Théologie et spiritualité;Métaphysique</t>
+        </is>
+      </c>
+      <c r="L83" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ZHIYI;SAICHŌ</t>
+        </is>
+      </c>
+      <c r="M83" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">asie-est</t>
+        </is>
+      </c>
+      <c r="N83"/>
+    </row>
+    <row r="84" customFormat="false" ht="225.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A84" s="1">
+        <v>600</v>
+      </c>
+      <c r="C84" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">600</t>
+        </is>
+      </c>
+      <c r="D84" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huayan</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Huayan" title=" Wikipedia"&gt;Le Huayan&lt;/a&gt;, ou « école de l’Ornementation fleurie », est une école du bouddhisme chinois fondée sur l’&lt;a href="https://fr.wikipedia.org/wiki/Avata%E1%B9%83saka_s%C5%ABtra" title=" Wikipedia"&gt;&lt;em&gt;Avataṃsaka sūtra&lt;/em&gt;&lt;/a&gt;, immense texte qui décrit l’univers tel que le voit un bouddha éveillé. Elle se forme aux VIe et VIIe siècles autour de &lt;a href="https://fr.wikipedia.org/wiki/Dushun" title=" Wikipedia"&gt;Dushun&lt;/a&gt;, son premier patriarche, puis de Zhiyan, et trouve son grand systématicien en Fazang (643-712), qui l’expose à la cour de l’impératrice Wu Zetian.&lt;/p&gt; &lt;p&gt;Sa philosophie est celle de l’interdépendance totale : chaque chose contient toutes les autres et se trouve contenue en elles, sans que leurs différences soient abolies. Pour le faire comprendre à l’impératrice, Fazang prend l’image d’un lion d’or : l’or est la nature unique et vide, le lion la forme qu’elle prend, et chaque poil du lion contient le lion tout entier. Il reprend aussi celle du filet d’Indra, filet céleste dont chaque nœud porte une perle qui reflète toutes les autres perles, à l’infini. Le Huayan distingue quatre plans de réalité : celui des phénomènes, celui du principe, celui de leur non-obstruction mutuelle, et enfin celui de la non-obstruction de tous les phénomènes entre eux, qui est la vision de l’éveil.&lt;/p&gt; &lt;p&gt;En Chine, &lt;a href="https://fr.wikipedia.org/wiki/Zongmi" title=" Wikipedia"&gt;Zongmi&lt;/a&gt; (780-841) le concilie avec le chan. Ŭisang l’apporte en Corée, où il devient l’école Hwaeom, que Chinul unira plus tard à la méditation seon ; au Japon, il prend le nom de &lt;a href="https://fr.wikipedia.org/wiki/Kegon" title=" Wikipedia"&gt;Kegon&lt;/a&gt; et c’est à lui que se rattache le grand Bouddha de Nara. Le Huayan a profondément marqué le zen et le néoconfucianisme. On rapproche parfois aujourd’hui sa vision d’un monde entièrement relié de la pensée écologique.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J84" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">école bouddhiste chinoise de l’interdépendance totale, où chaque chose contient toutes les autres.</t>
+        </is>
+      </c>
+      <c r="K84" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Métaphysique;Théologie et spiritualité</t>
+        </is>
+      </c>
+      <c r="L84" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FAZANG;UISANG</t>
+        </is>
+      </c>
+      <c r="M84" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">asie-est</t>
+        </is>
+      </c>
+      <c r="N84"/>
+    </row>
+    <row r="85" customFormat="false" ht="225.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A85" s="1">
+        <v>600</v>
+      </c>
+      <c r="C85" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">600</t>
+        </is>
+      </c>
+      <c r="D85" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bhakti</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Bhakti" title=" Wikipedia"&gt;La bhakti&lt;/a&gt;, la « dévotion » ou « l’amour de Dieu », est une voie spirituelle de l’hindouisme qui place l’amour personnel d’une divinité au-dessus des rites, des sacrifices et du savoir. Annoncée dans la &lt;em&gt;Bhagavad-Gītā&lt;/em&gt;, où Krishna enseigne que l’abandon aimant à Dieu est le plus sûr chemin vers la délivrance, elle devient un grand mouvement dans l’Inde du Sud entre le VIe et le IXe siècle, avec les poètes tamouls : les &lt;a href="https://fr.wikipedia.org/wiki/Alvar" title=" Wikipedia"&gt;Alvars&lt;/a&gt;, dévots de Vishnou, et les &lt;a href="https://fr.wikipedia.org/wiki/Nayanar" title=" Wikipedia"&gt;Nayanars&lt;/a&gt;, dévots de Shiva.&lt;/p&gt; &lt;p&gt;Ces saints chantent leur dieu dans la langue du peuple et non en sanskrit, et beaucoup viennent de basses castes : la bhakti affirme que l’amour de Dieu est ouvert à tous, sans distinction de naissance ni de sexe. Elle reçoit une base philosophique avec Rāmānuja, au XIe siècle, qui défend contre Shankara la réalité de l’âme et du monde, distincts de Dieu tout en dépendant de lui ; Madhva va plus loin dans le dualisme. L’âme ne se fond pas dans l’absolu : elle demeure, pour aimer. Du XIIIe au XVIIe siècle, la bhakti gagne l’Inde du Nord : Kabir, tisserand de Bénarès, unit hindous et musulmans dans le culte d’un Dieu sans forme ; la princesse Mīrābāī chante Krishna en bravant les conventions ; Chaitanya, au Bengale, fait du chant et de la danse une prière extatique ; &lt;a href="https://fr.wikipedia.org/wiki/Tuls%C3%AEd%C3%A2s" title=" Wikipedia"&gt;Tulsîdâs&lt;/a&gt; écrit le &lt;em&gt;Ramcharitmanas&lt;/em&gt;.&lt;/p&gt; &lt;p&gt;Mouvement de réforme autant que de piété, la bhakti a façonné l’hindouisme populaire, inspiré le sikhisme et nourri, jusqu’à Gandhi, l’idée que la religion se vit d’abord dans le cœur.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J85" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">voie hindoue de la dévotion amoureuse à Dieu, ouverte à tous sans distinction de caste ni de sexe.</t>
+        </is>
+      </c>
+      <c r="K85" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Théologie et spiritualité;Éthique</t>
+        </is>
+      </c>
+      <c r="L85" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RAMANUJA;KABIR;MIRABAI</t>
+        </is>
+      </c>
+      <c r="M85" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">inde</t>
+        </is>
+      </c>
+      <c r="N85"/>
+    </row>
+    <row r="86" customFormat="false" ht="225.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A86" s="1">
+        <v>850</v>
+      </c>
+      <c r="C86" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">850</t>
+        </is>
+      </c>
+      <c r="D86" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shivaïsme du Cachemire</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Shiva%C3%AFsme_du_Cachemire" title=" Wikipedia"&gt;Le shivaïsme du Cachemire&lt;/a&gt; est une école philosophique et mystique hindoue qui s’épanouit dans la vallée du Cachemire entre le IXe et le XIe siècle. Il naît, selon la tradition, des &lt;em&gt;Śiva Sūtra&lt;/em&gt; que &lt;a href="https://fr.wikipedia.org/wiki/Vasugupta" title=" Wikipedia"&gt;Vasugupta&lt;/a&gt; aurait reçus en rêve. À la différence du shivaïsme dualiste du Sud, il est résolument non dualiste : il n’existe qu’une seule réalité, Shiva, conscience absolue, libre et lumineuse, dont l’univers entier est la manifestation. Il appartient au monde des tantras, qui valorise le corps, l’énergie et la vie dans le monde plutôt que le renoncement.&lt;/p&gt; &lt;p&gt;Là où l’Advaita Védanta de Shankara voit dans le monde une illusion, le shivaïsme du Cachemire y voit le jeu bien réel de la liberté divine. La conscience n’est pas seulement une lumière immobile ; elle est aussi &lt;a href="https://fr.wikipedia.org/wiki/Spanda" title=" Wikipedia"&gt;&lt;em&gt;spanda&lt;/em&gt;&lt;/a&gt;, « vibration », énergie créatrice qui se déploie sous la forme des choses. Utpaladeva fonde l’école de la « Reconnaissance » (&lt;em&gt;Pratyabhijñā&lt;/em&gt;) : l’être humain n’a pas à devenir Shiva, il l’est déjà, et la libération consiste à le reconnaître, comme on reconnaît soudain un ami qu’on avait sous les yeux. Le grand penseur de l’école, Abhinavagupta, en fait la synthèse dans son immense &lt;em&gt;Tantrāloka&lt;/em&gt;, « Lumière sur les tantras ». Il pense aussi l’art : l’émotion esthétique (&lt;em&gt;rasa&lt;/em&gt;) éprouvée au théâtre ou devant un poème est un avant-goût de la joie de la conscience libérée.&lt;/p&gt; &lt;p&gt;Presque oublié après le XIIe siècle, il a été redécouvert au XXe siècle, notamment grâce à l’indianiste &lt;a href="https://fr.wikipedia.org/wiki/Lilian_Silburn" title=" Wikipedia"&gt;Lilian Silburn&lt;/a&gt; en France et au maître cachemirien Swami Lakshman Joo.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J86" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">non-dualisme hindou pour qui le monde est le libre jeu de la conscience divine, Shiva, que l’être humain doit reconnaître en lui.</t>
+        </is>
+      </c>
+      <c r="K86" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Métaphysique;Théologie et spiritualité</t>
+        </is>
+      </c>
+      <c r="L86" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ABHINAVAGUPTA;UTPALADEVA</t>
+        </is>
+      </c>
+      <c r="M86" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">inde</t>
+        </is>
+      </c>
+      <c r="N86"/>
+    </row>
+    <row r="87" customFormat="false" ht="225.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A87" s="1">
+        <v>1890</v>
+      </c>
+      <c r="C87" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1890</t>
+        </is>
+      </c>
+      <c r="D87" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Néo-védanta</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;On appelle &lt;a href="https://fr.wikipedia.org/wiki/N%C3%A9o-v%C3%A9danta" title=" Wikipedia"&gt;néo-védanta&lt;/a&gt; la forme moderne du Védanta qui se développe en Inde à partir du XIXe siècle, en anglais plutôt qu’en sanskrit, au contact de l’Occident et de la domination britannique. Elle renouvelle la philosophie non dualiste de Shankara pour en faire une réponse aux critiques des missionnaires et un fondement de la fierté indienne.&lt;/p&gt; &lt;p&gt;Son point de départ est le mystique bengali &lt;a href="https://fr.wikipedia.org/wiki/R%C3%A2makrishna" title=" Wikipedia"&gt;Râmakrishna&lt;/a&gt; (1836-1886), qui affirme, après avoir pratiqué plusieurs religions, que toutes mènent au même but. Son disciple Vivekananda porte ce message au &lt;a href="https://fr.wikipedia.org/wiki/Parlement_des_religions" title=" Wikipedia"&gt;Parlement des religions&lt;/a&gt; de Chicago, en 1893 : le Védanta y devient une religion universelle et rationnelle, compatible avec la science, qui reconnaît la divinité présente en chaque être humain. Il en découle une éthique de l’action : servir les pauvres, c’est servir Dieu ; Vivekananda fonde à cette fin la Mission Ramakrishna, vouée à l’enseignement et aux soins. Au XXe siècle, Sri Aurobindo en propose, depuis son ashram de Pondichéry, une version évolutionniste, où la conscience divine descend dans la matière et où l’humanité doit s’élever vers un « supramental ». Sarvepalli Radhakrishnan, professeur à Oxford devenu président de l’Inde, en donne l’exposé savant et le présente comme la synthèse de l’expérience religieuse de l’humanité.&lt;/p&gt; &lt;p&gt;Le néo-védanta a façonné l’image de l’hindouisme dans le monde et nourri le nationalisme indien. Des historiens lui reprochent cependant d’avoir unifié une tradition très diverse en la lisant à travers des catégories occidentales.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J87" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">relecture moderne du Védanta par Vivekananda, Aurobindo et Radhakrishnan : une religion universelle et rationnelle.</t>
+        </is>
+      </c>
+      <c r="K87" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Métaphysique;Théologie et spiritualité</t>
+        </is>
+      </c>
+      <c r="L87" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VIVEKANANDA;Sri AUROBINDO;Sarvepalli RADHAKRISHNAN</t>
+        </is>
+      </c>
+      <c r="M87" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">inde</t>
+        </is>
+      </c>
+      <c r="N87"/>
+    </row>
+    <row r="88" customFormat="false" ht="225.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A88" s="1">
+        <v>765</v>
+      </c>
+      <c r="C88" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">765</t>
+        </is>
+      </c>
+      <c r="D88" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ismaélisme</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Isma%C3%A9lisme" title=" Wikipedia"&gt;L’ismaélisme&lt;/a&gt; est une branche du chiisme née au VIIIe siècle d’une querelle de succession : à la mort de l’imam Ja’far al-Sadiq, en 765, ses fidèles reconnaissent pour héritier son fils Ismaïl, et non son frère. Pour les ismaéliens, l’imam vivant, descendant du Prophète, est le guide qui détient le sens véritable de la révélation.&lt;/p&gt; &lt;p&gt;Leur pensée repose sur la distinction entre l’apparent (&lt;em&gt;zâhir&lt;/em&gt;), la lettre de la Loi et les rites, et le caché (&lt;em&gt;bâtin&lt;/em&gt;), la vérité spirituelle qu’ils contiennent. L’interprétation (&lt;em&gt;ta’wîl&lt;/em&gt;) consiste à remonter de l’un à l’autre. Pour exprimer ce sens caché, les penseurs ismaéliens des Xe et XIe siècles bâtissent une grande philosophie inspirée du néoplatonisme : Dieu, au-delà de tout attribut, fait émaner un premier Intellect, dont procèdent l’Âme et l’univers ; &lt;a href="https://fr.wikipedia.org/wiki/Hamid_al-Din_al-Kirmani" title=" Wikipedia"&gt;al-Kirmani&lt;/a&gt; décrit ainsi une hiérarchie de dix intelligences. On rattache souvent à ce milieu les &lt;a href="https://fr.wikipedia.org/wiki/Ikhwan_al-Safa" title=" Wikipedia"&gt;Frères de la Pureté&lt;/a&gt;, auteurs d’une encyclopédie des sciences. Le califat des &lt;a href="https://fr.wikipedia.org/wiki/Fatimides" title=" Wikipedia"&gt;Fatimides&lt;/a&gt;, qui règne sur l’Égypte de 969 à 1171 et fonde Le Caire et la mosquée al-Azhar, en fait une doctrine d’État.&lt;/p&gt; &lt;p&gt;Le poète persan Nasir Khusraw en est l’un des grands maîtres ; la branche nizârite s’établit en Iran dans la forteresse d’&lt;a href="https://fr.wikipedia.org/wiki/Alamut" title=" Wikipedia"&gt;Alamut&lt;/a&gt;, où le savant Nasir al-Din al-Tusi travaille de longues années, jusqu’à sa prise par les Mongols en 1256. Dépeints à tort par leurs ennemis comme une secte d’« Assassins », les ismaéliens sont aujourd’hui plusieurs millions dans le monde, et la branche nizârite reconnaît pour imam l’&lt;a href="https://fr.wikipedia.org/wiki/Aga_Khan" title=" Wikipedia"&gt;Aga Khan&lt;/a&gt;.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J88" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">branche du chiisme qui cherche le sens caché du Coran et l’exprime dans une grande philosophie néoplatonicienne.</t>
+        </is>
+      </c>
+      <c r="K88" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Théologie et spiritualité;Métaphysique</t>
+        </is>
+      </c>
+      <c r="L88" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hamid al-Din AL-KIRMANI;NASIR KHUSRAW;Nasir AL-DIN AL-TUSI</t>
+        </is>
+      </c>
+      <c r="M88" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">islam-juif</t>
+        </is>
+      </c>
+      <c r="N88"/>
+    </row>
+    <row r="89" customFormat="false" ht="225.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A89" s="1">
+        <v>900</v>
+      </c>
+      <c r="C89" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">900</t>
+        </is>
+      </c>
+      <c r="D89" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Maturidisme</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Maturidisme" title=" Wikipedia"&gt;Le maturidisme&lt;/a&gt; est l’une des deux grandes écoles de théologie rationnelle (&lt;em&gt;kalâm&lt;/em&gt;) de l’islam sunnite, avec l’acharisme. Il est fondé au Xe siècle à Samarcande, en Asie centrale, par Abu Mansur al-Maturidi, qui se réclame de l’héritage de l’imam &lt;a href="https://fr.wikipedia.org/wiki/Ab%C3%BB_Han%C3%AEfa" title=" Wikipedia"&gt;Abû Hanîfa&lt;/a&gt;, fondateur de l’école juridique &lt;a href="https://fr.wikipedia.org/wiki/Hanafisme" title=" Wikipedia"&gt;hanafite&lt;/a&gt;. Comme son contemporain al-Ash’ari, al-Maturidi cherche une voie moyenne entre les mutazilites, qui soumettaient la foi à la raison, et les traditionalistes, qui refusaient tout raisonnement sur Dieu.&lt;/p&gt; &lt;p&gt;Mais il fait une plus grande place à la raison. Pour les maturidites, l’être humain peut savoir par sa seule intelligence que Dieu existe et distinguer le bien du mal, même sans avoir reçu de révélation : le bien et le mal sont inscrits dans les choses, et la révélation vient confirmer et préciser ce que la raison entrevoit. Ils défendent aussi plus nettement la liberté humaine : Dieu crée les actes, mais l’être humain les choisit réellement et en porte la responsabilité. La foi, enfin, est l’adhésion du cœur, confirmée par la parole ; elle ne grandit ni ne diminue avec les œuvres. Les différences avec l’acharisme sont subtiles, et les deux écoles finissent par se reconnaître mutuellement comme orthodoxes.&lt;/p&gt; &lt;p&gt;Porté par les dynasties turques, le maturidisme devient la théologie dominante de l’Asie centrale, de l’Empire ottoman et du monde indien. Le petit credo d’al-Nasafi, au XIIe siècle, commenté par al-Taftazani, est étudié dans les écoles jusqu’à nos jours. Il reste aujourd’hui la théologie de référence d’une grande partie des musulmans sunnites, de la Turquie au Pakistan.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J89" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">école de théologie sunnite fondée à Samarcande par al-Maturidi : la raison peut connaître Dieu et le bien avant toute révélation.</t>
+        </is>
+      </c>
+      <c r="K89" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Théologie et spiritualité;Épistémologie</t>
+        </is>
+      </c>
+      <c r="L89" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Abu Mansur AL-MATURIDI;Abu Hafs AL-NASAFI</t>
+        </is>
+      </c>
+      <c r="M89" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">islam-juif</t>
+        </is>
+      </c>
+      <c r="N89"/>
+    </row>
+    <row r="90" customFormat="false" ht="225.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A90" s="1">
+        <v>1200</v>
+      </c>
+      <c r="C90" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1200</t>
+        </is>
+      </c>
+      <c r="D90" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kabbale</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Kabbale" title=" Wikipedia"&gt;La Kabbale&lt;/a&gt;, la « tradition reçue », est la grande tradition mystique et ésotérique du judaïsme. Elle apparaît à la fin du XIIe siècle en Provence, puis en Catalogne, où Nahmanide, à Gérone, lui donne son autorité, et en Castille, où &lt;a href="https://fr.wikipedia.org/wiki/Mo%C3%AFse_de_Le%C3%B3n" title=" Wikipedia"&gt;Moïse de León&lt;/a&gt; compose vers 1280 le &lt;em&gt;Zohar&lt;/em&gt;, « livre de la Splendeur », qui en devient le texte majeur.&lt;/p&gt; &lt;p&gt;Elle distingue en Dieu l’&lt;em&gt;En Sof&lt;/em&gt;, « l’Infini », absolument caché, et les dix &lt;a href="https://fr.wikipedia.org/wiki/Sephiroth_%28Kabbale%29" title=" Wikipedia"&gt;&lt;em&gt;sefirot&lt;/em&gt;&lt;/a&gt;, émanations par lesquelles il se manifeste : sagesse, intelligence, amour, rigueur, beauté, jusqu’à la &lt;a href="https://fr.wikipedia.org/wiki/Shekhina" title=" Wikipedia"&gt;&lt;em&gt;Shekhina&lt;/em&gt;&lt;/a&gt;, la présence divine dans le monde, que la Kabbale conçoit comme féminine et exilée avec le peuple. Chaque mot de la Torah, chaque commandement accompli, agit sur l’harmonie de ces puissances. Après l’expulsion des Juifs d’Espagne, en 1492, la Kabbale se renouvelle à Safed, en Galilée, autour d’&lt;a href="https://fr.wikipedia.org/wiki/Isaac_Louria" title=" Wikipedia"&gt;Isaac Louria&lt;/a&gt;. Pour faire place au monde, l’Infini a dû se retirer en lui-même : c’est le &lt;a href="https://fr.wikipedia.org/wiki/Tsimtsoum" title=" Wikipedia"&gt;&lt;em&gt;tsimtsoum&lt;/em&gt;&lt;/a&gt;. Puis les « vases » qui devaient recevoir sa lumière se sont brisés, et des étincelles divines sont tombées dans la matière. La tâche de l’être humain est le &lt;a href="https://fr.wikipedia.org/wiki/Tikkoun_Olam" title=" Wikipedia"&gt;&lt;em&gt;tikkoun&lt;/em&gt;&lt;/a&gt;, la réparation du monde, en relevant ces étincelles par la prière et les actes justes. Ce messianisme intérieur nourrit au XVIIe siècle l’aventure de Sabbataï Tsevi, puis, au XVIIIe, le hassidisme.&lt;/p&gt; &lt;p&gt;À la Renaissance, Pic de la Mirandole fonde une « Kabbale chrétienne ». Longtemps méprisée par les historiens, la Kabbale a été réhabilitée au XXe siècle par les travaux de Gershom Scholem, qui en a fait un objet d’étude majeur.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J90" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tradition mystique du judaïsme qui contemple les dix émanations de Dieu et appelle l’être humain à réparer le monde.</t>
+        </is>
+      </c>
+      <c r="K90" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Théologie et spiritualité;Métaphysique</t>
+        </is>
+      </c>
+      <c r="L90" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Isaac LOURIA;Moïse de LEÓN;NAHMANIDE;Abraham ABOULAFIA</t>
+        </is>
+      </c>
+      <c r="M90" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">islam-juif</t>
+        </is>
+      </c>
+      <c r="N90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" customFormat="false" ht="225.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A91" s="1">
+        <v>1740</v>
+      </c>
+      <c r="C91" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1740</t>
+        </is>
+      </c>
+      <c r="D91" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hassidisme</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Hassidisme" title=" Wikipedia"&gt;Le hassidisme&lt;/a&gt;, de l’hébreu &lt;em&gt;hassid&lt;/em&gt;, « pieux », est un mouvement de renouveau mystique du judaïsme né au XVIIIe siècle en Podolie, dans l’actuelle Ukraine, alors polonaise, autour du Baal Shem Tov, le « Maître du Bon Nom ». Il paraît dans des communautés juives pauvres et éprouvées par les massacres et par la faillite du faux messie Sabbataï Tsevi, où le savoir talmudique est réservé à une élite.&lt;/p&gt; &lt;p&gt;Reprenant les idées de la Kabbale, le hassidisme les met à la portée de tous. Dieu est présent partout, jusque dans les choses les plus humbles : on peut donc le servir non seulement par l’étude, mais par la prière fervente, le chant, la danse et chaque geste du quotidien, accompli avec attention. La joie est une forme de piété, la tristesse un obstacle. La ferveur du cœur compte plus que l’érudition, et le plus simple des fidèles peut s’unir à Dieu. Au centre de chaque communauté se tient le &lt;a href="https://fr.wikipedia.org/wiki/Tsadik" title=" Wikipedia"&gt;&lt;em&gt;tsaddik&lt;/em&gt;&lt;/a&gt;, le « juste », maître spirituel qui guide ses disciples et intercède pour eux. Les maîtres hassidiques enseignent par des récits et des paraboles, comme ceux de &lt;a href="https://fr.wikipedia.org/wiki/Nahman_de_Bratslav" title=" Wikipedia"&gt;Nahman de Bratslav&lt;/a&gt;, arrière-petit-fils du Baal Shem Tov.&lt;/p&gt; &lt;p&gt;Combattu d’abord par les rabbins traditionnels, les &lt;a href="https://fr.wikipedia.org/wiki/Mitnagdim" title=" Wikipedia"&gt;Mitnagdim&lt;/a&gt;, le mouvement gagne une grande partie des Juifs d’Europe de l’Est. Presque anéanti par la Shoah, il renaît aux États-Unis et en Israël, où ses communautés, comme celle de Loubavitch, sont aujourd’hui très vivantes. Martin Buber a fait connaître ses récits en Occident ; Abraham Heschel et Elie Wiesel, issus de familles hassidiques, en ont transmis l’esprit.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J91" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement mystique juif né en Ukraine autour du Baal Shem Tov : servir Dieu dans la joie, l’humilité et chaque geste du quotidien.</t>
+        </is>
+      </c>
+      <c r="K91" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Théologie et spiritualité;Éthique</t>
+        </is>
+      </c>
+      <c r="L91" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BAAL SHEM TOV;Martin BUBER</t>
+        </is>
+      </c>
+      <c r="M91" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">islam-juif</t>
+        </is>
+      </c>
+      <c r="N91"/>
+    </row>
+    <row r="92" customFormat="false" ht="225.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A92" s="1">
+        <v>1770</v>
+      </c>
+      <c r="C92" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1770</t>
+        </is>
+      </c>
+      <c r="D92" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Haskala</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Haskala" title=" Wikipedia"&gt;La Haskala&lt;/a&gt;, de l’hébreu &lt;em&gt;sekhel&lt;/em&gt;, « intelligence », est le mouvement des Lumières juives, né à Berlin dans les années 1770. Ses partisans, les &lt;em&gt;maskilim&lt;/em&gt;, veulent faire sortir les Juifs du ghetto culturel où les ont enfermés des siècles de discriminations, en les ouvrant aux sciences, à la philosophie et aux langues de l’Europe, sans qu’ils renoncent pour autant à leur foi.&lt;/p&gt; &lt;p&gt;Son inspirateur est Moses Mendelssohn, surnommé le « Socrate de Berlin », admiré de Kant et ami de &lt;a href="https://fr.wikipedia.org/wiki/Gotthold_Ephraim_Lessing" title=" Wikipedia"&gt;Lessing&lt;/a&gt;, qui fait de lui le modèle de son &lt;em&gt;Nathan le Sage&lt;/em&gt;. Il traduit la Torah en allemand, imprimée en caractères hébraïques, pour que les Juifs apprennent la langue du pays. Dans &lt;em&gt;Jérusalem&lt;/em&gt; (1783), il défend la liberté de conscience et la séparation de l’État et de la religion : le judaïsme, dit-il, n’impose pas de croyances, il prescrit des pratiques, et ses vérités sont celles de la raison, accessibles à tous les hommes. Autour de lui, le médecin Marcus Herz, élève de Kant, et David Friedländer, qui plaide pour l’émancipation civile des Juifs de Prusse, poursuivent son œuvre. La Haskala fonde des écoles modernes, une presse et fait renaître l’hébreu comme langue littéraire profane.&lt;/p&gt; &lt;p&gt;Au XIXe siècle, elle gagne la Galicie et l’Empire russe. Elle prépare le &lt;a href="https://fr.wikipedia.org/wiki/Juda%C3%AFsme_r%C3%A9form%C3%A9" title=" Wikipedia"&gt;judaïsme libéral&lt;/a&gt;, la &lt;a href="https://fr.wikipedia.org/wiki/Wissenschaft_des_Judentums" title=" Wikipedia"&gt;« science du judaïsme »&lt;/a&gt;, l’étude historique de sa tradition, et indirectement le sionisme. Ses adversaires lui ont reproché d’ouvrir la voie à l’assimilation ; ses héritiers y voient l’entrée du judaïsme dans la modernité.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J92" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">les « Lumières juives » de Mendelssohn : unir la fidélité au judaïsme, la raison et la culture européenne.</t>
+        </is>
+      </c>
+      <c r="K92" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Philosophie politique;Théologie et spiritualité</t>
+        </is>
+      </c>
+      <c r="L92" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Moses MENDELSSOHN</t>
+        </is>
+      </c>
+      <c r="M92" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">islam-juif</t>
+        </is>
+      </c>
+      <c r="N92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" customFormat="false" ht="225.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A93" s="1">
+        <v>1600</v>
+      </c>
+      <c r="C93" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1600</t>
+        </is>
+      </c>
+      <c r="D93" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">École d'Ispahan</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;On appelle &lt;a href="https://fr.wikipedia.org/wiki/%C3%89cole_d%27Ispahan" title=" Wikipedia"&gt;École d’Ispahan&lt;/a&gt; le grand renouveau philosophique qui se produit en Iran au XVIIe siècle, à Ispahan, capitale de la dynastie &lt;a href="https://fr.wikipedia.org/wiki/Dynastie_des_S%C3%A9f%C3%A9vides" title=" Wikipedia"&gt;safavide&lt;/a&gt; qui a fait du chiisme la religion d’État. Alors que l’on a longtemps cru la philosophie islamique morte après Averroès, elle connaît là une nouvelle floraison, qui unit l’héritage d’Avicenne, la sagesse de l’illumination de Sohrawardi, la mystique d’Ibn Arabî et la théologie chiite.&lt;/p&gt; &lt;p&gt;Son premier maître est &lt;a href="https://fr.wikipedia.org/wiki/Mir_Damad" title=" Wikipedia"&gt;Mir Damad&lt;/a&gt;, philosophe et théologien, qui réfléchit sur le rapport entre l’éternité et le temps et signe ses poèmes du nom d’« Ishrâq », l’illumination. Son disciple Molla Sadra en est le génie. Dans ses &lt;em&gt;Quatre voyages de l’intellect&lt;/em&gt;, il fonde la « sagesse transcendante » (&lt;em&gt;al-hikma al-muta’aliya&lt;/em&gt;), qui veut unir la démonstration rationnelle, l’expérience spirituelle et la révélation. Sa thèse centrale est la primauté de l’existence : ce qui est réel, ce n’est pas l’essence, la définition des choses, mais l’acte d’exister, unique et présent en toutes choses à des degrés différents, comme une même lumière plus ou moins intense. Il affirme aussi le « mouvement substantiel » : l’être des choses n’est pas fixe, il est lui-même en devenir, si bien que le monde tout entier est en marche vers sa perfection.&lt;/p&gt; &lt;p&gt;Prolongée en Iran jusqu’à nos jours, par Sabzevari au XIXe siècle puis par Allameh Tabatabaï et Morteza Motahhari, cette école a été révélée au public occidental par &lt;a href="https://fr.wikipedia.org/wiki/Henry_Corbin" title=" Wikipedia"&gt;Henry Corbin&lt;/a&gt;, qui lui a donné son nom. Elle a aussi profondément marqué le clergé chiite iranien du XXe siècle.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J93" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">renaissance de la philosophie dans l’Iran chiite des Safavides, dont Molla Sadra est le sommet avec sa « sagesse transcendante ».</t>
+        </is>
+      </c>
+      <c r="K93" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Métaphysique;Théologie et spiritualité</t>
+        </is>
+      </c>
+      <c r="L93" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Molla SADRA;MIR DAMAD;Allameh TABATABAÏ</t>
+        </is>
+      </c>
+      <c r="M93" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">islam-juif</t>
+        </is>
+      </c>
+      <c r="N93"/>
+    </row>
+    <row r="94" customFormat="false" ht="225.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A94" s="1">
+        <v>1878</v>
+      </c>
+      <c r="C94" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1878</t>
+        </is>
+      </c>
+      <c r="D94" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sophiologie</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Sophiologie" title=" Wikipedia"&gt;La sophiologie&lt;/a&gt; est un courant de la philosophie religieuse russe, né à la fin du XIXe siècle, qui fait de la &lt;a href="https://fr.wikipedia.org/wiki/Sophia_%28philosophie%29" title=" Wikipedia"&gt;Sagesse divine&lt;/a&gt;, Sophia, le cœur de sa réflexion. Elle reprend une figure de la Bible, où la Sagesse est présentée comme la compagne de Dieu lors de la création, et une longue tradition mystique, du platonisme à Jacob Boehme. Son fondateur est Vladimir Soloviev, qui raconte avoir eu trois visions de Sophia, la dernière dans le désert d’Égypte, en 1875.&lt;/p&gt; &lt;p&gt;Dans ses &lt;em&gt;Leçons sur la divino-humanité&lt;/em&gt; (1878), Soloviev décrit Sophia comme l’âme du monde, l’unité idéale de toutes les créatures en Dieu : elle est le lien entre le Créateur et la création, ce par quoi le monde n’est pas étranger à Dieu. L’histoire a pour sens la réunion progressive de l’humanité et du divin, dont le Christ, Dieu fait homme, est le modèle. Le prêtre et savant Pavel Florensky reprend cette intuition dans &lt;em&gt;La Colonne et le Fondement de la vérité&lt;/em&gt; (1914), en y mêlant mathématiques, théologie et histoire de l’art. Mais c’est Sergueï Boulgakov, économiste marxiste devenu prêtre orthodoxe, qui en fait un vaste système théologique dans son exil parisien, à l’&lt;a href="https://fr.wikipedia.org/wiki/Institut_Saint-Serge" title=" Wikipedia"&gt;Institut Saint-Serge&lt;/a&gt; : la Sagesse est la nature même de Dieu, qui se révèle dans le monde créé, si bien que la création tout entière est appelée à être transfigurée.&lt;/p&gt; &lt;p&gt;En 1935, l’Église orthodoxe russe condamne les thèses de Boulgakov, et les théologiens Vladimir Lossky et Georges Florovsky les critiquent sévèrement. La sophiologie a pourtant marqué les poètes symbolistes, comme Alexandre Blok et Andreï Biély, et elle inspire aujourd’hui une théologie de la création attentive à l’écologie.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J94" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">philosophie religieuse russe de la Sagesse divine, Sophia, qui unit Dieu et le monde : Soloviev, Florensky, Boulgakov.</t>
+        </is>
+      </c>
+      <c r="K94" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Théologie et spiritualité;Métaphysique</t>
+        </is>
+      </c>
+      <c r="L94" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vladimir SOLOVIEV;Sergueï BOULGAKOV;Pavel FLORENSKY</t>
+        </is>
+      </c>
+      <c r="M94" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">russe</t>
+        </is>
+      </c>
+      <c r="N94"/>
+    </row>
+    <row r="95" customFormat="false" ht="225.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A95" s="1">
+        <v>1921</v>
+      </c>
+      <c r="C95" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1921</t>
+        </is>
+      </c>
+      <c r="D95" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Eurasisme</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Eurasisme" title=" Wikipedia"&gt;L’eurasisme&lt;/a&gt; est un courant de pensée né en 1921 dans l’émigration russe, après la révolution bolchevique, avec le recueil &lt;em&gt;L’Exode vers l’Orient&lt;/em&gt;, publié à Sofia par un petit groupe de jeunes intellectuels exilés : le linguiste &lt;a href="https://fr.wikipedia.org/wiki/Nikola%C3%AF_Sergue%C3%AFevitch_Troubetsko%C3%AF" title=" Wikipedia"&gt;Nikolaï Troubetskoï&lt;/a&gt;, le géographe Piotr Savitski, le musicologue Pierre Souvtchinski et le théologien Georges Florovsky.&lt;/p&gt; &lt;p&gt;Leur thèse est que la Russie n’est ni une partie de l’Europe ni une partie de l’Asie, mais un monde à part, l’« Eurasie », dont la grande plaine, des Carpates au Pacifique, a façonné l’unité des peuples slaves, turcs et finno-ougriens. Contre les occidentalistes, ils refusent l’idée d’une civilisation européenne universelle : dans &lt;em&gt;L’Europe et l’humanité&lt;/em&gt; (1920), Troubetskoï y voit l’égoïsme d’une culture « romano-germanique » qui s’impose aux autres. Contre les slavophiles, ils réhabilitent l’héritage asiatique de la Russie, et jusqu’à l’empire de Gengis Khan, qui aurait le premier unifié cet espace. Ils rêvent d’un État fondé sur une idéologie commune et sur l’orthodoxie, distinct à la fois de la démocratie libérale et du communisme. Florovsky s’en éloigne vite et critique en 1928 ce qu’il appelle une « vérité des questions » devenue une « erreur des réponses ». Le mouvement se divise à la fin des années 1920, une partie se rapprochant du régime soviétique.&lt;/p&gt; &lt;p&gt;Prolongé en URSS par l’historien &lt;a href="https://fr.wikipedia.org/wiki/Lev_Goumilev" title=" Wikipedia"&gt;Lev Goumilev&lt;/a&gt;, l’eurasisme renaît après 1991 sous la forme d’un « néo-eurasisme » porté par &lt;a href="https://fr.wikipedia.org/wiki/Alexandre_Douguine" title=" Wikipedia"&gt;Alexandre Douguine&lt;/a&gt;, idéologue d’extrême droite, et influence aujourd’hui la géopolitique nationaliste et impériale de la Russie.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J95" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">doctrine née dans l’émigration russe : la Russie ne serait ni l’Europe ni l’Asie, mais une civilisation à part, l’« Eurasie ».</t>
+        </is>
+      </c>
+      <c r="K95" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Philosophie politique</t>
+        </is>
+      </c>
+      <c r="L95" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nikolaï TROUBETSKOÏ;Georges FLOROVSKY</t>
+        </is>
+      </c>
+      <c r="M95" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">russe</t>
+        </is>
+      </c>
+      <c r="N95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">asie-est</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" customFormat="false" ht="225.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A96" s="1">
+        <v>1945</v>
+      </c>
+      <c r="C96" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1945</t>
+        </is>
+      </c>
+      <c r="D96" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ethnophilosophie</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://en.wikipedia.org/wiki/Ethnophilosophy" title=" Wikipedia (en)"&gt;L’ethnophilosophie&lt;/a&gt; désigne la démarche qui cherche la philosophie d’un peuple dans ses langues, ses proverbes, ses mythes et ses croyances, plutôt que dans les œuvres de penseurs individuels. Elle naît en 1945 avec &lt;a href="https://fr.wikipedia.org/wiki/La_Philosophie_bantoue" title=" Wikipedia"&gt;&lt;em&gt;La Philosophie bantoue&lt;/em&gt;&lt;/a&gt; du missionnaire belge &lt;a href="https://fr.wikipedia.org/wiki/Placide_Tempels" title=" Wikipedia"&gt;Placide Tempels&lt;/a&gt;, qui veut montrer, contre le préjugé colonial, que les Africains ont une pensée cohérente, fondée sur l’idée de « force vitale » : pour les Bantous, l’être est force, et toute chose est une force qui peut croître ou décroître.&lt;/p&gt; &lt;p&gt;Des penseurs africains reprennent cette démarche en la retournant contre le regard colonial. Le prêtre rwandais Alexis Kagame, dans &lt;em&gt;La Philosophie bantu-rwandaise de l’être&lt;/em&gt; (1956), dégage les catégories de la pensée à partir de la grammaire du kinyarwanda, comme Aristote l’avait fait, selon lui, à partir du grec. Le théologien kényan John Mbiti décrit dans &lt;em&gt;Religions et philosophie africaines&lt;/em&gt; (1969) une conception du temps tournée vers le passé plus que vers l’avenir. Dans l’esprit de la Négritude, il s’agit d’affirmer la dignité des cultures africaines.&lt;/p&gt; &lt;p&gt;À partir des années 1970, cette démarche est vivement critiquée par d’autres philosophes africains. Paulin Hountondji, dans &lt;em&gt;Sur la « philosophie africaine »&lt;/em&gt; (1976), dénonce le « mythe de l’unanimité » : une philosophie n’est pas une vision du monde collective et figée, mais un discours critique, signé, argumenté et ouvert à la discussion. Marcien Towa et Fabien Eboussi Boulaga vont dans le même sens. Le débat sur l’ethnophilosophie a structuré toute la philosophie africaine contemporaine.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J96" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">recherche d’une philosophie africaine dans les langues, les croyances et les traditions des peuples, et débat qu’elle a suscité.</t>
+        </is>
+      </c>
+      <c r="K96" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Métaphysique;Épistémologie</t>
+        </is>
+      </c>
+      <c r="L96" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Placide TEMPELS;Alexis KAGAME;John MBITI</t>
+        </is>
+      </c>
+      <c r="M96" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sud</t>
+        </is>
+      </c>
+      <c r="N96"/>
+    </row>
+    <row r="97" customFormat="false" ht="225.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A97" s="1">
+        <v>1960</v>
+      </c>
+      <c r="C97" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1960</t>
+        </is>
+      </c>
+      <c r="D97" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Socialisme africain</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;On appelle &lt;a href="https://fr.wikipedia.org/wiki/Socialisme_africain" title=" Wikipedia"&gt;socialisme africain&lt;/a&gt; l’ensemble des doctrines par lesquelles plusieurs dirigeants des indépendances africaines, autour de 1960, ont voulu définir une voie propre de développement, distincte à la fois du capitalisme des anciennes puissances coloniales et du communisme soviétique.&lt;/p&gt; &lt;p&gt;Leur idée commune est que l’Afrique n’a pas besoin d’importer le socialisme, car elle le porte déjà dans ses traditions : la solidarité de la famille élargie et du village, la propriété commune de la terre, le partage des biens. Il ne s’agit donc pas de mener une lutte des classes, que les sociétés africaines n’auraient pas connue, mais de moderniser ces solidarités. Au Sénégal, Léopold Sédar Senghor défend un socialisme humaniste et spirituel, nourri de la Négritude et de la pensée de Teilhard de Chardin, qui refuse l’athéisme marxiste. Au Ghana, Kwame Nkrumah, plus proche du marxisme, cherche dans son « consciencisme » une synthèse entre la tradition africaine, l’islam et le christianisme. En Tanzanie, Julius Nyerere en donne la version la plus élaborée avec l’&lt;a href="https://fr.wikipedia.org/wiki/Ujamaa" title=" Wikipedia"&gt;&lt;em&gt;ujamaa&lt;/em&gt;&lt;/a&gt;, mot swahili qui signifie « esprit de famille » : la nation doit vivre comme une grande famille où chacun travaille et où personne n’exploite personne. La &lt;a href="https://fr.wikipedia.org/wiki/D%C3%A9claration_d%27Arusha" title=" Wikipedia"&gt;déclaration d’Arusha&lt;/a&gt; (1967) en fait le programme du pays.&lt;/p&gt; &lt;p&gt;Dans les faits, ces politiques ont souvent abouti à des partis uniques et, en Tanzanie, au regroupement forcé des paysans dans des villages collectifs, qui fut un échec économique, reconnu par Nyerere lui-même. Elles restent pourtant une tentative originale de penser le développement à partir des valeurs africaines.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J97" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">socialisme des indépendances fondé sur les solidarités communautaires africaines plutôt que sur la lutte des classes.</t>
+        </is>
+      </c>
+      <c r="K97" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Philosophie politique;Éthique</t>
+        </is>
+      </c>
+      <c r="L97" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Julius NYERERE;Léopold Sédar SENGHOR;Kwame NKRUMAH</t>
+        </is>
+      </c>
+      <c r="M97" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sud</t>
+        </is>
+      </c>
+      <c r="N97"/>
+    </row>
+    <row r="98" customFormat="false" ht="225.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A98" s="1">
+        <v>1968</v>
+      </c>
+      <c r="C98" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1968</t>
+        </is>
+      </c>
+      <c r="D98" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Théologie de la libération</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Th%C3%A9ologie_de_la_lib%C3%A9ration" title=" Wikipedia"&gt;La théologie de la libération&lt;/a&gt; est un courant de pensée chrétien, surtout catholique, né en Amérique latine à la fin des années 1960, dans un continent marqué par la misère, les inégalités et les dictatures. Elle s’appuie sur le renouveau du concile Vatican II et sur la &lt;a href="https://fr.wikipedia.org/wiki/Conf%C3%A9rence_de_Medell%C3%ADn" title=" Wikipedia"&gt;conférence des évêques latino-américains de Medellín&lt;/a&gt;, en 1968, qui dénonce la « violence institutionnalisée » de l’injustice sociale.&lt;/p&gt; &lt;p&gt;Son texte fondateur est &lt;em&gt;Théologie de la libération&lt;/em&gt; (1971) du prêtre péruvien &lt;a href="https://fr.wikipedia.org/wiki/Gustavo_Guti%C3%A9rrez_Merino" title=" Wikipedia"&gt;Gustavo Gutiérrez&lt;/a&gt;. La théologie n’y est plus seulement une réflexion abstraite sur Dieu, mais une « réflexion critique sur la pratique » : elle part de la situation concrète des pauvres et de leur lutte pour leur dignité. Dieu prend parti pour les opprimés, comme il a libéré Israël de l’esclavage en Égypte ; le salut ne concerne pas seulement l’au-delà, il commence par la libération de toutes les servitudes. D’où l’« option préférentielle pour les pauvres ». Pour comprendre les causes de la pauvreté, ces théologiens utilisent les sciences sociales, y compris l’analyse marxiste. La foi se vit dans les &lt;a href="https://fr.wikipedia.org/wiki/Communaut%C3%A9_eccl%C3%A9siale_de_base" title=" Wikipedia"&gt;communautés ecclésiales de base&lt;/a&gt;, où les pauvres lisent eux-mêmes la Bible à la lumière de leur vie. Le Brésilien Leonardo Boff, le jésuite Ignacio Ellacuría, assassiné au Salvador en 1989, et les réflexions de Paulo Freire et d’Enrique Dussel lui sont proches.&lt;/p&gt; &lt;p&gt;Rome, sous Jean-Paul II, critique dans les années 1980 son usage du marxisme et impose le silence à Boff. Sa reconnaissance vient avec le pape François, et l’option pour les pauvres est aujourd’hui reprise par toute l’Église catholique.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J98" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">courant chrétien latino-américain qui place au cœur de la foi l’engagement aux côtés des pauvres et contre l’injustice.</t>
+        </is>
+      </c>
+      <c r="K98" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Théologie et spiritualité;Philosophie politique</t>
+        </is>
+      </c>
+      <c r="L98" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gustavo GUTIÉRREZ;Leonardo BOFF;Enrique DUSSEL;Paulo FREIRE</t>
+        </is>
+      </c>
+      <c r="M98" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sud</t>
+        </is>
+      </c>
+      <c r="N98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" customFormat="false" ht="225.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A99" s="1">
+        <v>1971</v>
+      </c>
+      <c r="C99" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1971</t>
+        </is>
+      </c>
+      <c r="D99" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Philosophie de la libération</t>
+        </is>
+      </c>
+      <c r="E99" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Philosophie_de_la_lib%C3%A9ration" title=" Wikipedia"&gt;La philosophie de la libération&lt;/a&gt; est un mouvement philosophique latino-américain apparu au début des années 1970, en Argentine surtout, autour du congrès national de philosophie de Córdoba en 1971. Il veut faire de la philosophie un instrument d’émancipation pour les peuples d’Amérique latine, dominés économiquement et culturellement, en écho à la &lt;a href="https://fr.wikipedia.org/wiki/Th%C3%A9orie_de_la_d%C3%A9pendance" title=" Wikipedia"&gt;théorie de la dépendance&lt;/a&gt; des économistes.&lt;/p&gt; &lt;p&gt;Il naît d’un débat. En 1968, le Péruvien Augusto Salazar Bondy demande « Existe-t-il une philosophie de notre Amérique ? » et répond qu’une culture dépendante ne peut produire qu’une pensée imitée, inauthentique, tant que dure la domination. Le Mexicain Leopoldo Zea lui répond que la pensée latino-américaine est déjà une philosophie à part entière, qui réfléchit sur sa propre histoire. L’Argentin Enrique Dussel en devient la figure majeure. S’inspirant d’&lt;a href="https://fr.wikipedia.org/wiki/Emmanuel_Levinas" title=" Wikipedia"&gt;Emmanuel Levinas&lt;/a&gt;, il fait de l’Autre, le pauvre, l’Indien, le colonisé, la femme, le point de départ de l’éthique : la philosophie doit écouter la parole de celui que le système exclut. Pour lui, la modernité ne commence pas avec le « je pense » de Descartes, mais en 1492, avec le « je conquiers » des conquistadors. Rodolfo Kusch, de son côté, cherche dans la pensée des peuples andins une autre manière d’être au monde, celle de l’« être là » plutôt que de l’« être quelqu’un ».&lt;/p&gt; &lt;p&gt;Persécutés par la dictature militaire, Dussel et plusieurs autres partent en exil en 1975. Le mouvement a nourri la théologie de la libération, puis la pensée décoloniale, et reste une référence des philosophies du Sud.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J99" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">philosophie latino-américaine qui pense à partir des peuples dominés et dénonce la dépendance culturelle envers l’Europe.</t>
+        </is>
+      </c>
+      <c r="K99" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Éthique;Philosophie politique</t>
+        </is>
+      </c>
+      <c r="L99" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Enrique DUSSEL;Augusto SALAZAR BONDY;Leopoldo ZEA-AGUILAR</t>
+        </is>
+      </c>
+      <c r="M99" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sud</t>
+        </is>
+      </c>
+      <c r="N99"/>
+    </row>
+    <row r="100" customFormat="false" ht="225.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A100" s="1">
+        <v>1981</v>
+      </c>
+      <c r="C100" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1981</t>
+        </is>
+      </c>
+      <c r="D100" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Créolisation</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;La &lt;a href="https://fr.wikipedia.org/wiki/Cr%C3%A9olisation_%28concept%29" title=" Wikipedia"&gt;créolisation&lt;/a&gt; est un courant de pensée né aux Antilles autour de l’œuvre d’Édouard Glissant. Le mot désigne d’abord la naissance des langues et des cultures créoles dans les sociétés de plantation des Caraïbes, où des peuples arrachés à l’Afrique, des colons européens, des Amérindiens et plus tard des travailleurs venus d’Inde ont dû inventer ensemble un monde nouveau. Glissant en fait un concept philosophique pour penser le monde entier.&lt;/p&gt; &lt;p&gt;Dans &lt;a href="https://fr.wikipedia.org/wiki/Le_Discours_antillais" title=" Wikipedia"&gt;&lt;em&gt;Le Discours antillais&lt;/em&gt;&lt;/a&gt; (1981), il développe d’abord l’&lt;a href="https://fr.wikipedia.org/wiki/Antillanit%C3%A9" title=" Wikipedia"&gt;antillanité&lt;/a&gt; : l’identité des Antilles ne se trouve ni dans un retour à l’Afrique, comme le voulait la Négritude, ni dans l’imitation de la France, mais dans l’archipel caribéen lui-même. Avec la créolisation, il montre que la rencontre des cultures ne produit pas un simple mélange prévisible, mais de l’inédit. Reprenant une image de Deleuze et Guattari, il oppose l’« identité-racine », unique, qui exclut l’autre, à l’« identité-rhizome », qui se construit dans la relation. Dans &lt;em&gt;Poétique de la Relation&lt;/em&gt; (1990), il défend le « droit à l’opacité » : comprendre l’autre ne signifie pas le réduire à soi. Il appelle &lt;a href="https://fr.wikipedia.org/wiki/Tout-monde" title=" Wikipedia"&gt;« Tout-Monde »&lt;/a&gt; ce monde où toutes les cultures sont désormais en contact, pour le meilleur et pour le pire, et où nul ne peut plus vivre à l’écart des autres.&lt;/p&gt; &lt;p&gt;En 1989, les écrivains martiniquais Jean Bernabé, &lt;a href="https://fr.wikipedia.org/wiki/Patrick_Chamoiseau" title=" Wikipedia"&gt;Patrick Chamoiseau&lt;/a&gt; et Raphaël Confiant prolongent ce mouvement dans leur &lt;em&gt;Éloge de la &lt;a href="https://fr.wikipedia.org/wiki/Cr%C3%A9olit%C3%A9" title=" Wikipedia"&gt;créolité&lt;/a&gt;&lt;/em&gt;. La pensée de Glissant est aujourd’hui l’une des grandes références de la réflexion sur la mondialisation et les identités.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J100" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pensée antillaise de Glissant : les cultures en contact créent de l’imprévisible ; à l’identité-racine s’oppose l’identité-relation.</t>
+        </is>
+      </c>
+      <c r="K100" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Métaphysique;Philosophie politique</t>
+        </is>
+      </c>
+      <c r="L100" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Édouard GLISSANT</t>
+        </is>
+      </c>
+      <c r="M100" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sud</t>
+        </is>
+      </c>
+      <c r="N100"/>
+    </row>
+    <row r="101" customFormat="false" ht="225.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A101" s="1">
+        <v>1992</v>
+      </c>
+      <c r="C101" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1992</t>
+        </is>
+      </c>
+      <c r="D101" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pensée décoloniale</t>
+        </is>
+      </c>
+      <c r="E101" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;La pensée décoloniale, ou &lt;a href="https://fr.wikipedia.org/wiki/%C3%89tudes_d%C3%A9coloniales" title=" Wikipedia"&gt;études décoloniales&lt;/a&gt;, est un courant né en Amérique latine dans les années 1990. Son point de départ est un article de 1992 du sociologue péruvien &lt;a href="https://fr.wikipedia.org/wiki/An%C3%ADbal_Quijano" title=" Wikipedia"&gt;Aníbal Quijano&lt;/a&gt;, qui forge la notion de « colonialité du pouvoir » : le colonialisme, comme domination politique directe, a pris fin, mais la colonialité, elle, a survécu.&lt;/p&gt; &lt;p&gt;Pour ces penseurs, la modernité européenne et la colonisation des Amériques, à partir de 1492, sont les deux faces d’un même processus. La colonisation a installé une hiérarchie des êtres humains fondée sur la race, une division du travail mondiale et une hiérarchie des savoirs, qui présente la science et la philosophie européennes comme universelles et relègue les autres savoirs au rang de croyances ou de folklore. Cette colonialité continue d’organiser le monde après les indépendances. Le &lt;a href="https://fr.wikipedia.org/wiki/Groupe_modernit%C3%A9/colonialit%C3%A9" title=" Wikipedia"&gt;groupe « modernité/colonialité »&lt;/a&gt;, qui réunit autour de Quijano l’Argentin &lt;a href="https://fr.wikipedia.org/wiki/Walter_Mignolo" title=" Wikipedia"&gt;Walter Mignolo&lt;/a&gt;, Enrique Dussel et d’autres, appelle à une « désobéissance épistémique » : penser à partir des expériences et des savoirs des peuples colonisés, pour un monde où plusieurs mondes seraient possibles. Sylvia Wynter et Lewis Gordon prolongent cette réflexion dans la Caraïbe et chez les Afro-Américains.&lt;/p&gt; &lt;p&gt;Le courant se distingue des études postcoloniales anglophones d’Edward Saïd ou de &lt;a href="https://fr.wikipedia.org/wiki/Gayatri_Chakravorty_Spivak" title=" Wikipedia"&gt;Gayatri Spivak&lt;/a&gt;, nées de la critique littéraire et centrées sur l’Asie et le Moyen-Orient. Il suscite aussi des critiques, y compris en Amérique latine, où Silvia Rivera Cusicanqui lui reproche d’être devenu une mode universitaire du Nord.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J101" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">courant latino-américain pour qui la colonialité du pouvoir et du savoir a survécu à la fin des colonies.</t>
+        </is>
+      </c>
+      <c r="K101" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Philosophie politique;Épistémologie</t>
+        </is>
+      </c>
+      <c r="L101" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aníbal QUIJANO;Walter MIGNOLO;Enrique DUSSEL;Sylvia WYNTER</t>
+        </is>
+      </c>
+      <c r="M101" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sud</t>
+        </is>
+      </c>
+      <c r="N101"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
Silvia Rivera Cusicanqui : portrait, vidéo et texte ; Kalâm : crédit de la vidéo
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-courant-pensee-oriental.xlsx
+++ b/data/frise-courant-pensee-oriental.xlsx
@@ -2621,88 +2621,80 @@
         </is>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="132.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="14" t="n">
-        <v>1090</v>
-      </c>
-      <c r="B8" s="14"/>
-      <c r="C8" s="14" t="s">
-        <v>44</v>
-      </c>
-      <c r="D8" s="15" t="s">
-        <v>45</v>
-      </c>
-      <c r="E8" s="16" t="s">
-        <v>46</v>
-      </c>
-      <c r="F8" s="14" t="s">
-        <v>47</v>
-      </c>
-      <c r="G8" s="16" t="s">
-        <v>48</v>
-      </c>
-      <c r="H8" s="14"/>
-      <c r="I8" s="14"/>
-      <c r="J8" s="2" t="s">
-        <v>49</v>
+    <row r="8" customFormat="false" ht="353.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="n">
+        <v>720</v>
+      </c>
+      <c r="C8" s="1" t="n">
+        <v>720</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>212</v>
+      </c>
+      <c r="E8" s="21" t="s">
+        <v>213</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">le kalâm musulman par ikarim</t>
+        </is>
+      </c>
+      <c r="J8" s="21" t="s">
+        <v>216</v>
       </c>
       <c r="K8" s="2" t="s">
         <v>22</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="N8" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="O8" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mouvement</t>
-        </is>
-      </c>
-      <c r="P8" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Christianisme antique et médiéval</t>
-        </is>
-      </c>
-      <c r="Q8" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Néoplatonisme</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="135.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1" t="n">
-        <v>-1000</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Herm%C3%A9neutique_biblique" title=" Wikipedia"&gt;L’Herméneutique juive&lt;/a&gt; désigne l’ensemble des méthodes d’interprétation des textes sacrés du judaïsme : la Torah et la Bible hébraïque, puis la Mishna et le &lt;a href="https://fr.wikipedia.org/wiki/Talmud" title=" Wikipedia"&gt;Talmud&lt;/a&gt;. Elle repose sur une idée fondatrice : à côté de la Torah écrite, Moïse aurait reçu au Sinaï une Torah orale, transmise de maître à disciple, qui en donne le sens. Le texte n’est donc jamais clos, il appelle un commentaire sans fin, et l’étude elle-même devient un acte religieux. « La Torah a soixante-dix visages », dit un adage rabbinique.&lt;/p&gt; &lt;p&gt;Cette tradition prend forme avec les sages de l’époque du Second Temple. Hillel, vers le début de notre ère, formule sept règles d’interprétation, que Rabbi Ishmaël porte à treize au IIe siècle, tandis que Rabbi Akiva cherche un sens à chaque lettre. Le &lt;a href="https://fr.wikipedia.org/wiki/Midrash" title=" Wikipedia"&gt;midrash&lt;/a&gt; commente les versets pour en tirer soit des lois (&lt;em&gt;halakha&lt;/em&gt;), soit des récits et des leçons morales (&lt;em&gt;aggada&lt;/em&gt;). La Mishna, mise par écrit vers 200, puis les Talmuds de Jérusalem et de Babylone, achevés vers 400 et 500, consignent des débats où l’opinion minoritaire est conservée à côté de celle qui l’emporte. Au Moyen Âge, on distingue quatre niveaux de sens, résumés par le mot PaRDeS : &lt;em&gt;peshat&lt;/em&gt;, le sens littéral, &lt;em&gt;remez&lt;/em&gt;, l’allusion, &lt;em&gt;derash&lt;/em&gt;, l’interprétation, et &lt;em&gt;sod&lt;/em&gt;, le secret mystique de la Kabbale.&lt;/p&gt; &lt;p&gt;Rachi de Troyes, Maïmonide et Nahmanide en sont les grands commentateurs. Au XXe siècle, Emmanuel Levinas renouvelle la lecture du Talmud, et cette tradition a nourri les théories modernes de l’interprétation.&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>56</v>
-      </c>
+        <v>58</v>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Théologie de l’islam (kalâm)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="132.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="14" t="n">
+        <v>1090</v>
+      </c>
+      <c r="B9" s="14"/>
+      <c r="C9" s="14" t="s">
+        <v>44</v>
+      </c>
+      <c r="D9" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="E9" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="F9" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="G9" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="H9" s="14"/>
+      <c r="I9" s="14"/>
       <c r="J9" s="2" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="K9" s="2" t="s">
         <v>22</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="N9" s="1" t="s">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="O9" s="1" t="inlineStr">
         <is>
@@ -2711,11 +2703,16 @@
       </c>
       <c r="P9" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pensée juive</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="138" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+          <t xml:space="preserve">Christianisme antique et médiéval</t>
+        </is>
+      </c>
+      <c r="Q9" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Néoplatonisme</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="135.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="n">
         <v>-1000</v>
       </c>
@@ -2723,119 +2720,114 @@
         <v>52</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>60</v>
+        <v>53</v>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Herm%C3%A9neutique_biblique" title=" Wikipedia"&gt;L’Herméneutique juive&lt;/a&gt; désigne l’ensemble des méthodes d’interprétation des textes sacrés du judaïsme : la Torah et la Bible hébraïque, puis la Mishna et le &lt;a href="https://fr.wikipedia.org/wiki/Talmud" title=" Wikipedia"&gt;Talmud&lt;/a&gt;. Elle repose sur une idée fondatrice : à côté de la Torah écrite, Moïse aurait reçu au Sinaï une Torah orale, transmise de maître à disciple, qui en donne le sens. Le texte n’est donc jamais clos, il appelle un commentaire sans fin, et l’étude elle-même devient un acte religieux. « La Torah a soixante-dix visages », dit un adage rabbinique.&lt;/p&gt; &lt;p&gt;Cette tradition prend forme avec les sages de l’époque du Second Temple. Hillel, vers le début de notre ère, formule sept règles d’interprétation, que Rabbi Ishmaël porte à treize au IIe siècle, tandis que Rabbi Akiva cherche un sens à chaque lettre. Le &lt;a href="https://fr.wikipedia.org/wiki/Midrash" title=" Wikipedia"&gt;midrash&lt;/a&gt; commente les versets pour en tirer soit des lois (&lt;em&gt;halakha&lt;/em&gt;), soit des récits et des leçons morales (&lt;em&gt;aggada&lt;/em&gt;). La Mishna, mise par écrit vers 200, puis les Talmuds de Jérusalem et de Babylone, achevés vers 400 et 500, consignent des débats où l’opinion minoritaire est conservée à côté de celle qui l’emporte. Au Moyen Âge, on distingue quatre niveaux de sens, résumés par le mot PaRDeS : &lt;em&gt;peshat&lt;/em&gt;, le sens littéral, &lt;em&gt;remez&lt;/em&gt;, l’allusion, &lt;em&gt;derash&lt;/em&gt;, l’interprétation, et &lt;em&gt;sod&lt;/em&gt;, le secret mystique de la Kabbale.&lt;/p&gt; &lt;p&gt;Rachi de Troyes, Maïmonide et Nahmanide en sont les grands commentateurs. Au XXe siècle, Emmanuel Levinas renouvelle la lecture du Talmud, et cette tradition a nourri les théories modernes de l’interprétation.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F10" s="1" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="K10" s="2" t="s">
         <v>22</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mouvement</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Pensées autochtones</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="144.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="9" t="n">
-        <v>-700</v>
-      </c>
-      <c r="B11" s="9"/>
-      <c r="C11" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="D11" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="E11" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="F11" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="G11" s="11" t="s">
-        <v>69</v>
-      </c>
-      <c r="H11" s="9"/>
-      <c r="I11" s="9"/>
+        <v>58</v>
+      </c>
+      <c r="N10" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="O10" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P10" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pensée juive</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="138" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="n">
+        <v>-1000</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>62</v>
+      </c>
       <c r="J11" s="2" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="K11" s="2" t="s">
         <v>22</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="N11" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="O11" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mouvement</t>
-        </is>
-      </c>
-      <c r="P11" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ésotérismes et gnoses</t>
-        </is>
-      </c>
-      <c r="Q11" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Egypte antique;Platonisme</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="50.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="1" t="n">
-        <v>1340</v>
-      </c>
-      <c r="C12" s="1" t="n">
-        <v>1340</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/H%C3%A9sychasme" title=" Wikipedia"&gt;L’Hésychasme&lt;/a&gt; est une tradition mystique et contemplative du christianisme orthodoxe. Son nom vient du grec &lt;em&gt;hésychia&lt;/em&gt;, « silence, tranquillité » : il s’agit de faire taire les pensées pour s’unir à Dieu dans le calme du cœur. Ses racines remontent aux moines et ermites d’Égypte et de Syrie, les Pères du désert, aux IVe et Ve siècles, puis à des maîtres comme Jean Climaque, auteur de &lt;em&gt;L’Échelle sainte&lt;/em&gt; au VIIe siècle, et Syméon le Nouveau Théologien vers l’an mil.&lt;/p&gt; &lt;p&gt;Sa pratique centrale est la &lt;a href="https://fr.wikipedia.org/wiki/Pri%C3%A8re_du_c%C5%93ur" title=" Wikipedia"&gt;prière de Jésus&lt;/a&gt; : le moine répète sans cesse « Seigneur Jésus-Christ, Fils de Dieu, aie pitié de moi », au rythme de sa respiration, la tête inclinée vers la poitrine, pour que la prière descende de l’intelligence dans le cœur. Au XIVe siècle, des moines du mont Athos disent voir ainsi la lumière divine, celle qui entoura le Christ lors de sa Transfiguration sur le mont Thabor. Le moine calabrais Barlaam les accuse de superstition : Dieu ne peut pas être vu. &lt;a href="https://fr.wikipedia.org/wiki/Gr%C3%A9goire_Palamas" title=" Wikipedia"&gt;Grégoire Palamas&lt;/a&gt;, futur archevêque de Thessalonique, répond en distinguant l’essence de Dieu, à jamais inaccessible, et ses énergies, qui se communiquent réellement à l’homme et rendent possible sa « divinisation ». Des conciles réunis à Constantinople lui donnent raison en 1341 et en 1351.&lt;/p&gt; &lt;p&gt;En 1782 paraît la &lt;em&gt;Philocalie&lt;/em&gt;, recueil de textes hésychastes bientôt traduit en slavon. L’hésychasme inspire alors les « startsy », les maîtres spirituels de Russie, et les &lt;em&gt;Récits d’un pèlerin russe&lt;/em&gt; ; il reste au cœur de la spiritualité orthodoxe.&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>74</v>
-      </c>
+        <v>64</v>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pensées autochtones</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="144.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="9" t="n">
+        <v>-700</v>
+      </c>
+      <c r="B12" s="9"/>
+      <c r="C12" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="D12" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="E12" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="G12" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="H12" s="9"/>
+      <c r="I12" s="9"/>
       <c r="J12" s="2" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="K12" s="2" t="s">
         <v>22</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>50</v>
+        <v>23</v>
       </c>
       <c r="N12" s="1" t="s">
-        <v>76</v>
+        <v>58</v>
       </c>
       <c r="O12" s="1" t="inlineStr">
         <is>
@@ -2844,81 +2836,91 @@
       </c>
       <c r="P12" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Christianisme antique et médiéval</t>
+          <t xml:space="preserve">Ésotérismes et gnoses</t>
         </is>
       </c>
       <c r="Q12" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Patristique</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="111.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="14" t="n">
-        <v>-600</v>
-      </c>
-      <c r="B13" s="14"/>
-      <c r="C13" s="14" t="s">
-        <v>77</v>
-      </c>
-      <c r="D13" s="15" t="s">
-        <v>78</v>
-      </c>
-      <c r="E13" s="16" t="s">
-        <v>79</v>
-      </c>
-      <c r="F13" s="14" t="s">
-        <v>80</v>
-      </c>
-      <c r="G13" s="16" t="s">
-        <v>81</v>
-      </c>
-      <c r="H13" s="14"/>
-      <c r="I13" s="14"/>
+          <t xml:space="preserve">Egypte antique;Platonisme</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="50.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="n">
+        <v>1340</v>
+      </c>
+      <c r="C13" s="1" t="n">
+        <v>1340</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/H%C3%A9sychasme" title=" Wikipedia"&gt;L’Hésychasme&lt;/a&gt; est une tradition mystique et contemplative du christianisme orthodoxe. Son nom vient du grec &lt;em&gt;hésychia&lt;/em&gt;, « silence, tranquillité » : il s’agit de faire taire les pensées pour s’unir à Dieu dans le calme du cœur. Ses racines remontent aux moines et ermites d’Égypte et de Syrie, les Pères du désert, aux IVe et Ve siècles, puis à des maîtres comme Jean Climaque, auteur de &lt;em&gt;L’Échelle sainte&lt;/em&gt; au VIIe siècle, et Syméon le Nouveau Théologien vers l’an mil.&lt;/p&gt; &lt;p&gt;Sa pratique centrale est la &lt;a href="https://fr.wikipedia.org/wiki/Pri%C3%A8re_du_c%C5%93ur" title=" Wikipedia"&gt;prière de Jésus&lt;/a&gt; : le moine répète sans cesse « Seigneur Jésus-Christ, Fils de Dieu, aie pitié de moi », au rythme de sa respiration, la tête inclinée vers la poitrine, pour que la prière descende de l’intelligence dans le cœur. Au XIVe siècle, des moines du mont Athos disent voir ainsi la lumière divine, celle qui entoura le Christ lors de sa Transfiguration sur le mont Thabor. Le moine calabrais Barlaam les accuse de superstition : Dieu ne peut pas être vu. &lt;a href="https://fr.wikipedia.org/wiki/Gr%C3%A9goire_Palamas" title=" Wikipedia"&gt;Grégoire Palamas&lt;/a&gt;, futur archevêque de Thessalonique, répond en distinguant l’essence de Dieu, à jamais inaccessible, et ses énergies, qui se communiquent réellement à l’homme et rendent possible sa « divinisation ». Des conciles réunis à Constantinople lui donnent raison en 1341 et en 1351.&lt;/p&gt; &lt;p&gt;En 1782 paraît la &lt;em&gt;Philocalie&lt;/em&gt;, recueil de textes hésychastes bientôt traduit en slavon. L’hésychasme inspire alors les « startsy », les maîtres spirituels de Russie, et les &lt;em&gt;Récits d’un pèlerin russe&lt;/em&gt; ; il reste au cœur de la spiritualité orthodoxe.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>74</v>
+      </c>
       <c r="J13" s="2" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="K13" s="2" t="s">
         <v>22</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mouvement</t>
-        </is>
-      </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Les voies dissidentes de l’Inde</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="N13" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O13" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P13" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Christianisme antique et médiéval</t>
+        </is>
+      </c>
+      <c r="Q13" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Patristique</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="111.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="14" t="n">
         <v>-600</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="B14" s="14"/>
+      <c r="C14" s="14" t="s">
         <v>77</v>
       </c>
-      <c r="D14" s="12" t="s">
-        <v>83</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>86</v>
-      </c>
+      <c r="D14" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="E14" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="F14" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="G14" s="16" t="s">
+        <v>81</v>
+      </c>
+      <c r="H14" s="14"/>
+      <c r="I14" s="14"/>
       <c r="J14" s="2" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>88</v>
+        <v>22</v>
       </c>
       <c r="M14" s="2" t="s">
         <v>43</v>
@@ -2934,30 +2936,30 @@
         </is>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="164.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="n">
-        <v>-550</v>
-      </c>
-      <c r="C15" s="17" t="s">
-        <v>89</v>
+        <v>-600</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>77</v>
       </c>
       <c r="D15" s="12" t="s">
-        <v>90</v>
-      </c>
-      <c r="E15" s="13" t="s">
-        <v>91</v>
+        <v>83</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>84</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>92</v>
+        <v>85</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="J15" s="13" t="s">
-        <v>94</v>
+        <v>86</v>
+      </c>
+      <c r="J15" s="2" t="s">
+        <v>87</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>22</v>
+        <v>88</v>
       </c>
       <c r="M15" s="2" t="s">
         <v>43</v>
@@ -2969,141 +2971,141 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Védas et brahmanisme</t>
-        </is>
-      </c>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Védisme</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="174" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="9" t="n">
-        <v>-520</v>
-      </c>
-      <c r="B16" s="9"/>
-      <c r="C16" s="9" t="s">
-        <v>95</v>
-      </c>
-      <c r="D16" s="10" t="s">
-        <v>96</v>
-      </c>
-      <c r="E16" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Confucianisme"  title=" Wikipedia"&gt;Le Confucianisme&lt;/a&gt; est la tradition de pensée issue de &lt;a href="https://fr.wikipedia.org/wiki/Confucius" title=" Wikipedia"&gt;Confucius&lt;/a&gt; (551-479 av. J.-C.), lettré de l’État de Lu, en Chine, qui chercha en vain un prince prêt à appliquer ses idées. Ses paroles, recueillies par ses disciples dans les &lt;em&gt;Entretiens&lt;/em&gt;, proposent de restaurer l’harmonie d’une société en crise non par la force ou par la loi, mais par la vertu, l’éducation et le respect des rites.&lt;/p&gt; &lt;p&gt;Son idéal est l’« homme de bien » (&lt;em&gt;junzi&lt;/em&gt;), qui se perfectionne sans cesse par l’étude. Les vertus cardinales sont l’humanité ou bienveillance (&lt;em&gt;ren&lt;/em&gt;), la droiture (&lt;em&gt;yi&lt;/em&gt;), les rites (&lt;em&gt;li&lt;/em&gt;), qui règlent avec justesse les relations humaines, la sagesse (&lt;em&gt;zhi&lt;/em&gt;) et la fidélité à la parole donnée (&lt;em&gt;xin&lt;/em&gt;). La société repose sur la famille et la piété filiale : chacun doit tenir son rôle dans les relations entre souverain et sujet, père et fils, époux, aînés et cadets, amis. Le prince gouverne par l’exemple, et les mots doivent correspondre aux choses : c’est la « rectification des noms ». Après Confucius, &lt;a href="https://fr.wikipedia.org/wiki/Mencius" title=" Wikipedia"&gt;Mencius&lt;/a&gt; affirme que la nature humaine est bonne, Xunzi qu’elle doit être redressée par l’éducation. Sous les Han, le confucianisme devient la doctrine officielle de l’empire, et les concours de recrutement des fonctionnaires, fondés sur ses classiques, durent jusqu’en 1905. Au XIIe siècle, Zhu Xi le renouvelle par une métaphysique : c’est le néoconfucianisme.&lt;/p&gt; &lt;p&gt;Il s’étend à la Corée, au Japon et au Viêt Nam. Combattu au XXe siècle comme cause du retard chinois, il connaît aujourd’hui un renouveau en Chine.&lt;/p&gt;  &lt;audio controls title="Le Confucianisme et les valeurs asiatiques par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/18755-14.05.2019-ITEMA_22061347-2.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;</t>
-        </is>
-      </c>
-      <c r="F16" s="9" t="s">
-        <v>98</v>
-      </c>
-      <c r="G16" s="11" t="s">
-        <v>99</v>
-      </c>
-      <c r="H16" s="9"/>
-      <c r="I16" s="9"/>
-      <c r="J16" s="2" t="s">
-        <v>100</v>
+          <t xml:space="preserve">Les voies dissidentes de l’Inde</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="164.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="1" t="n">
+        <v>-550</v>
+      </c>
+      <c r="C16" s="17" t="s">
+        <v>89</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="E16" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="J16" s="13" t="s">
+        <v>94</v>
       </c>
       <c r="K16" s="2" t="s">
         <v>22</v>
       </c>
       <c r="M16" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Védas et brahmanisme</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Védisme</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="174" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="9" t="n">
+        <v>-520</v>
+      </c>
+      <c r="B17" s="9"/>
+      <c r="C17" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="D17" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="E17" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Confucianisme"  title=" Wikipedia"&gt;Le Confucianisme&lt;/a&gt; est la tradition de pensée issue de &lt;a href="https://fr.wikipedia.org/wiki/Confucius" title=" Wikipedia"&gt;Confucius&lt;/a&gt; (551-479 av. J.-C.), lettré de l’État de Lu, en Chine, qui chercha en vain un prince prêt à appliquer ses idées. Ses paroles, recueillies par ses disciples dans les &lt;em&gt;Entretiens&lt;/em&gt;, proposent de restaurer l’harmonie d’une société en crise non par la force ou par la loi, mais par la vertu, l’éducation et le respect des rites.&lt;/p&gt; &lt;p&gt;Son idéal est l’« homme de bien » (&lt;em&gt;junzi&lt;/em&gt;), qui se perfectionne sans cesse par l’étude. Les vertus cardinales sont l’humanité ou bienveillance (&lt;em&gt;ren&lt;/em&gt;), la droiture (&lt;em&gt;yi&lt;/em&gt;), les rites (&lt;em&gt;li&lt;/em&gt;), qui règlent avec justesse les relations humaines, la sagesse (&lt;em&gt;zhi&lt;/em&gt;) et la fidélité à la parole donnée (&lt;em&gt;xin&lt;/em&gt;). La société repose sur la famille et la piété filiale : chacun doit tenir son rôle dans les relations entre souverain et sujet, père et fils, époux, aînés et cadets, amis. Le prince gouverne par l’exemple, et les mots doivent correspondre aux choses : c’est la « rectification des noms ». Après Confucius, &lt;a href="https://fr.wikipedia.org/wiki/Mencius" title=" Wikipedia"&gt;Mencius&lt;/a&gt; affirme que la nature humaine est bonne, Xunzi qu’elle doit être redressée par l’éducation. Sous les Han, le confucianisme devient la doctrine officielle de l’empire, et les concours de recrutement des fonctionnaires, fondés sur ses classiques, durent jusqu’en 1905. Au XIIe siècle, Zhu Xi le renouvelle par une métaphysique : c’est le néoconfucianisme.&lt;/p&gt; &lt;p&gt;Il s’étend à la Corée, au Japon et au Viêt Nam. Combattu au XXe siècle comme cause du retard chinois, il connaît aujourd’hui un renouveau en Chine.&lt;/p&gt;  &lt;audio controls title="Le Confucianisme et les valeurs asiatiques par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/18755-14.05.2019-ITEMA_22061347-2.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="G17" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="H17" s="9"/>
+      <c r="I17" s="9"/>
+      <c r="J17" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="K17" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="M17" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mouvement</t>
-        </is>
-      </c>
-      <c r="P16" t="inlineStr">
+      <c r="O17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
         <is>
           <t xml:space="preserve">Confucianismes</t>
         </is>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="14" t="n">
+    <row r="18" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="14" t="n">
         <v>-510</v>
       </c>
-      <c r="B17" s="14"/>
-      <c r="C17" s="14" t="s">
+      <c r="B18" s="14"/>
+      <c r="C18" s="14" t="s">
         <v>102</v>
       </c>
-      <c r="D17" s="15" t="s">
+      <c r="D18" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="E17" s="16" t="s">
+      <c r="E18" s="16" t="s">
         <v>104</v>
       </c>
-      <c r="F17" s="14" t="s">
+      <c r="F18" s="14" t="s">
         <v>105</v>
       </c>
-      <c r="G17" s="16" t="s">
+      <c r="G18" s="16" t="s">
         <v>106</v>
       </c>
-      <c r="H17" s="14"/>
-      <c r="I17" s="14"/>
-      <c r="J17" s="2" t="s">
+      <c r="H18" s="14"/>
+      <c r="I18" s="14"/>
+      <c r="J18" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="K17" s="2" t="s">
+      <c r="K18" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="M17" s="2" t="s">
+      <c r="M18" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mouvement</t>
-        </is>
-      </c>
-      <c r="P17" t="inlineStr">
+      <c r="O18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
         <is>
           <t xml:space="preserve">Pensées africaines</t>
         </is>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="1" t="n">
-        <v>-500</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="D18" s="12" t="s">
-        <v>110</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="F18" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="G18" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="J18" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="K18" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="M18" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="O18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mouvement</t>
-        </is>
-      </c>
-      <c r="P18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Les voies dissidentes de l’Inde</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="208.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="n">
         <v>-500</v>
       </c>
@@ -3111,22 +3113,22 @@
         <v>109</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>120</v>
+        <v>22</v>
       </c>
       <c r="M19" s="2" t="s">
         <v>43</v>
@@ -3138,42 +3140,34 @@
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les écoles orthodoxes de l’Inde</t>
-        </is>
-      </c>
-      <c r="Q19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Sâmkhya</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="138.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="9" t="n">
+          <t xml:space="preserve">Les voies dissidentes de l’Inde</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="208.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="1" t="n">
         <v>-500</v>
       </c>
-      <c r="B20" s="9"/>
-      <c r="C20" s="9" t="s">
+      <c r="C20" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="D20" s="10" t="s">
-        <v>121</v>
-      </c>
-      <c r="E20" s="11" t="s">
-        <v>122</v>
-      </c>
-      <c r="F20" s="9" t="s">
-        <v>123</v>
-      </c>
-      <c r="G20" s="11" t="s">
-        <v>124</v>
-      </c>
-      <c r="H20" s="9"/>
-      <c r="I20" s="9"/>
+      <c r="D20" s="12" t="s">
+        <v>115</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>118</v>
+      </c>
       <c r="J20" s="2" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>22</v>
+        <v>120</v>
       </c>
       <c r="M20" s="2" t="s">
         <v>43</v>
@@ -3185,39 +3179,39 @@
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Védas et brahmanisme</t>
+          <t xml:space="preserve">Les écoles orthodoxes de l’Inde</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brahmanisme</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+          <t xml:space="preserve">Sâmkhya</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="138.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="9" t="n">
-        <v>-470</v>
+        <v>-500</v>
       </c>
       <c r="B21" s="9"/>
       <c r="C21" s="9" t="s">
-        <v>126</v>
+        <v>109</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="E21" s="11" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="F21" s="9" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="G21" s="11" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="H21" s="9"/>
       <c r="I21" s="9"/>
       <c r="J21" s="2" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="K21" s="2" t="s">
         <v>22</v>
@@ -3225,94 +3219,94 @@
       <c r="M21" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="N21" s="1" t="s">
+      <c r="O21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Védas et brahmanisme</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Brahmanisme</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="9" t="n">
+        <v>-470</v>
+      </c>
+      <c r="B22" s="9"/>
+      <c r="C22" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="D22" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="E22" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="F22" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="G22" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="H22" s="9"/>
+      <c r="I22" s="9"/>
+      <c r="J22" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="K22" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="M22" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="N22" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="O21" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mouvement</t>
-        </is>
-      </c>
-      <c r="P21" s="1" t="inlineStr">
+      <c r="O22" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P22" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Bouddhismes</t>
         </is>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="14" t="n">
+    <row r="23" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="14" t="n">
         <v>-450</v>
       </c>
-      <c r="B22" s="14"/>
-      <c r="C22" s="14" t="s">
+      <c r="B23" s="14"/>
+      <c r="C23" s="14" t="s">
         <v>132</v>
       </c>
-      <c r="D22" s="15" t="s">
+      <c r="D23" s="15" t="s">
         <v>133</v>
       </c>
-      <c r="E22" s="16" t="s">
+      <c r="E23" s="16" t="s">
         <v>134</v>
       </c>
-      <c r="F22" s="14" t="s">
+      <c r="F23" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="G22" s="16" t="s">
+      <c r="G23" s="16" t="s">
         <v>136</v>
       </c>
-      <c r="H22" s="14"/>
-      <c r="I22" s="14"/>
-      <c r="J22" s="2" t="s">
+      <c r="H23" s="14"/>
+      <c r="I23" s="14"/>
+      <c r="J23" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="K22" s="2" t="s">
+      <c r="K23" s="2" t="s">
         <v>108</v>
-      </c>
-      <c r="M22" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="O22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mouvement</t>
-        </is>
-      </c>
-      <c r="P22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Les Cent Écoles de la Chine antique</t>
-        </is>
-      </c>
-      <c r="Q22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Confucianisme</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="9" t="n">
-        <v>-410</v>
-      </c>
-      <c r="B23" s="9"/>
-      <c r="C23" s="9" t="s">
-        <v>138</v>
-      </c>
-      <c r="D23" s="10" t="s">
-        <v>139</v>
-      </c>
-      <c r="E23" s="11" t="s">
-        <v>140</v>
-      </c>
-      <c r="F23" s="9" t="s">
-        <v>141</v>
-      </c>
-      <c r="G23" s="11" t="s">
-        <v>142</v>
-      </c>
-      <c r="H23" s="9"/>
-      <c r="I23" s="9"/>
-      <c r="J23" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="K23" s="2" t="s">
-        <v>22</v>
       </c>
       <c r="M23" s="2" t="s">
         <v>101</v>
@@ -3324,34 +3318,39 @@
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Japon : shintō et voies nationales</t>
+          <t xml:space="preserve">Les Cent Écoles de la Chine antique</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confucianisme</t>
         </is>
       </c>
     </row>
     <row r="24" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="14" t="n">
-        <v>-400</v>
-      </c>
-      <c r="B24" s="14"/>
-      <c r="C24" s="14" t="s">
-        <v>144</v>
-      </c>
-      <c r="D24" s="15" t="s">
-        <v>145</v>
-      </c>
-      <c r="E24" s="16" t="s">
-        <v>146</v>
-      </c>
-      <c r="F24" s="14" t="s">
-        <v>147</v>
-      </c>
-      <c r="G24" s="16" t="s">
-        <v>148</v>
-      </c>
-      <c r="H24" s="14"/>
-      <c r="I24" s="14"/>
+      <c r="A24" s="9" t="n">
+        <v>-410</v>
+      </c>
+      <c r="B24" s="9"/>
+      <c r="C24" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="D24" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="E24" s="11" t="s">
+        <v>140</v>
+      </c>
+      <c r="F24" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="G24" s="11" t="s">
+        <v>142</v>
+      </c>
+      <c r="H24" s="9"/>
+      <c r="I24" s="9"/>
       <c r="J24" s="2" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="K24" s="2" t="s">
         <v>22</v>
@@ -3366,34 +3365,37 @@
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Taoïsme et syncrétismes</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="1" t="n">
+          <t xml:space="preserve">Japon : shintō et voies nationales</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="14" t="n">
         <v>-400</v>
       </c>
-      <c r="C25" s="1" t="s">
+      <c r="B25" s="14"/>
+      <c r="C25" s="14" t="s">
         <v>144</v>
       </c>
-      <c r="D25" s="12" t="s">
-        <v>150</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="F25" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="G25" s="2" t="s">
-        <v>153</v>
-      </c>
+      <c r="D25" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="E25" s="16" t="s">
+        <v>146</v>
+      </c>
+      <c r="F25" s="14" t="s">
+        <v>147</v>
+      </c>
+      <c r="G25" s="16" t="s">
+        <v>148</v>
+      </c>
+      <c r="H25" s="14"/>
+      <c r="I25" s="14"/>
       <c r="J25" s="2" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="K25" s="2" t="s">
-        <v>155</v>
+        <v>22</v>
       </c>
       <c r="M25" s="2" t="s">
         <v>101</v>
@@ -3405,172 +3407,164 @@
       </c>
       <c r="P25" t="inlineStr">
         <is>
+          <t xml:space="preserve">Taoïsme et syncrétismes</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="94.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="1" t="n">
+        <v>-400</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="D26" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="J26" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="K26" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="M26" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
           <t xml:space="preserve">Les Cent Écoles de la Chine antique</t>
         </is>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="9" t="n">
+    <row r="27" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="9" t="n">
         <v>-350</v>
       </c>
-      <c r="B26" s="9"/>
-      <c r="C26" s="9" t="s">
+      <c r="B27" s="9"/>
+      <c r="C27" s="9" t="s">
         <v>156</v>
       </c>
-      <c r="D26" s="10" t="s">
+      <c r="D27" s="10" t="s">
         <v>157</v>
       </c>
-      <c r="E26" s="18" t="s">
+      <c r="E27" s="18" t="s">
         <v>158</v>
       </c>
-      <c r="F26" s="9" t="s">
+      <c r="F27" s="9" t="s">
         <v>159</v>
       </c>
-      <c r="G26" s="11" t="s">
+      <c r="G27" s="11" t="s">
         <v>160</v>
       </c>
-      <c r="H26" s="9"/>
-      <c r="I26" s="9"/>
-      <c r="J26" s="2" t="s">
+      <c r="H27" s="9"/>
+      <c r="I27" s="9"/>
+      <c r="J27" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="K26" s="2" t="s">
+      <c r="K27" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="M26" s="2" t="s">
+      <c r="M27" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="O26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mouvement</t>
-        </is>
-      </c>
-      <c r="P26" t="inlineStr">
+      <c r="O27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
         <is>
           <t xml:space="preserve">Les écoles orthodoxes de l’Inde</t>
         </is>
       </c>
-      <c r="Q26" t="inlineStr">
+      <c r="Q27" t="inlineStr">
         <is>
           <t xml:space="preserve">Brahmanisme</t>
         </is>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="105" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="1" t="n">
+    <row r="28" customFormat="false" ht="105" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="1" t="n">
         <v>-350</v>
       </c>
-      <c r="C27" s="1" t="s">
+      <c r="C28" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="D27" s="12" t="s">
+      <c r="D28" s="12" t="s">
         <v>162</v>
       </c>
-      <c r="E27" s="2" t="s">
+      <c r="E28" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="F27" s="1" t="s">
+      <c r="F28" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="G27" s="2" t="s">
+      <c r="G28" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="J27" s="2" t="s">
+      <c r="J28" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="K27" s="2" t="s">
+      <c r="K28" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="M27" s="2" t="s">
+      <c r="M28" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="O27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mouvement</t>
-        </is>
-      </c>
-      <c r="P27" t="inlineStr">
+      <c r="O28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
         <is>
           <t xml:space="preserve">Les Cent Écoles de la Chine antique</t>
         </is>
       </c>
-      <c r="Q27" t="inlineStr">
+      <c r="Q28" t="inlineStr">
         <is>
           <t xml:space="preserve">Confucianisme</t>
         </is>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="1" t="n">
+    <row r="29" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="1" t="n">
         <v>-250</v>
       </c>
-      <c r="C28" s="1" t="s">
+      <c r="C29" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="D28" s="12" t="s">
+      <c r="D29" s="12" t="s">
         <v>168</v>
       </c>
-      <c r="E28" s="2" t="s">
+      <c r="E29" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="F28" s="1" t="s">
+      <c r="F29" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="G28" s="2" t="s">
+      <c r="G29" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="J28" s="2" t="s">
+      <c r="J29" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="K28" s="2" t="s">
+      <c r="K29" s="2" t="s">
         <v>22</v>
-      </c>
-      <c r="M28" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="O28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mouvement</t>
-        </is>
-      </c>
-      <c r="P28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bouddhismes</t>
-        </is>
-      </c>
-      <c r="Q28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bouddhisme</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="14" t="n">
-        <v>-150</v>
-      </c>
-      <c r="B29" s="14"/>
-      <c r="C29" s="14" t="s">
-        <v>173</v>
-      </c>
-      <c r="D29" s="15" t="s">
-        <v>174</v>
-      </c>
-      <c r="E29" s="19" t="s">
-        <v>175</v>
-      </c>
-      <c r="F29" s="14" t="s">
-        <v>176</v>
-      </c>
-      <c r="G29" s="16" t="s">
-        <v>177</v>
-      </c>
-      <c r="H29" s="14"/>
-      <c r="I29" s="14"/>
-      <c r="J29" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="K29" s="2" t="s">
-        <v>155</v>
       </c>
       <c r="M29" s="2" t="s">
         <v>43</v>
@@ -3582,42 +3576,42 @@
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les écoles orthodoxes de l’Inde</t>
+          <t xml:space="preserve">Bouddhismes</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brahmanisme</t>
+          <t xml:space="preserve">Bouddhisme</t>
         </is>
       </c>
     </row>
     <row r="30" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="9" t="n">
-        <v>-100</v>
-      </c>
-      <c r="B30" s="9"/>
-      <c r="C30" s="9" t="s">
-        <v>179</v>
-      </c>
-      <c r="D30" s="10" t="s">
-        <v>180</v>
-      </c>
-      <c r="E30" s="18" t="s">
-        <v>181</v>
-      </c>
-      <c r="F30" s="9" t="s">
-        <v>182</v>
-      </c>
-      <c r="G30" s="11" t="s">
-        <v>183</v>
-      </c>
-      <c r="H30" s="9"/>
-      <c r="I30" s="9"/>
+      <c r="A30" s="14" t="n">
+        <v>-150</v>
+      </c>
+      <c r="B30" s="14"/>
+      <c r="C30" s="14" t="s">
+        <v>173</v>
+      </c>
+      <c r="D30" s="15" t="s">
+        <v>174</v>
+      </c>
+      <c r="E30" s="19" t="s">
+        <v>175</v>
+      </c>
+      <c r="F30" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="G30" s="16" t="s">
+        <v>177</v>
+      </c>
+      <c r="H30" s="14"/>
+      <c r="I30" s="14"/>
       <c r="J30" s="2" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="K30" s="2" t="s">
-        <v>88</v>
+        <v>155</v>
       </c>
       <c r="M30" s="2" t="s">
         <v>43</v>
@@ -3638,176 +3632,179 @@
         </is>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="C31" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="D31" s="12" t="s">
-        <v>185</v>
-      </c>
-      <c r="E31" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="F31" s="1" t="s">
-        <v>187</v>
-      </c>
-      <c r="G31" s="2" t="s">
-        <v>188</v>
-      </c>
+    <row r="31" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="9" t="n">
+        <v>-100</v>
+      </c>
+      <c r="B31" s="9"/>
+      <c r="C31" s="9" t="s">
+        <v>179</v>
+      </c>
+      <c r="D31" s="10" t="s">
+        <v>180</v>
+      </c>
+      <c r="E31" s="18" t="s">
+        <v>181</v>
+      </c>
+      <c r="F31" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="G31" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="H31" s="9"/>
+      <c r="I31" s="9"/>
       <c r="J31" s="2" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="K31" s="2" t="s">
-        <v>22</v>
+        <v>88</v>
       </c>
       <c r="M31" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="N31" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="O31" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mouvement</t>
-        </is>
-      </c>
-      <c r="P31" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bouddhismes</t>
-        </is>
-      </c>
-      <c r="Q31" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bouddhisme</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="14" t="n">
-        <v>250</v>
-      </c>
-      <c r="B32" s="14"/>
-      <c r="C32" s="14" t="s">
-        <v>190</v>
-      </c>
-      <c r="D32" s="15" t="s">
-        <v>191</v>
-      </c>
-      <c r="E32" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Mimamsa"  title=" Wikipedia"&gt;La Mimamsa&lt;/a&gt;, « réflexion » ou « exégèse », est l’une des six écoles orthodoxes de la philosophie indienne. Elle est fondée par Jaimini, à qui l’on attribue les &lt;em&gt;Mīmāṃsā Sūtra&lt;/em&gt;, composés entre le IIIe et le Ier siècle avant notre ère. Son objet est l’interprétation des &lt;a href="https://fr.wikipedia.org/wiki/Veda" title=" Wikipedia"&gt;Védas&lt;/a&gt;, et surtout de leur partie rituelle : comment comprendre les injonctions des textes sacrés pour accomplir correctement les sacrifices et réaliser ainsi le &lt;em&gt;dharma&lt;/em&gt;, l’ordre juste du monde.&lt;/p&gt; &lt;p&gt;Pour la Mimamsa, les Védas sont éternels, sans auteur, ni humain ni divin, et donc infaillibles : ils sont la seule source de connaissance du devoir religieux. Pour les lire, elle développe une science très rigoureuse du langage et de l’interprétation, qui influencera le droit indien. Les injonctions (&lt;em&gt;vidhi&lt;/em&gt;) prescrivent des actes, et chaque acte rituel produit une force invisible, l’&lt;em&gt;apūrva&lt;/em&gt;, qui en porte les fruits dans cette vie ou dans une autre. La Mimamsa ancienne ne fait pas appel à un dieu créateur : l’efficacité des rites suffit à expliquer l’ordre du monde. Elle défend l’existence d’un Soi éternel et la réalité du monde extérieur. Au VIIe siècle, deux grands commentateurs, &lt;a href="https://fr.wikipedia.org/wiki/Kumarila_Bhatta" title=" Wikipedia"&gt;Kumarila Bhatta&lt;/a&gt; et Prabhakara, fondent deux écoles rivales, qui débattent avec le bouddhisme et le Nyāya de la valeur de la connaissance par le témoignage (&lt;em&gt;śabda&lt;/em&gt;).&lt;/p&gt; &lt;p&gt;On l’appelle aussi « première Mimamsa », par opposition au Vedānta, ou « Mimamsa ultérieure », qui s’attache à la partie spéculative des Védas, les Upanishads. Ses principes d’interprétation guident encore les pratiques des brahmanes.&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="F32" s="14" t="s">
-        <v>193</v>
-      </c>
-      <c r="G32" s="16" t="s">
-        <v>194</v>
-      </c>
-      <c r="H32" s="14"/>
-      <c r="I32" s="14"/>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Les écoles orthodoxes de l’Inde</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Brahmanisme</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="C32" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="D32" s="12" t="s">
+        <v>185</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>188</v>
+      </c>
       <c r="J32" s="2" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="K32" s="2" t="s">
-        <v>196</v>
+        <v>22</v>
       </c>
       <c r="M32" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="O32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mouvement</t>
-        </is>
-      </c>
-      <c r="P32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Les écoles orthodoxes de l’Inde</t>
-        </is>
-      </c>
-      <c r="Q32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Védisme</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="108.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="N32" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="O32" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P32" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bouddhismes</t>
+        </is>
+      </c>
+      <c r="Q32" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bouddhisme</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="14" t="n">
-        <v>450</v>
+        <v>250</v>
       </c>
       <c r="B33" s="14"/>
-      <c r="C33" s="14" t="n">
-        <v>450</v>
+      <c r="C33" s="14" t="s">
+        <v>190</v>
       </c>
       <c r="D33" s="15" t="s">
-        <v>197</v>
-      </c>
-      <c r="E33" s="20" t="s">
-        <v>198</v>
+        <v>191</v>
+      </c>
+      <c r="E33" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Mimamsa"  title=" Wikipedia"&gt;La Mimamsa&lt;/a&gt;, « réflexion » ou « exégèse », est l’une des six écoles orthodoxes de la philosophie indienne. Elle est fondée par Jaimini, à qui l’on attribue les &lt;em&gt;Mīmāṃsā Sūtra&lt;/em&gt;, composés entre le IIIe et le Ier siècle avant notre ère. Son objet est l’interprétation des &lt;a href="https://fr.wikipedia.org/wiki/Veda" title=" Wikipedia"&gt;Védas&lt;/a&gt;, et surtout de leur partie rituelle : comment comprendre les injonctions des textes sacrés pour accomplir correctement les sacrifices et réaliser ainsi le &lt;em&gt;dharma&lt;/em&gt;, l’ordre juste du monde.&lt;/p&gt; &lt;p&gt;Pour la Mimamsa, les Védas sont éternels, sans auteur, ni humain ni divin, et donc infaillibles : ils sont la seule source de connaissance du devoir religieux. Pour les lire, elle développe une science très rigoureuse du langage et de l’interprétation, qui influencera le droit indien. Les injonctions (&lt;em&gt;vidhi&lt;/em&gt;) prescrivent des actes, et chaque acte rituel produit une force invisible, l’&lt;em&gt;apūrva&lt;/em&gt;, qui en porte les fruits dans cette vie ou dans une autre. La Mimamsa ancienne ne fait pas appel à un dieu créateur : l’efficacité des rites suffit à expliquer l’ordre du monde. Elle défend l’existence d’un Soi éternel et la réalité du monde extérieur. Au VIIe siècle, deux grands commentateurs, &lt;a href="https://fr.wikipedia.org/wiki/Kumarila_Bhatta" title=" Wikipedia"&gt;Kumarila Bhatta&lt;/a&gt; et Prabhakara, fondent deux écoles rivales, qui débattent avec le bouddhisme et le Nyāya de la valeur de la connaissance par le témoignage (&lt;em&gt;śabda&lt;/em&gt;).&lt;/p&gt; &lt;p&gt;On l’appelle aussi « première Mimamsa », par opposition au Vedānta, ou « Mimamsa ultérieure », qui s’attache à la partie spéculative des Védas, les Upanishads. Ses principes d’interprétation guident encore les pratiques des brahmanes.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F33" s="14" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="G33" s="16" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="H33" s="14"/>
       <c r="I33" s="14"/>
       <c r="J33" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="K33" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="M33" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Les écoles orthodoxes de l’Inde</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Védisme</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="108.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="14" t="n">
+        <v>450</v>
+      </c>
+      <c r="B34" s="14"/>
+      <c r="C34" s="14" t="n">
+        <v>450</v>
+      </c>
+      <c r="D34" s="15" t="s">
+        <v>197</v>
+      </c>
+      <c r="E34" s="20" t="s">
+        <v>198</v>
+      </c>
+      <c r="F34" s="14" t="s">
+        <v>199</v>
+      </c>
+      <c r="G34" s="16" t="s">
+        <v>200</v>
+      </c>
+      <c r="H34" s="14"/>
+      <c r="I34" s="14"/>
+      <c r="J34" s="2" t="s">
         <v>201</v>
-      </c>
-      <c r="K33" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="M33" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="O33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mouvement</t>
-        </is>
-      </c>
-      <c r="P33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Proche-Orient ancien et Iran</t>
-        </is>
-      </c>
-      <c r="Q33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Zoroastrisme</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="1" t="n">
-        <v>500</v>
-      </c>
-      <c r="C34" s="1" t="n">
-        <v>500</v>
-      </c>
-      <c r="D34" s="12" t="s">
-        <v>202</v>
-      </c>
-      <c r="E34" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="F34" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="G34" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="J34" s="2" t="s">
-        <v>206</v>
       </c>
       <c r="K34" s="2" t="s">
         <v>22</v>
       </c>
       <c r="M34" s="2" t="s">
-        <v>101</v>
+        <v>23</v>
       </c>
       <c r="O34" t="inlineStr">
         <is>
@@ -3816,98 +3813,103 @@
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bouddhismes</t>
+          <t xml:space="preserve">Proche-Orient ancien et Iran</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bouddhisme Mahayana;Taoïsme</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="104.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+          <t xml:space="preserve">Zoroastrisme</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="n">
-        <v>700</v>
+        <v>500</v>
       </c>
       <c r="C35" s="1" t="n">
-        <v>700</v>
+        <v>500</v>
       </c>
       <c r="D35" s="12" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="J35" s="2" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="K35" s="2" t="s">
         <v>22</v>
       </c>
       <c r="M35" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="N35" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="O35" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mouvement</t>
-        </is>
-      </c>
-      <c r="P35" s="1" t="inlineStr">
+      <c r="O35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
         <is>
           <t xml:space="preserve">Bouddhismes</t>
         </is>
       </c>
-      <c r="Q35" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bouddhisme Mahayana</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="353.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bouddhisme Mahayana;Taoïsme</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="104.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="n">
-        <v>720</v>
+        <v>700</v>
       </c>
       <c r="C36" s="1" t="n">
-        <v>720</v>
+        <v>700</v>
       </c>
       <c r="D36" s="12" t="s">
-        <v>212</v>
-      </c>
-      <c r="E36" s="21" t="s">
-        <v>213</v>
+        <v>207</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>208</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>215</v>
-      </c>
-      <c r="J36" s="21" t="s">
-        <v>216</v>
+        <v>210</v>
+      </c>
+      <c r="J36" s="2" t="s">
+        <v>211</v>
       </c>
       <c r="K36" s="2" t="s">
         <v>22</v>
       </c>
       <c r="M36" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="O36" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mouvement</t>
-        </is>
-      </c>
-      <c r="P36" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Théologie de l’islam (kalâm)</t>
+        <v>43</v>
+      </c>
+      <c r="N36" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="O36" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouvement</t>
+        </is>
+      </c>
+      <c r="P36" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bouddhismes</t>
+        </is>
+      </c>
+      <c r="Q36" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bouddhisme Mahayana</t>
         </is>
       </c>
     </row>
@@ -7228,18 +7230,18 @@
     <mergeCell ref="A2:I2"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="E10" r:id="rId1" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Religions_m%C3%A9soam%C3%A9ricaines&quot;  title=&quot; Wikipedia&quot;&gt;Le Mysticisme mésoaméricain&lt;/a&gt; désigne les traditions philosophiques et spirituelles des civilisations précolombiennes d'Amérique centrale, en particulier les Aztèques, les Mayas et les Toltèques. Ces pensées forment un univers conceptuel original, structuré autour de la relation entre l'homme, le cosmos et les forces divines.&lt;/p&gt;&lt;p&gt;Au cœur de ces traditions se trouve la notion de &lt;em&gt;teotl&lt;/em&gt; (divinité, énergie sacrée) chez les Aztèques, ou de &lt;em&gt;k'ul&lt;/em&gt; (force vitale sacrée) chez les Mayas. La cosmologie mésoaméricaine conçoit l'univers comme un système de cycles temporels, où les dieux et les hommes sont liés par des obligations réciproques. Le sacrifice rituel, loin d'être une simple pratique violente, est pensé comme une nécessité cosmique pour maintenir l'équilibre du monde.&lt;/p&gt;&lt;p&gt;Des figures comme Quetzalcóatl (le Serpent à plumes) incarnent une sagesse éthique et philosophique : tempérance, connaissance, opposition au sacrifice humain selon certaines traditions. Les philosophes aztèques, les &lt;em&gt;tlamatinime&lt;/em&gt;, s'interrogeaient sur la nature du vrai, du beau, du bien, et sur la condition humaine — une tradition philosophique autonome redécouverte par des chercheurs comme Miguel León-Portilla.&lt;/p&gt;"/>
-    <hyperlink ref="E12" r:id="rId2" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/H%C3%A9sychasme&quot; title=&quot; Wikipedia&quot;&gt;L'Hésychasme&lt;/a&gt; est une tradition mystique et contemplative du christianisme oriental, dont le nom vient du grec &lt;em&gt;hésychia&lt;/em&gt; (silence, tranquillité). Il désigne une pratique spirituelle visant à atteindre l'union avec Dieu par la prière continue, le silence intérieur et la maîtrise du souffle.&lt;/p&gt;&lt;p&gt;Ses origines remontent aux Pères du désert des IVe-Ve siècles, mais c'est au XIVe siècle que l'hésychasme devient un courant théologique et philosophique structuré, notamment grâce à Grégoire Palamas, archevêque de Thessalonique, qui en formule la doctrine dans ses &lt;em&gt;Triades&lt;/em&gt;. Palamas distingue l'essence divine (inaccessible) des énergies divines (accessibles à l'expérience mystique), permettant de fonder théologiquement la possibilité d'une véritable union de l'homme avec Dieu.&lt;/p&gt;&lt;p&gt;Cette distinction essence-énergies est l'une des contributions philosophiques les plus originales de la pensée byzantine. L'hésychasme a profondément marqué la spiritualité orthodoxe russe, grecque et serbe, et continue d'irriguer la théologie et la philosophie orthodoxes contemporaines.&lt;/p&gt;"/>
-    <hyperlink ref="E14" r:id="rId3" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Ch%C3%A2rv%C3%A2ka&quot;  title=&quot;Wikipedia&quot;&gt;Le Lokayata&lt;/a&gt;, également connu sous le nom de Carvaka, est la seule école philosophique de l'Inde ancienne à avoir défendu un matérialisme radical et un athéisme déclaré. Fondée vers le VIe siècle avant notre ère, elle rejette tout ce qui ne peut être appréhendé par les sens : pas d'âme immortelle, pas d'au-delà, pas de loi karmique.&lt;/p&gt;&lt;p&gt;Sa devise pourrait se résumer ainsi : ce que l'on voit existe ; ce que l'on ne peut percevoir n'est qu'invention. Les Carvakas refusent les Védas et leur autorité, les rituels brahmaniques, et toute forme de spéculation métaphysique. L'univers est composé des quatre éléments — terre, eau, feu et air — sans qu'intervienne aucune divinité créatrice.&lt;/p&gt;&lt;p&gt;En matière d'éthique, la philosophie Carvaka est franchement hédoniste : le plaisir est le seul bien réel, la souffrance le seul mal. Mieux vaut jouir de la vie maintenant plutôt qu'espérer une récompense illusoire après la mort. Ce réalisme sans concession en fait une voix singulière, souvent persécutée, de la pensée indienne classique.&lt;/p&gt;&lt;p&gt;Bien que ses textes originaux aient presque tous disparu — connus surtout par les réfutations de ses adversaires — son influence demeure dans les courants matérialistes et rationalistes qui traversent la philosophie indienne jusqu'à aujourd'hui.&lt;/p&gt;"/>
-    <hyperlink ref="E19" r:id="rId4" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Yoga_s%C5%ABtra&quot; title=&quot; Wikipedia&quot;&gt; Le Yoga&lt;/a&gt; en tant qu’école philosophique (darshana) est distinct de la pratique physique popularisée en Occident. Systématisé par Patanjali dans les Yoga Sutra (entre 200 av. J.-C. et 500 apr. J.-C.), il partage la métaphysique dualiste du Samkhya — Purusha (conscience) et Prakriti (matière) — mais y ajoute une méthode pratique précise pour la libération.&lt;/p&gt;&lt;p&gt;Les huit membres (ashtanga) du Yoga structurent ce chemin : discipline éthique (yama, niyama), posture (asana), maîtrise du souffle (pranayama), retrait des sens (pratyahara), concentration (dharana), méditation (dhyana) et absorption (samadhi). Chaque étape prépare la suivante dans une progression méthodique vers l’arrêt des fluctuations du mental (chitta vritti nirodha).&lt;/p&gt;&lt;p&gt;Contrairement au Samkhya, purement théorique, le Yoga de Patanjali introduit îshvara (un principe divin, seigneur particulier parmi les âmes) comme objet de concentration facultatif — une nuance théiste absente du Samkhya classique. Cette différence a nourri des siècles de commentaires et de débats entre les deux écoles sœurs.&lt;/p&gt;&lt;p&gt;Aujourd’hui mondialement diffusée, la dimension physique du yoga occulte souvent sa profondeur philosophique originelle : une discipline rigoureuse de la conscience, visant non le bien-être mais la discrimination (viveka) entre le Soi éternel et les fluctuations passagères du mental.&lt;/p&gt;"/>
-    <hyperlink ref="E21" r:id="rId5" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Bouddhisme&quot;  title=&quot; Wikipedia&quot;&gt; Le Bouddhisme&lt;/a&gt; est une tradition philosophique qui s'est développée à partir des enseignements du Bouddha, un prince indien du 5ème siècle avant JC qui a atteint l'éveil spirituel en méditant sous un arbre, maintenant connu sous le nom de l'Arbre de la Bodhi. &lt;/p&gt; &lt;p&gt;La philosophie bouddhiste repose sur le principe fondamental de la cessation de la souffrance, connu sous le nom de Nirvana, et cherche à atteindre cet état par une compréhension profonde de la nature de la réalité. &lt;/p&gt;    &lt;p&gt; Le Bouddhisme enseigne que la souffrance est causée par le désir et l'attachement aux choses matérielles et éphémères, et que la libération de la souffrance peut être atteinte par la compréhension de la nature de l'existence et de la réalité. Pour atteindre cet état de libération, le bouddhisme propose la pratique de la méditation et le développement de la sagesse, de la compassion et de la bienveillance envers tous les êtres vivants. &lt;/p&gt; &lt;p&gt; Il est également connu pour ses enseignements sur les Quatre Nobles Vérités et le Noble Chemin Octuple, qui sont considérés comme les fondements de la pratique bouddhiste. Les Quatre Nobles Vérités décrivent la nature de la souffrance, ses causes, sa cessation et le chemin menant à la cessation de la souffrance. Le Noble Chemin Octuple est une série d'étapes pratiques pour développer la sagesse, la moralité et la concentration, afin d'atteindre l'éveil spirituel. &lt;/p&gt; &lt;p&gt; En outre, la philosophie bouddhiste met l'accent sur l'interdépendance de tous les phénomènes, la nature impermanente de l'existence et la non-existence d'un soi permanent et autonome.&lt;/p&gt; &lt;audio controls title=&quot;Le Taoïsme par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/18755-11.03.2019-ITEMA_22005213-1.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt; &lt;p&gt; &lt;/p&gt;"/>
-    <hyperlink ref="E25" r:id="rId6" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/École_des_Noms&quot;  title=&quot;Wikipedia&quot;&gt;L'École des Noms&lt;/a&gt; (ming jia, 名家) est une école de philosophie chinoise qui s'est développée pendant la période des Royaumes combattants. Sa préoccupation centrale : la relation entre les mots et les choses, entre les noms et la réalité qu'ils désignent.&lt;/p&gt;&lt;p&gt;Ses représentants les plus célèbres, Gongsun Long et Hui Shi, sont connus pour leurs paradoxes vertigineux. Gongsun Long affirmait que &quot;le cheval blanc n'est pas un cheval&quot; — non par provocation, mais pour distinguer le concept général (cheval) du particulier concret (ce cheval blanc). Hui Shi proclamait que &quot;le ciel et la terre sont d'une même hauteur&quot;, explorant les limites relatives de toute catégorisation.&lt;/p&gt;&lt;p&gt;Ces réflexions sur le langage anticipent certaines problématiques de la logique et de la philosophie analytique moderne. Comment les mots nous permettent-ils — ou nous empêchent-ils — de saisir la réalité ? Toute classification n'implique-t-elle pas une distorsion du monde ?&lt;/p&gt;&lt;p&gt;Peu influente politiquement, l'École des Noms fut souvent moquée par ses contemporains confu céens et taoïstes. Mais elle constitue une contribution unique à la logique asiatique et à la philosophie du langage dans la pensée mondiale.&lt;/p&gt;"/>
-    <hyperlink ref="E26" r:id="rId7" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/S%C3%A2mkhya&quot;  title=&quot; Wikipedia&quot;&gt;Le Sâmkhya&lt;/a&gt; est l'une des plus anciennes écoles philosophiques de l'Inde, considérée comme un darshana orthodoxe de l'hindouisme. Il propose une analyse rationnelle de la réalité pour libérer l'individu du cycle des renaissances et de la souffrance. Ce système dualiste distingue deux réalités ultimes : Purusha, la conscience pure et passive (esprit, principe masculin), et Prakriti, la matière primordiale active (énergie universelle, principe féminin). Prakriti évolue sous l'influence des trois guṇas (sattva : harmonie ; rajas : activité ; tamas : inertie), générant le monde manifesté à travers 23 tattvas (principes), comme buddhi (intelligence), ahaṃkāra (ego) et les sens. &lt;/p&gt; &lt;p&gt; Il explique la création comme une transformation de Prakriti, sans recours à un dieu créateur : de l'état non manifesté (avyakta) naît le manifesté (vyakta), incluant le corps subtil qui transmigre. L'ignorance (avidyā) cause l'identification erronée du Purusha à la matière, source de souffrance (duḥkha). &lt;/p&gt; &lt;p&gt; Fondement théorique du Yoga de Patañjali, le Sâmkhya met l'accent sur la discrimination (viveka) entre Purusha et Prakriti pour atteindre la libération (kaivalya). Il influence largement la philosophie indienne, des Puranas au Vedānta. &lt;/p&gt;"/>
-    <hyperlink ref="E28" r:id="rId8" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Therav%C4%81da&quot; title=&quot;Wikipedia&quot;&gt;Le Bouddhisme Theravada&lt;/a&gt; (« École des Anciens ») est la plus ancienne forme du bouddhisme conservée jusqu'à nos jours. Héritière directe des enseignements du Bouddha historique, elle s'enracina progressivement en Asie du Sud-Est : Sri Lanka, Thaïlande, Myanmar, Cambodge, Laos.&lt;/p&gt;&lt;p&gt;Au cœur du Theravada se trouve le Pali Canon (Tipitaka), le corpus scripturaire le plus ancien du bouddhisme. Sa philosophie insiste sur la voie individuelle vers l'éveil : chaque être doit parcourir lui-même le Noble Sentier Octuple — juste compréhension, juste intention, juste parole, juste action, juste mode de vie, juste effort, juste attention, juste concentration.&lt;/p&gt;&lt;p&gt;L'idéal du Theravada est l'Arhat : le sage qui, par sa propre pratique, a éteint les &quot;feux&quot; de l'attachement, de la haine et de l'illusion, et atteint le Nirvana. Cette voie solitaire et rigoureuse contraste avec l'idéal du bodhisattva du Mahayana, qui renonce à son propre éveil pour sauver tous les êtres.&lt;/p&gt;&lt;p&gt;La méditation de pleine conscience (sati), aujourd'hui mondialement répandue, trouve ses racines dans les pratiques contemplatives du Theravada, notamment la méditation vipassana qui vise à observer directement l'impermanence, la souffrance et l'absence de soi.&lt;/p&gt;"/>
-    <hyperlink ref="E30" r:id="rId9" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Vaisheshika&quot;  title=&quot; Wikipedia&quot;&gt;Le Vaisheshika&lt;/a&gt;  est une école philosophique orthodoxe hindoue, fondée par le sage Kaṇāda, qui se distingue par son atomisme et son réalisme ontologique. Exposée dans les Vaiśeṣika Sūtra (non antérieurs à l'ère chrétienne), elle vise la libération (mokṣa) par la connaissance des catégories fondamentales de la réalité. Le système repose sur six ou sept padārthas (catégories) : dravya (substance), guṇa (qualité), karma (action/mouvement), sāmānya (universalité), viśeṣa (particularité) et samavāya (inhérence). Parmi les neuf substances, quatre sont atomiques (terre, eau, feu, air) : les paramāṇu (atomes éternels, indivisibles) s'assemblent en dyades puis en objets composites non éternels. &lt;/p&gt; &lt;p&gt; Sans dieu créateur direct, l'univers émerge de combinaisons atomiques influencées par une cause efficiente (adrisṭa, karma résiduel). Ākāśa (espace), kāla (temps), dik (direction) et cit (âme) complètent les substances ; les atomes sphériques se lient par forces intrinsèques, formant un monde discontinu mais perceptible. &lt;/p&gt; &lt;p&gt; Souvent fusionné avec le Nyâya (logique), il postule un Īśvara ordonnateur. La délivrance est un état pur de l'âme (sans qualités, conscience ou douleur), libérée des agrégats par la gnose discriminante. &lt;/p&gt;"/>
-    <hyperlink ref="E31" r:id="rId10" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Bouddhisme_mah%C4%81y%C4%81na&quot; title=&quot;Wikipedia&quot;&gt;Le Bouddhisme Mahayana&lt;/a&gt; (« Grand Véhicule ») est apparu en Inde au tournant de l'ère chrétienne, s'étendant progressivement vers la Chine, le Japon, la Corée et le Vietnam. Par rapport au Theravada, il représente une transformation profonde de la vision bouddhiste : l'éveil n'est plus un idéal solitaire mais une aspiration collective.&lt;/p&gt;&lt;p&gt;L'idéal central du Mahayana est le bodhisattva : l'être qui, sur le point d'atteindre le Nirvana, choisit de demeurer dans le cycle des renaissances (samsara) pour guider et libérer tous les êtres sensibles. Cette compassion universelle (karuna) devient le moteur de la voie spirituelle, indissociable de la sagesse (prajna).&lt;/p&gt;&lt;p&gt;Le Mahayana introduit également la notion révolutionnaire de sunyata (vacuité) : toutes choses sont dénues d'existence propre et intrinsèque — elles n'existent que de façon interdependante. Nagarjuna, au IIe siècle, en développa la philosophie dans ses Stances du Milieu, fondant l'école Madhyamaka qui influencça toute la pensée bouddhiste ultérieure.&lt;/p&gt;&lt;p&gt;C'est sur le sol du Mahayana que fleuriront le bouddhisme Zen, le bouddhisme tibétain Vajrayana, et l'École de la Terre Pure. Avec ses sutras nouveaux (Lotus, Vimalakirti, Prajnaparamita), le Mahayana offre une vision du monde d'une richesse philosophique et spirituelle sans équivalent.&lt;/p&gt;"/>
-    <hyperlink ref="E33" r:id="rId11" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Mazdakisme&quot; title=&quot;Wikipedia&quot;&gt;Le Mazdakisme&lt;/a&gt; est un mouvement religieux et social apparu en Perse sous l’Empire sassanide. Fondé par le réformateur Mazdak, ce courant tire ses origines à la fois du mazdéisme et du manichéisme, en proposant une relecture dualiste du monde axée sur la lumière et les ténèbres. &lt;/p&gt; &lt;p&gt; Contrairement aux structures sociales hiérarchisées de l’époque, le mazdakisme prônait une égalité radicale entre les individus. Mazdak soutenait que les causes des conflits humains résidaient dans la soif de richesses et de pouvoir, ce qui l'a conduit à prôner la mise en commun des biens matériels et, selon certaines sources, des femmes. &lt;/p&gt; &lt;p&gt; Cette doctrine a été perçue comme une menace par l’aristocratie et le clergé zoroastrien traditionnel, qui y voyaient une hérésie dangereuse pour l'ordre établi. Après avoir initialement bénéficié de l'intérêt de l'empereur Kavadh Ier, le mouvement fut sévèrement réprimé lors de grandes purges organisées entre 524 et 529. &lt;/p&gt; &lt;p&gt; Bien que le mazdakisme ait été marginalisé après ces persécutions, il a laissé une trace durable dans la pensée iranienne. Parfois qualifié, de manière anachronique, de mouvement proto-socialiste, son idéal de justice sociale a influencé certains courants contestataires qui se sont manifestés en Iran jusqu'au XIVe siècle environ. &lt;/p&gt; &#10;"/>
-    <hyperlink ref="E35" r:id="rId12" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Bouddhisme_vajrayana&quot;  title=&quot;Wikipedia&quot;&gt;Le Vajrayana&lt;/a&gt; (« Véhicule de Diamant ») est la troisième grande forme du bouddhisme, développée en Inde entre le VIIe et le Xe siècle, puis transmise au Tibet, en Mongolie et dans l'Himalaya. Il représente la voie tantrique du bouddhisme, utilisant des pratiques ésotériques pour accélérer le chemin vers l'éveil.&lt;/p&gt;&lt;p&gt;Là où le Theravada vise l'éveil en de nombreuses vies et le Mahayana en d'innombrables éons, le Vajrayana affirme qu'il est possible d'atteindre l'éveil en une seule vie — voire en un seul instant. Pour cela, il mobilise un arsenal de techniques : mantras, mandalas, mudras, visualisations de divinités, pratiques yogiques subtiles sur les énergies intérieures du corps.&lt;/p&gt;&lt;p&gt;Le Bouddhisme tibétain, la forme la plus répandue du Vajrayana, s'est développé dès le VIIe siècle sous le règne du roi Songtsen Gampo. Il intègre des éléments de la religion Bön préexistante et du Mahayana indien. Ses figures tutlaires — Padmasambhava, Milarepa, Tsongkhapa — sont au cœur d'une tradition d'une richesse philosophique et rituelle incomparable.&lt;/p&gt;&lt;p&gt;La notion de &quot;nature de bouddha&quot; (tathagatagarbha) — l'idée que chaque être possède en lui la graine de l'éveil — est centrale dans le Vajrayana. La pratique vise à reconnaître directement cette nature lumineuse originelle, au-delà des voiles de l'ignorance et de l'égo.&lt;/p&gt;"/>
+    <hyperlink ref="E11" r:id="rId1" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Religions_m%C3%A9soam%C3%A9ricaines&quot;  title=&quot; Wikipedia&quot;&gt;Le Mysticisme mésoaméricain&lt;/a&gt; désigne les traditions philosophiques et spirituelles des civilisations précolombiennes d'Amérique centrale, en particulier les Aztèques, les Mayas et les Toltèques. Ces pensées forment un univers conceptuel original, structuré autour de la relation entre l'homme, le cosmos et les forces divines.&lt;/p&gt;&lt;p&gt;Au cœur de ces traditions se trouve la notion de &lt;em&gt;teotl&lt;/em&gt; (divinité, énergie sacrée) chez les Aztèques, ou de &lt;em&gt;k'ul&lt;/em&gt; (force vitale sacrée) chez les Mayas. La cosmologie mésoaméricaine conçoit l'univers comme un système de cycles temporels, où les dieux et les hommes sont liés par des obligations réciproques. Le sacrifice rituel, loin d'être une simple pratique violente, est pensé comme une nécessité cosmique pour maintenir l'équilibre du monde.&lt;/p&gt;&lt;p&gt;Des figures comme Quetzalcóatl (le Serpent à plumes) incarnent une sagesse éthique et philosophique : tempérance, connaissance, opposition au sacrifice humain selon certaines traditions. Les philosophes aztèques, les &lt;em&gt;tlamatinime&lt;/em&gt;, s'interrogeaient sur la nature du vrai, du beau, du bien, et sur la condition humaine — une tradition philosophique autonome redécouverte par des chercheurs comme Miguel León-Portilla.&lt;/p&gt;"/>
+    <hyperlink ref="E13" r:id="rId2" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/H%C3%A9sychasme&quot; title=&quot; Wikipedia&quot;&gt;L'Hésychasme&lt;/a&gt; est une tradition mystique et contemplative du christianisme oriental, dont le nom vient du grec &lt;em&gt;hésychia&lt;/em&gt; (silence, tranquillité). Il désigne une pratique spirituelle visant à atteindre l'union avec Dieu par la prière continue, le silence intérieur et la maîtrise du souffle.&lt;/p&gt;&lt;p&gt;Ses origines remontent aux Pères du désert des IVe-Ve siècles, mais c'est au XIVe siècle que l'hésychasme devient un courant théologique et philosophique structuré, notamment grâce à Grégoire Palamas, archevêque de Thessalonique, qui en formule la doctrine dans ses &lt;em&gt;Triades&lt;/em&gt;. Palamas distingue l'essence divine (inaccessible) des énergies divines (accessibles à l'expérience mystique), permettant de fonder théologiquement la possibilité d'une véritable union de l'homme avec Dieu.&lt;/p&gt;&lt;p&gt;Cette distinction essence-énergies est l'une des contributions philosophiques les plus originales de la pensée byzantine. L'hésychasme a profondément marqué la spiritualité orthodoxe russe, grecque et serbe, et continue d'irriguer la théologie et la philosophie orthodoxes contemporaines.&lt;/p&gt;"/>
+    <hyperlink ref="E15" r:id="rId3" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Ch%C3%A2rv%C3%A2ka&quot;  title=&quot;Wikipedia&quot;&gt;Le Lokayata&lt;/a&gt;, également connu sous le nom de Carvaka, est la seule école philosophique de l'Inde ancienne à avoir défendu un matérialisme radical et un athéisme déclaré. Fondée vers le VIe siècle avant notre ère, elle rejette tout ce qui ne peut être appréhendé par les sens : pas d'âme immortelle, pas d'au-delà, pas de loi karmique.&lt;/p&gt;&lt;p&gt;Sa devise pourrait se résumer ainsi : ce que l'on voit existe ; ce que l'on ne peut percevoir n'est qu'invention. Les Carvakas refusent les Védas et leur autorité, les rituels brahmaniques, et toute forme de spéculation métaphysique. L'univers est composé des quatre éléments — terre, eau, feu et air — sans qu'intervienne aucune divinité créatrice.&lt;/p&gt;&lt;p&gt;En matière d'éthique, la philosophie Carvaka est franchement hédoniste : le plaisir est le seul bien réel, la souffrance le seul mal. Mieux vaut jouir de la vie maintenant plutôt qu'espérer une récompense illusoire après la mort. Ce réalisme sans concession en fait une voix singulière, souvent persécutée, de la pensée indienne classique.&lt;/p&gt;&lt;p&gt;Bien que ses textes originaux aient presque tous disparu — connus surtout par les réfutations de ses adversaires — son influence demeure dans les courants matérialistes et rationalistes qui traversent la philosophie indienne jusqu'à aujourd'hui.&lt;/p&gt;"/>
+    <hyperlink ref="E20" r:id="rId4" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Yoga_s%C5%ABtra&quot; title=&quot; Wikipedia&quot;&gt; Le Yoga&lt;/a&gt; en tant qu’école philosophique (darshana) est distinct de la pratique physique popularisée en Occident. Systématisé par Patanjali dans les Yoga Sutra (entre 200 av. J.-C. et 500 apr. J.-C.), il partage la métaphysique dualiste du Samkhya — Purusha (conscience) et Prakriti (matière) — mais y ajoute une méthode pratique précise pour la libération.&lt;/p&gt;&lt;p&gt;Les huit membres (ashtanga) du Yoga structurent ce chemin : discipline éthique (yama, niyama), posture (asana), maîtrise du souffle (pranayama), retrait des sens (pratyahara), concentration (dharana), méditation (dhyana) et absorption (samadhi). Chaque étape prépare la suivante dans une progression méthodique vers l’arrêt des fluctuations du mental (chitta vritti nirodha).&lt;/p&gt;&lt;p&gt;Contrairement au Samkhya, purement théorique, le Yoga de Patanjali introduit îshvara (un principe divin, seigneur particulier parmi les âmes) comme objet de concentration facultatif — une nuance théiste absente du Samkhya classique. Cette différence a nourri des siècles de commentaires et de débats entre les deux écoles sœurs.&lt;/p&gt;&lt;p&gt;Aujourd’hui mondialement diffusée, la dimension physique du yoga occulte souvent sa profondeur philosophique originelle : une discipline rigoureuse de la conscience, visant non le bien-être mais la discrimination (viveka) entre le Soi éternel et les fluctuations passagères du mental.&lt;/p&gt;"/>
+    <hyperlink ref="E22" r:id="rId5" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Bouddhisme&quot;  title=&quot; Wikipedia&quot;&gt; Le Bouddhisme&lt;/a&gt; est une tradition philosophique qui s'est développée à partir des enseignements du Bouddha, un prince indien du 5ème siècle avant JC qui a atteint l'éveil spirituel en méditant sous un arbre, maintenant connu sous le nom de l'Arbre de la Bodhi. &lt;/p&gt; &lt;p&gt;La philosophie bouddhiste repose sur le principe fondamental de la cessation de la souffrance, connu sous le nom de Nirvana, et cherche à atteindre cet état par une compréhension profonde de la nature de la réalité. &lt;/p&gt;    &lt;p&gt; Le Bouddhisme enseigne que la souffrance est causée par le désir et l'attachement aux choses matérielles et éphémères, et que la libération de la souffrance peut être atteinte par la compréhension de la nature de l'existence et de la réalité. Pour atteindre cet état de libération, le bouddhisme propose la pratique de la méditation et le développement de la sagesse, de la compassion et de la bienveillance envers tous les êtres vivants. &lt;/p&gt; &lt;p&gt; Il est également connu pour ses enseignements sur les Quatre Nobles Vérités et le Noble Chemin Octuple, qui sont considérés comme les fondements de la pratique bouddhiste. Les Quatre Nobles Vérités décrivent la nature de la souffrance, ses causes, sa cessation et le chemin menant à la cessation de la souffrance. Le Noble Chemin Octuple est une série d'étapes pratiques pour développer la sagesse, la moralité et la concentration, afin d'atteindre l'éveil spirituel. &lt;/p&gt; &lt;p&gt; En outre, la philosophie bouddhiste met l'accent sur l'interdépendance de tous les phénomènes, la nature impermanente de l'existence et la non-existence d'un soi permanent et autonome.&lt;/p&gt; &lt;audio controls title=&quot;Le Taoïsme par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/18755-11.03.2019-ITEMA_22005213-1.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt; &lt;p&gt; &lt;/p&gt;"/>
+    <hyperlink ref="E26" r:id="rId6" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/École_des_Noms&quot;  title=&quot;Wikipedia&quot;&gt;L'École des Noms&lt;/a&gt; (ming jia, 名家) est une école de philosophie chinoise qui s'est développée pendant la période des Royaumes combattants. Sa préoccupation centrale : la relation entre les mots et les choses, entre les noms et la réalité qu'ils désignent.&lt;/p&gt;&lt;p&gt;Ses représentants les plus célèbres, Gongsun Long et Hui Shi, sont connus pour leurs paradoxes vertigineux. Gongsun Long affirmait que &quot;le cheval blanc n'est pas un cheval&quot; — non par provocation, mais pour distinguer le concept général (cheval) du particulier concret (ce cheval blanc). Hui Shi proclamait que &quot;le ciel et la terre sont d'une même hauteur&quot;, explorant les limites relatives de toute catégorisation.&lt;/p&gt;&lt;p&gt;Ces réflexions sur le langage anticipent certaines problématiques de la logique et de la philosophie analytique moderne. Comment les mots nous permettent-ils — ou nous empêchent-ils — de saisir la réalité ? Toute classification n'implique-t-elle pas une distorsion du monde ?&lt;/p&gt;&lt;p&gt;Peu influente politiquement, l'École des Noms fut souvent moquée par ses contemporains confu céens et taoïstes. Mais elle constitue une contribution unique à la logique asiatique et à la philosophie du langage dans la pensée mondiale.&lt;/p&gt;"/>
+    <hyperlink ref="E27" r:id="rId7" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/S%C3%A2mkhya&quot;  title=&quot; Wikipedia&quot;&gt;Le Sâmkhya&lt;/a&gt; est l'une des plus anciennes écoles philosophiques de l'Inde, considérée comme un darshana orthodoxe de l'hindouisme. Il propose une analyse rationnelle de la réalité pour libérer l'individu du cycle des renaissances et de la souffrance. Ce système dualiste distingue deux réalités ultimes : Purusha, la conscience pure et passive (esprit, principe masculin), et Prakriti, la matière primordiale active (énergie universelle, principe féminin). Prakriti évolue sous l'influence des trois guṇas (sattva : harmonie ; rajas : activité ; tamas : inertie), générant le monde manifesté à travers 23 tattvas (principes), comme buddhi (intelligence), ahaṃkāra (ego) et les sens. &lt;/p&gt; &lt;p&gt; Il explique la création comme une transformation de Prakriti, sans recours à un dieu créateur : de l'état non manifesté (avyakta) naît le manifesté (vyakta), incluant le corps subtil qui transmigre. L'ignorance (avidyā) cause l'identification erronée du Purusha à la matière, source de souffrance (duḥkha). &lt;/p&gt; &lt;p&gt; Fondement théorique du Yoga de Patañjali, le Sâmkhya met l'accent sur la discrimination (viveka) entre Purusha et Prakriti pour atteindre la libération (kaivalya). Il influence largement la philosophie indienne, des Puranas au Vedānta. &lt;/p&gt;"/>
+    <hyperlink ref="E29" r:id="rId8" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Therav%C4%81da&quot; title=&quot;Wikipedia&quot;&gt;Le Bouddhisme Theravada&lt;/a&gt; (« École des Anciens ») est la plus ancienne forme du bouddhisme conservée jusqu'à nos jours. Héritière directe des enseignements du Bouddha historique, elle s'enracina progressivement en Asie du Sud-Est : Sri Lanka, Thaïlande, Myanmar, Cambodge, Laos.&lt;/p&gt;&lt;p&gt;Au cœur du Theravada se trouve le Pali Canon (Tipitaka), le corpus scripturaire le plus ancien du bouddhisme. Sa philosophie insiste sur la voie individuelle vers l'éveil : chaque être doit parcourir lui-même le Noble Sentier Octuple — juste compréhension, juste intention, juste parole, juste action, juste mode de vie, juste effort, juste attention, juste concentration.&lt;/p&gt;&lt;p&gt;L'idéal du Theravada est l'Arhat : le sage qui, par sa propre pratique, a éteint les &quot;feux&quot; de l'attachement, de la haine et de l'illusion, et atteint le Nirvana. Cette voie solitaire et rigoureuse contraste avec l'idéal du bodhisattva du Mahayana, qui renonce à son propre éveil pour sauver tous les êtres.&lt;/p&gt;&lt;p&gt;La méditation de pleine conscience (sati), aujourd'hui mondialement répandue, trouve ses racines dans les pratiques contemplatives du Theravada, notamment la méditation vipassana qui vise à observer directement l'impermanence, la souffrance et l'absence de soi.&lt;/p&gt;"/>
+    <hyperlink ref="E31" r:id="rId9" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Vaisheshika&quot;  title=&quot; Wikipedia&quot;&gt;Le Vaisheshika&lt;/a&gt;  est une école philosophique orthodoxe hindoue, fondée par le sage Kaṇāda, qui se distingue par son atomisme et son réalisme ontologique. Exposée dans les Vaiśeṣika Sūtra (non antérieurs à l'ère chrétienne), elle vise la libération (mokṣa) par la connaissance des catégories fondamentales de la réalité. Le système repose sur six ou sept padārthas (catégories) : dravya (substance), guṇa (qualité), karma (action/mouvement), sāmānya (universalité), viśeṣa (particularité) et samavāya (inhérence). Parmi les neuf substances, quatre sont atomiques (terre, eau, feu, air) : les paramāṇu (atomes éternels, indivisibles) s'assemblent en dyades puis en objets composites non éternels. &lt;/p&gt; &lt;p&gt; Sans dieu créateur direct, l'univers émerge de combinaisons atomiques influencées par une cause efficiente (adrisṭa, karma résiduel). Ākāśa (espace), kāla (temps), dik (direction) et cit (âme) complètent les substances ; les atomes sphériques se lient par forces intrinsèques, formant un monde discontinu mais perceptible. &lt;/p&gt; &lt;p&gt; Souvent fusionné avec le Nyâya (logique), il postule un Īśvara ordonnateur. La délivrance est un état pur de l'âme (sans qualités, conscience ou douleur), libérée des agrégats par la gnose discriminante. &lt;/p&gt;"/>
+    <hyperlink ref="E32" r:id="rId10" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Bouddhisme_mah%C4%81y%C4%81na&quot; title=&quot;Wikipedia&quot;&gt;Le Bouddhisme Mahayana&lt;/a&gt; (« Grand Véhicule ») est apparu en Inde au tournant de l'ère chrétienne, s'étendant progressivement vers la Chine, le Japon, la Corée et le Vietnam. Par rapport au Theravada, il représente une transformation profonde de la vision bouddhiste : l'éveil n'est plus un idéal solitaire mais une aspiration collective.&lt;/p&gt;&lt;p&gt;L'idéal central du Mahayana est le bodhisattva : l'être qui, sur le point d'atteindre le Nirvana, choisit de demeurer dans le cycle des renaissances (samsara) pour guider et libérer tous les êtres sensibles. Cette compassion universelle (karuna) devient le moteur de la voie spirituelle, indissociable de la sagesse (prajna).&lt;/p&gt;&lt;p&gt;Le Mahayana introduit également la notion révolutionnaire de sunyata (vacuité) : toutes choses sont dénues d'existence propre et intrinsèque — elles n'existent que de façon interdependante. Nagarjuna, au IIe siècle, en développa la philosophie dans ses Stances du Milieu, fondant l'école Madhyamaka qui influencça toute la pensée bouddhiste ultérieure.&lt;/p&gt;&lt;p&gt;C'est sur le sol du Mahayana que fleuriront le bouddhisme Zen, le bouddhisme tibétain Vajrayana, et l'École de la Terre Pure. Avec ses sutras nouveaux (Lotus, Vimalakirti, Prajnaparamita), le Mahayana offre une vision du monde d'une richesse philosophique et spirituelle sans équivalent.&lt;/p&gt;"/>
+    <hyperlink ref="E34" r:id="rId11" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Mazdakisme&quot; title=&quot;Wikipedia&quot;&gt;Le Mazdakisme&lt;/a&gt; est un mouvement religieux et social apparu en Perse sous l’Empire sassanide. Fondé par le réformateur Mazdak, ce courant tire ses origines à la fois du mazdéisme et du manichéisme, en proposant une relecture dualiste du monde axée sur la lumière et les ténèbres. &lt;/p&gt; &lt;p&gt; Contrairement aux structures sociales hiérarchisées de l’époque, le mazdakisme prônait une égalité radicale entre les individus. Mazdak soutenait que les causes des conflits humains résidaient dans la soif de richesses et de pouvoir, ce qui l'a conduit à prôner la mise en commun des biens matériels et, selon certaines sources, des femmes. &lt;/p&gt; &lt;p&gt; Cette doctrine a été perçue comme une menace par l’aristocratie et le clergé zoroastrien traditionnel, qui y voyaient une hérésie dangereuse pour l'ordre établi. Après avoir initialement bénéficié de l'intérêt de l'empereur Kavadh Ier, le mouvement fut sévèrement réprimé lors de grandes purges organisées entre 524 et 529. &lt;/p&gt; &lt;p&gt; Bien que le mazdakisme ait été marginalisé après ces persécutions, il a laissé une trace durable dans la pensée iranienne. Parfois qualifié, de manière anachronique, de mouvement proto-socialiste, son idéal de justice sociale a influencé certains courants contestataires qui se sont manifestés en Iran jusqu'au XIVe siècle environ. &lt;/p&gt; &#10;"/>
+    <hyperlink ref="E36" r:id="rId12" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Bouddhisme_vajrayana&quot;  title=&quot;Wikipedia&quot;&gt;Le Vajrayana&lt;/a&gt; (« Véhicule de Diamant ») est la troisième grande forme du bouddhisme, développée en Inde entre le VIIe et le Xe siècle, puis transmise au Tibet, en Mongolie et dans l'Himalaya. Il représente la voie tantrique du bouddhisme, utilisant des pratiques ésotériques pour accélérer le chemin vers l'éveil.&lt;/p&gt;&lt;p&gt;Là où le Theravada vise l'éveil en de nombreuses vies et le Mahayana en d'innombrables éons, le Vajrayana affirme qu'il est possible d'atteindre l'éveil en une seule vie — voire en un seul instant. Pour cela, il mobilise un arsenal de techniques : mantras, mandalas, mudras, visualisations de divinités, pratiques yogiques subtiles sur les énergies intérieures du corps.&lt;/p&gt;&lt;p&gt;Le Bouddhisme tibétain, la forme la plus répandue du Vajrayana, s'est développé dès le VIIe siècle sous le règne du roi Songtsen Gampo. Il intègre des éléments de la religion Bön préexistante et du Mahayana indien. Ses figures tutlaires — Padmasambhava, Milarepa, Tsongkhapa — sont au cœur d'une tradition d'une richesse philosophique et rituelle incomparable.&lt;/p&gt;&lt;p&gt;La notion de &quot;nature de bouddha&quot; (tathagatagarbha) — l'idée que chaque être possède en lui la graine de l'éveil — est centrale dans le Vajrayana. La pratique vise à reconnaître directement cette nature lumineuse originelle, au-delà des voiles de l'ignorance et de l'égo.&lt;/p&gt;"/>
     <hyperlink ref="E38" r:id="rId13" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/V%C3%A9danta&quot;  title=&quot; Wikipedia&quot;&gt;Le Védanta&lt;/a&gt; ou Uttara Mīmāṃsā, est l'école philosophique hindoue qui culmine les enseignements ésotériques des Upaniṣad, du Brahma Sūtra et de la Bhagavad Gītā, visant à réaliser l'unité entre l'ātman (Soi individuel) et le Brahman (Réalité absolue). C'est le couronnement des six darśanas orthodoxes, opposé à la Mīmāṃsā rituelle par son accent sur la jñāna (connaissance).https://fr.wikipedia.org/wiki/Védanta&lt;/p&gt; &lt;p&gt; Il enseigne que seul le Brahman est réel (brahma satyam), le monde est illusoire (jagat mithyā) et l'individu n'est pas différent du Brahman (jīvo brahmaiva na aparah), l'ignorance (avidyā) causant la perception de dualité via māyā. Les guṇas (sattva, rajas, tamas) conditionnent cette apparence, et la libération (mokṣa) dissout l'illusion par la discrimination. &lt;/p&gt; &lt;p&gt; L'Advaita de Śaṅkara est non-dualiste : Brahman transcende toute distinction, avec trois niveaux de réalité (pāramārthika, vyāvahārika, prātibhāsika). Le Viśiṣṭādvaita de Rāmānuja est qualifié : Dieu (Viṣṇu), âmes et matière forment un tout organique. D'autres comme Dvaita (Madhva) sont dualistes.  &lt;/p&gt; &lt;p&gt; Via jñāna-yoga (discernement), bhakti (dévotion) ou karma-yoga, il guide vers kaivalya. Influençant hindouisme moderne (Vivekananda), yoga et spiritualité globale, il dialogue avec bouddhisme et illumine l'unité sous-jacente de l'existence. &lt;/p&gt;&#10;&#10;"/>
     <hyperlink ref="E40" r:id="rId14" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Soufisme&quot; title=&quot; Wikipedia&quot;&gt; Le Soufisme &lt;/a&gt;  est un courant spirituel de l'islam qui est apparu au début de l'ère islamique, vers le VIIIe siècle. Les soufis, qui sont les adeptes du soufisme, cherchent à atteindre une relation personnelle et directe avec Dieu à travers la pratique de la méditation, de la prière, de la récitation de poèmes mystiques, de la musique et d'autres pratiques spirituelles.&lt;/p&gt; &lt;p&gt;&#10;Les racines du soufisme remontent aux premiers temps de l'islam, lorsque les premiers musulmans cherchaient à approfondir leur relation avec Dieu en se concentrant sur l'intériorité de leur être. Cependant, le soufisme en tant que courant organisé est apparu plus tard, au VIIIe siècle, avec l'émergence de maîtres spirituels (ou &quot;soufis&quot;) qui ont commencé à enseigner des méthodes spécifiques pour atteindre la proximité divine.&lt;/p&gt; &lt;p&gt; &#10;Le soufisme a connu une expansion considérable au cours des siècles suivants, en particulier en Iran, en Égypte, en Turquie, en Inde et en Asie centrale. Les soufis ont produit une riche littérature mystique, composée de poèmes, de récits et de traités qui reflètent leur quête de l'union avec Dieu. &lt;/p&gt; &lt;p&gt;&#10;Le soufisme a également été influencé par les cultures et les traditions religieuses des régions où il s'est développé, notamment le zoroastrisme, le bouddhisme, le christianisme et le judaïsme. Cette influence s'est reflétée dans la diversité des pratiques et des enseignements soufis à travers le monde musulman. &lt;/p&gt; &lt;p&gt;&#10;Malgré sa popularité et son importance historique, le soufisme a été critiqué et même persécuté par certains courants de l'islam qui le considèrent comme une innovation religieuse non autorisée. Cependant, le soufisme a continué à exister et à se développer, et il reste une force spirituelle importante dans le monde musulman contemporain.&lt;/p&gt;  &lt;audio controls title=&quot;Qu'est ce que le Soufisme ? par France Culture&quot;&gt; &lt;source src=&quot;https://cdn.radiofrance.fr/s3/cruiser-production/static/culture/sons/2015/03/s11/NET_FC_93b4dc90-9bec-4619-a90c-6e2baee39849.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt; &lt;p&gt; &lt;/p&gt;"/>
     <hyperlink ref="E44" r:id="rId15" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Confucianisme_en_Cor%C3%A9e&quot; title=&quot; Wikipedia&quot;&gt; Le Confucianisme coréen&lt;/a&gt; désigne l’adaptation et l’approfondissement du néo-confucianisme chinois sur la péninsule coréenne, en particulier durant la dynastie Joseon (1392–1910) où il devint la doctrine d’État.&lt;/p&gt;&lt;p&gt;Deux figures dominent ce courant : Yi Hwang (Toegye, 1501–1570), qui affirme la primauté du principe immatériel (li) sur la matière (ki) et fonde l’école de Yeongnam, et Yi I (Yulgok, 1536–1584), qui défend au contraire leur interdépendance dynamique. Ce débat li-ki structura la philosophie coréenne pendant des siècles.&lt;/p&gt;&lt;p&gt;Au-delà de la métaphysique, le confucianisme coréen insiste sur la formation morale du lettré (seonbi) : intégrité, sobriété, sens du devoir envers la communauté et l’État. Les académies privées (seowon) diffusèrent cet idéal éducatif dans tout le pays.&lt;/p&gt;&lt;p&gt;Son empreinte demeure profonde dans la société coréenne contemporaine : hiérarchie des âges, valorisation de l’éducation, rites familiaux et éthique du travail y trouvent encore des racines directement confucéennes.&lt;/p&gt;"/>

</xml_diff>

<commit_message>
Nouvelle page Ressources (sources, émissions France Culture et chaînes YouTube les plus utilisées, nombres calculés) ; noms de chaînes uniformisés dans les crédits ; courants, textes lot 5 (Féminisme daté de 1791) ; Darwinisme social et Eurasisme (éditeur)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-courant-pensee-oriental.xlsx
+++ b/data/frise-courant-pensee-oriental.xlsx
@@ -2476,8 +2476,10 @@
       <c r="F4" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="G4" s="11" t="s">
-        <v>20</v>
+      <c r="G4" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"La Philosophie Egyptienne" par Le Précepteur</t>
+        </is>
       </c>
       <c r="H4" s="9"/>
       <c r="I4" s="9"/>
@@ -2598,8 +2600,10 @@
       <c r="F7" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="G7" s="2" t="s">
-        <v>41</v>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mythologie Hindoue Védisme à Hindouisme par Arcana Mystères du Monde</t>
+        </is>
       </c>
       <c r="J7" s="13" t="s">
         <v>42</v>
@@ -2963,8 +2967,10 @@
       <c r="D14" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="E14" s="2" t="s">
-        <v>60</v>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Religions_m%C3%A9soam%C3%A9ricaines"  title=" Wikipedia"&gt;Le Mysticisme mésoaméricain&lt;/a&gt; désigne les conceptions religieuses et philosophiques des civilisations de Mésoamérique, du Mexique central au Guatemala : les Olmèques dès le IIe millénaire avant notre ère, puis les Mayas, les Toltèques et les Aztèques. Malgré leur diversité, elles partagent la vision d’un monde sacré, cyclique et fragile, dont l’équilibre dépend de l’action des humains. Elles nous sont connues par les codex peints, les inscriptions mayas, l’architecture des cités et les récits recueillis après la conquête espagnole.&lt;/p&gt; &lt;p&gt;Le temps y est pensé en cycles : le calendrier rituel de 260 jours et l’année solaire de 365 jours se combinent en un « siècle » de 52 ans, et les Mayas datent aussi les événements sur de très longues périodes, le « compte long », depuis une origine mythique fixée en 3114 av. J.-C. Pour les Aztèques, le monde actuel est le cinquième « Soleil », après quatre créations détruites ; les dieux se sont sacrifiés pour mettre ce soleil en mouvement, et les humains leur doivent en retour leur propre sang. Le sacrifice est ainsi pensé comme une dette cosmique, nécessaire pour que le soleil poursuive sa course. Le &lt;em&gt;Popol Vuh&lt;/em&gt;, livre sacré des Mayas quichés, raconte la création des humains, façonnés dans le maïs après plusieurs essais manqués. La figure de &lt;a href="https://fr.wikipedia.org/wiki/Quetzalc%C3%B3atl" title=" Wikipedia"&gt;Quetzalcóatl&lt;/a&gt;, le Serpent à plumes, est associée au savoir, aux arts et au calendrier.&lt;/p&gt; &lt;p&gt;Les sages aztèques, les &lt;em&gt;tlamatinime&lt;/em&gt;, s’interrogeaient sur la vérité et la fragilité de l’existence. Leur pensée a été étudiée comme une véritable philosophie par Miguel León-Portilla.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F14" s="1" t="s">
         <v>61</v>
@@ -3130,8 +3136,10 @@
       <c r="F17" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="G17" s="2" t="s">
-        <v>74</v>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"L'hésychasme prière sacrée par Mystica</t>
+        </is>
       </c>
       <c r="J17" s="2" t="s">
         <v>75</v>
@@ -3305,8 +3313,10 @@
       <c r="F21" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="G21" s="11" t="s">
-        <v>99</v>
+      <c r="G21" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"Les enseignemants de Confucius" par Film 25 Production</t>
+        </is>
       </c>
       <c r="H21" s="9"/>
       <c r="I21" s="9"/>
@@ -3688,8 +3698,10 @@
       <c r="D30" s="12" t="s">
         <v>150</v>
       </c>
-      <c r="E30" s="2" t="s">
-        <v>151</v>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/École_des_Noms"  title="Wikipedia"&gt;L’École des Noms&lt;/a&gt;, en chinois &lt;em&gt;mingjia&lt;/em&gt;, est une école de la Chine des Royaumes combattants (Ve-IIIe siècle av. J.-C.) qui s’intéresse au rapport entre les noms et les choses, c’est-à-dire entre le langage et la réalité. À une époque où les Cent Écoles débattent sans cesse, ses penseurs, appelés aussi « disputeurs », cultivent l’art de l’argumentation et du paradoxe, au point de passer pour des sophistes aux yeux de leurs adversaires. Ils prolongent à leur manière une exigence de Confucius, la « rectification des noms », qui veut que les mots s’accordent avec la réalité.&lt;/p&gt; &lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Hui_Shi" title=" Wikipedia"&gt;Hui Shi&lt;/a&gt; (IVe siècle av. J.-C.), ami et contradicteur de Zhuangzi, avance dix paradoxes sur l’espace, le temps et l’unité du monde : « le ciel est aussi bas que la terre », « je pars aujourd’hui pour Yue et j’y suis arrivé hier », ou encore « aimez tous les êtres, car le ciel et la terre ne font qu’un corps ». Ils montrent que toute distinction, grand et petit, haut et bas, dépend du point de vue. Son cadet &lt;a href="https://fr.wikipedia.org/wiki/Gongsun_Long" title=" Wikipedia"&gt;Gongsun Long&lt;/a&gt; (vers 320-250 av. J.-C.) est célèbre pour sa thèse « un cheval blanc n’est pas un cheval » : le nom « cheval blanc » désigne à la fois une forme et une couleur, il ne se confond donc pas avec le nom « cheval ». Il distingue ainsi le concept général des choses particulières, et le nom de ce qu’il désigne.&lt;/p&gt; &lt;p&gt;Raillée par les confucéens et les taoïstes, l’école disparaît avec l’empire Qin. Redécouverte au XXe siècle, elle est vue comme l’un des rares foyers de logique et de philosophie du langage de la Chine ancienne, aux côtés des logiciens moïstes. Un seul de ses livres, le &lt;em&gt;Gongsun Longzi&lt;/em&gt;, nous est parvenu, en partie.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F30" s="1" t="s">
         <v>152</v>
@@ -3863,8 +3875,10 @@
       <c r="D34" s="15" t="s">
         <v>174</v>
       </c>
-      <c r="E34" s="19" t="s">
-        <v>175</v>
+      <c r="E34" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Ny%C3%A2ya" title=" Wikipedia"&gt;Le Nyâya&lt;/a&gt;, « la règle » ou « la méthode », est l’une des six écoles orthodoxes de la philosophie indienne, celle qui s’est consacrée à la logique et à la théorie de la connaissance. Ses textes fondateurs, les &lt;em&gt;Nyāya Sūtra&lt;/em&gt;, attribués à Akṣapāda Gautama, sont composés entre le IIe siècle avant et le IIe siècle de notre ère, à partir de traditions de débat plus anciennes. Leur but reste spirituel : seule la connaissance juste délivre de la souffrance et du cycle des renaissances.&lt;/p&gt; &lt;p&gt;Le Nyâya reconnaît quatre moyens de connaissance valide (&lt;em&gt;pramāṇa&lt;/em&gt;) : la perception, l’inférence, la comparaison et le témoignage digne de foi. Il codifie l’inférence en un raisonnement à cinq membres, illustré par un exemple célèbre : la colline est en feu, parce qu’elle fume ; tout ce qui fume est en feu, comme un foyer de cuisine ; or la colline fume ; donc elle est en feu. Il dresse aussi la liste des sophismes et des ruses de la discussion. Réaliste, il soutient que le monde extérieur existe tel que nous le percevons, contre les bouddhistes. Il défend l’existence d’un Soi permanent et d’un Dieu cause du monde, notamment avec Udayana vers l’an mil. Associé à l’école &lt;a href="https://fr.wikipedia.org/wiki/Vaisheshika" title=" Wikipedia"&gt;Vaiśeṣika&lt;/a&gt;, qui lui apporte sa théorie des atomes et des catégories, il forme avec elle le Nyāya-Vaiśeṣika.&lt;/p&gt; &lt;p&gt;Au XIVe siècle, Gaṅgeśa fonde le « nouveau Nyâya » (&lt;em&gt;Navya-Nyāya&lt;/em&gt;), dont le langage technique devient l’outil commun de toute la philosophie indienne. Ses analyses de l’inférence et du témoignage ont souvent été comparées à la logique d’Aristote.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F34" s="14" t="s">
         <v>176</v>
@@ -4797,7 +4811,7 @@
       </c>
       <c r="G54" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Le SIKHISME : La religion qui affirme que "DIEU N'A PAS DE RELIGION" (Le message de l'Unité)" par MYSTICA</t>
+          <t xml:space="preserve">"Le SIKHISME : La religion qui affirme que "DIEU N'A PAS DE RELIGION" (Le message de l'Unité)" par Mystica</t>
         </is>
       </c>
       <c r="J54" s="1" t="s">
@@ -4978,8 +4992,10 @@
       <c r="F58" s="14" t="s">
         <v>310</v>
       </c>
-      <c r="G58" s="16" t="s">
-        <v>311</v>
+      <c r="G58" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fondamentalisme par Le Savoir Partagé</t>
+        </is>
       </c>
       <c r="H58" s="14"/>
       <c r="I58" s="14"/>
@@ -6035,6 +6051,16 @@
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Eurasisme" title=" Wikipedia"&gt;L’eurasisme&lt;/a&gt; est un courant de pensée né en 1921 dans l’émigration russe, après la révolution bolchevique, avec le recueil &lt;em&gt;L’Exode vers l’Orient&lt;/em&gt;, publié à Sofia par un petit groupe de jeunes intellectuels exilés : le linguiste &lt;a href="https://fr.wikipedia.org/wiki/Nikola%C3%AF_Sergue%C3%AFevitch_Troubetsko%C3%AF" title=" Wikipedia"&gt;Nikolaï Troubetskoï&lt;/a&gt;, le géographe Piotr Savitski, le musicologue Pierre Souvtchinski et le théologien Georges Florovsky.&lt;/p&gt; &lt;p&gt;Leur thèse est que la Russie n’est ni une partie de l’Europe ni une partie de l’Asie, mais un monde à part, l’« Eurasie », dont la grande plaine, des Carpates au Pacifique, a façonné l’unité des peuples slaves, turcs et finno-ougriens. Contre les occidentalistes, ils refusent l’idée d’une civilisation européenne universelle : dans &lt;em&gt;L’Europe et l’humanité&lt;/em&gt; (1920), Troubetskoï y voit l’égoïsme d’une culture « romano-germanique » qui s’impose aux autres. Contre les slavophiles, ils réhabilitent l’héritage asiatique de la Russie, et jusqu’à l’empire de Gengis Khan, qui aurait le premier unifié cet espace. Ils rêvent d’un État fondé sur une idéologie commune et sur l’orthodoxie, distinct à la fois de la démocratie libérale et du communisme. Florovsky s’en éloigne vite et critique en 1928 ce qu’il appelle une « vérité des questions » devenue une « erreur des réponses ». Le mouvement se divise à la fin des années 1920, une partie se rapprochant du régime soviétique.&lt;/p&gt; &lt;p&gt;Prolongé en URSS par l’historien &lt;a href="https://fr.wikipedia.org/wiki/Lev_Goumilev" title=" Wikipedia"&gt;Lev Goumilev&lt;/a&gt;, l’eurasisme renaît après 1991 sous la forme d’un « néo-eurasisme » porté par &lt;a href="https://fr.wikipedia.org/wiki/Alexandre_Douguine" title=" Wikipedia"&gt;Alexandre Douguine&lt;/a&gt;, idéologue d’extrême droite, et influence aujourd’hui la géopolitique nationaliste et impériale de la Russie.&lt;/p&gt;  &lt;audio controls title="De l'idée à l'action : 4 doctrines géopolitiques . Eurasie : la Russie au centre du jeu par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/18720-25.03.2021-ITEMA_22614994-2021C16756S0084.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;</t>
         </is>
       </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">QodQ2ORmtKg</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"L'EURASISME : le projet géopolitique de la Russie ? - C Ce soir du 24 février 2022" par C Ce Soir - France Télévisions</t>
+        </is>
+      </c>
       <c r="J80" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">doctrine née dans l’émigration russe : la Russie ne serait ni l’Europe ni l’Asie, mais une civilisation à part, l’« Eurasie ».</t>
@@ -6292,8 +6318,10 @@
       <c r="F85" s="1" t="s">
         <v>440</v>
       </c>
-      <c r="G85" s="2" t="s">
-        <v>441</v>
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">le consciencisme de Kwane Nkrumah par Renaissance Africaine</t>
+        </is>
       </c>
       <c r="J85" s="2" t="s">
         <v>442</v>

</xml_diff>

<commit_message>
Vidéos : 12 vidéos principales supprimées ou non intégrables remplacées ; Anticolonialisme (Césaire, France Culture) et Haskala (Henry Abramson) à la place de vidéos orientées ; crédit du Kalâm corrigé
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-courant-pensee-oriental.xlsx
+++ b/data/frise-courant-pensee-oriental.xlsx
@@ -4591,11 +4591,15 @@
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Philosophie_azt%C3%A8que" title=" Wikipedia"&gt;La Pensée nahua&lt;/a&gt; désigne la réflexion philosophique des peuples de langue nahuatl, dont les Aztèques ou Mexicas, dans le Mexique central avant la conquête espagnole de 1521. Elle était portée par les &lt;em&gt;tlamatinime&lt;/em&gt;, « ceux qui savent quelque chose », sages et maîtres du &lt;em&gt;calmecac&lt;/em&gt;, l’école où l’on formait les jeunes nobles. Nous la connaissons par des codex, des chants et des discours recueillis après la conquête, notamment par le franciscain Bernardino de Sahagún.&lt;/p&gt; &lt;p&gt;L’historien mexicain &lt;a href="https://fr.wikipedia.org/wiki/Miguel_Le%C3%B3n-Portilla" title=" Wikipedia"&gt;Miguel León-Portilla&lt;/a&gt; l’a fait connaître dans &lt;em&gt;La filosofía náhuatl estudiada en sus fuentes&lt;/em&gt; (1956). Les sages s’interrogent sur la fragilité de l’existence : sur terre tout est passager, comme les fleurs qui se fanent, et l’on se demande si quelque chose est vrai, enraciné. Leur réponse est &lt;em&gt;in xochitl in cuicatl&lt;/em&gt;, « la fleur et le chant », c’est-à-dire la poésie, seule capable peut-être de dire le vrai. Le roi &lt;a href="https://fr.wikipedia.org/wiki/Nezahualc%C3%B3yotl" title=" Wikipedia"&gt;Nezahualcóyotl&lt;/a&gt;, souverain de Texcoco au XVe siècle, auquel on attribue de nombreux poèmes, en est la grande figure. Le principe suprême, Ometeotl, « dieu de la dualité », unit le masculin et le féminin ; le monde est fait de couples complémentaires, vie et mort, ordre et désordre, en équilibre instable. Le temps est cyclique : quatre « soleils », quatre âges du monde, ont déjà été détruits, et nous vivons sous le cinquième.&lt;/p&gt; &lt;p&gt;Plus récemment, le philosophe James Maffie a lu dans le &lt;em&gt;teotl&lt;/em&gt; une énergie sacrée, unique et toujours en mouvement, dont toutes choses sont des aspects. Cette pensée est aujourd’hui étudiée comme une véritable tradition philosophique.&lt;/p&gt;</t>
         </is>
       </c>
-      <c r="F49" s="1" t="s">
-        <v>266</v>
-      </c>
-      <c r="G49" s="2" t="s">
-        <v>267</v>
+      <c r="F49" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mLi2f452GNo</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"Aztec Philosophy with James Maffie" par Hermitix Podcast</t>
+        </is>
       </c>
       <c r="J49" s="2" t="s">
         <v>268</v>
@@ -4775,11 +4779,15 @@
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Philosophie_vietnamienne" title=" Wikipedia"&gt;La Philosophie vietnamienne&lt;/a&gt; se caractérise par le Tam Giáo, les « trois enseignements » : une alliance durable entre le confucianisme, le bouddhisme et le taoïsme, à laquelle s’ajoutent le culte des ancêtres et celui des génies protecteurs des villages. Un adage vietnamien dit que « les trois enseignements ont une même source ». Chacun a son domaine : le confucianisme règle la famille et l’État, le bouddhisme la vie spirituelle, le taoïsme la médecine, la divination et les rites du quotidien.&lt;/p&gt; &lt;p&gt;Le bouddhisme arrive très tôt, dès les premiers siècles de notre ère, par la mer et par la Chine. Après l’indépendance, en 939, les dynasties Lý et Trần le favorisent : le roi &lt;a href="https://fr.wikipedia.org/wiki/Tr%E1%BA%A7n_Nh%C3%A2n_T%C3%B4ng" title=" Wikipedia"&gt;Trần Nhân Tông&lt;/a&gt;, vainqueur des invasions mongoles, abdique en 1293 pour se faire moine et fonde l’école zen de Trúc Lâm, la « Forêt de bambous », proprement vietnamienne. Le confucianisme s’impose ensuite comme doctrine de l’État : le Temple de la Littérature est fondé à Hanoï en 1070, et les concours mandarinaux recrutent les fonctionnaires jusqu’en 1919. Mais les lettrés formés aux classiques confucéens pratiquaient souvent le bouddhisme dans leur vie personnelle et se retiraient volontiers en ermites taoïstes : les trois voies se complètent plus qu’elles ne s’opposent. &lt;a href="https://fr.wikipedia.org/wiki/Nguy%E1%BB%85n_Tr%C3%A3i" title=" Wikipedia"&gt;Nguyễn Trãi&lt;/a&gt; au XVe siècle, Nguyễn Bỉnh Khiêm au XVIe ou Lê Quý Đôn au XVIIIe illustrent cette sagesse composite.&lt;/p&gt; &lt;p&gt;Au XXe siècle, ce syncrétisme inspire de nouvelles religions comme le caodaïsme, tandis que le marxisme devient la doctrine officielle. L’empreinte du Tam Giáo demeure dans les rites familiaux et la morale.&lt;/p&gt;</t>
         </is>
       </c>
-      <c r="F53" s="1" t="s">
-        <v>288</v>
-      </c>
-      <c r="G53" s="2" t="s">
-        <v>289</v>
+      <c r="F53" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NOWcduKGZYI</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"Sự khác nhau của Nho giáo, Đạo giáo và Phật giáo - Tam Giáo Đồng Nguyên là gì?" par Radio Suy Ngẫm</t>
+        </is>
       </c>
       <c r="J53" s="2" t="s">
         <v>290</v>
@@ -5929,11 +5937,15 @@
       <c r="E77" s="2" t="s">
         <v>404</v>
       </c>
-      <c r="F77" s="1" t="s">
-        <v>405</v>
-      </c>
-      <c r="G77" s="2" t="s">
-        <v>406</v>
+      <c r="F77" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">imzO0eNziD4</t>
+        </is>
+      </c>
+      <c r="G77" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"B.R. Ambedkar: The Life of the Mind &amp; a Life in Politics" par Library of Congress</t>
+        </is>
       </c>
       <c r="J77" s="2" t="s">
         <v>407</v>

</xml_diff>

<commit_message>
Textes des courants, lots 6 et 7 : 20 textes portés à 1 420-1 550 caractères (Utopisme, Instrumentalisme, École de Kyōto, Idéalisme allemand, Computationnalisme, Néoconfucianisme, Bouddhisme Theravada, Vaisheshika, Pansophisme, Éthique de la sollicitude, Falsificationnisme, Sâmkhya, Ishraqisme, Zoroastrisme, Pluralisme, Ajīvika, Transhumanisme, Scotisme, Méthodisme, Légisme) ; éditeur : référence 1 500 ± 8 % ; vidéos Jeunes hégéliens et al-Maturidi, portrait d'al-Maturidi
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-courant-pensee-oriental.xlsx
+++ b/data/frise-courant-pensee-oriental.xlsx
@@ -2555,8 +2555,10 @@
       <c r="D6" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="E6" s="2" t="s">
-        <v>34</v>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Zoroastrisme" title="Wikipedia"&gt;Le Zoroastrisme&lt;/a&gt; est la religion fondée en Iran par le prophète &lt;a href="https://fr.wikipedia.org/wiki/Zarathoustra" title=" Wikipedia"&gt;Zarathoustra&lt;/a&gt;, dont on situe la vie, selon les auteurs, entre 1500 et 600 av. J.-C. Ses hymnes, les &lt;em&gt;Gâthâs&lt;/em&gt;, forment la partie la plus ancienne de l’&lt;a href="https://fr.wikipedia.org/wiki/Avesta" title=" Wikipedia"&gt;Avesta&lt;/a&gt;, le livre sacré. Religion des empires perses, des Achéménides aux Sassanides, il est aussi l’une des premières grandes pensées du bien et du mal.&lt;/p&gt; &lt;p&gt;Zarathoustra rompt avec le polythéisme de son temps pour célébrer un dieu suprême, Ahura Mazda, le « Seigneur Sage ». Le monde est le théâtre d’un combat entre deux esprits : l’Esprit saint, du côté de la vérité et de l’ordre (&lt;em&gt;asha&lt;/em&gt;), et l’Esprit destructeur, Angra Mainyu, du côté du mensonge. Chaque être humain doit choisir son camp ; sa liberté morale est au cœur de la doctrine, résumée par la triade « bonnes pensées, bonnes paroles, bonnes actions ». Après la mort, l’âme est jugée au pont Chinvat ; à la fin des temps, un sauveur viendra, les morts ressusciteront et le mal sera vaincu. Ces idées de jugement, de résurrection et de fin des temps ont pu influencer le judaïsme tardif, puis le christianisme et l’islam.&lt;/p&gt; &lt;p&gt;Après la conquête arabe, une partie des fidèles émigre en Inde, où elle forme la communauté des Parsis. Les zoroastriens, quelques centaines de milliers aujourd’hui, entretiennent toujours le feu sacré, symbole de la lumière divine. Le manichéisme et le mazdakisme en sont issus, et Nietzsche a fait de Zarathoustra le porte-parole de sa propre pensée.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F6" s="1" t="s">
         <v>35</v>
@@ -3402,8 +3404,10 @@
       <c r="D23" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="E23" s="2" t="s">
-        <v>111</v>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Ajivika"  title="Wikipedia"&gt;L’Ajīvika&lt;/a&gt; est une école ascétique de l’Inde ancienne, fondée ou réorganisée au Ve siècle av. J.-C. par Makkhali Gosala, contemporain du Bouddha et de &lt;a href="https://fr.wikipedia.org/wiki/Mahavira" title=" Wikipedia"&gt;Mahavira&lt;/a&gt;, le fondateur du jaïnisme, dont il fut un temps le compagnon. Ses textes sont perdus : nous ne la connaissons que par ses adversaires bouddhistes et jaïns, qui en font un portrait hostile. Le nom viendrait d’&lt;em&gt;ājīva&lt;/em&gt;, « mode de vie », allusion à leur règle d’existence.&lt;/p&gt; &lt;p&gt;Sa thèse centrale est un déterminisme radical, la doctrine de la &lt;em&gt;niyati&lt;/em&gt;, le destin. Tout ce qui arrive est fixé d’avance ; l’effort, la vertu ou les rites ne changent rien. Chaque être traverse un nombre immense de renaissances, 8 400 000 grands cycles selon les sources, puis atteint la fin de la souffrance au terme prévu, comme une pelote de fil qui se déroule jusqu’au bout. Le libre arbitre est une illusion. Cette position heurte de front le bouddhisme et le jaïnisme, pour qui les actes, le karma, déterminent l’avenir et l’effort moral conduit à la délivrance. Les Ajīvikas étaient pourtant de rigoureux ascètes, souvent nus, qui pratiquaient parfois le jeûne jusqu’à la mort. Selon les textes jaïns, Gosala mourut peu après une violente querelle avec Mahavira.&lt;/p&gt; &lt;p&gt;Ils connaissent un grand rayonnement sous l’empire Maurya : &lt;a href="https://fr.wikipedia.org/wiki/Ashoka" title=" Wikipedia"&gt;Ashoka&lt;/a&gt; leur fait creuser des &lt;a href="https://fr.wikipedia.org/wiki/Grottes_de_Barabar" title=" Wikipedia"&gt;grottes dans les collines de Barabar&lt;/a&gt;. L’école décline ensuite et disparaît vers le XIVe siècle dans le sud de l’Inde. On y voit l’une des premières formes de fatalisme philosophique, comparable à certaines thèses des stoïciens.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F23" s="1" t="s">
         <v>112</v>
@@ -3750,8 +3754,10 @@
       <c r="D31" s="10" t="s">
         <v>157</v>
       </c>
-      <c r="E31" s="18" t="s">
-        <v>158</v>
+      <c r="E31" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/S%C3%A2mkhya"  title=" Wikipedia"&gt;Le Sâmkhya&lt;/a&gt;, « dénombrement », est l’une des six écoles orthodoxes de la philosophie indienne, et sans doute la plus ancienne. On l’attribue au sage légendaire &lt;a href="https://fr.wikipedia.org/wiki/Kapila" title=" Wikipedia"&gt;Kapila&lt;/a&gt;, mais son texte de référence, les &lt;em&gt;Sāṃkhya-kārikā&lt;/em&gt; d’Īśvarakṛṣṇa, date des environs du IVe siècle de notre ère. Comme les autres écoles, il cherche à délivrer l’homme de la souffrance et du cycle des renaissances par la connaissance.&lt;/p&gt; &lt;p&gt;Le Sâmkhya est un dualisme : il distingue deux principes éternels. Le &lt;em&gt;puruṣa&lt;/em&gt; est la conscience pure, immobile, simple témoin ; il y en a une infinité, une par être. La &lt;em&gt;prakṛti&lt;/em&gt; est la nature, matière première active, faite de trois qualités (&lt;em&gt;guṇa&lt;/em&gt;) : la clarté (&lt;em&gt;sattva&lt;/em&gt;), l’énergie (&lt;em&gt;rajas&lt;/em&gt;) et l’inertie (&lt;em&gt;tamas&lt;/em&gt;). Quand leur équilibre se rompt, la nature se déploie en 23 principes : l’intellect, le sens du moi, l’esprit, les sens, puis les éléments subtils et grossiers. Tout effet préexiste dans sa cause, comme l’huile dans la graine, et le monde se forme sans dieu créateur. La souffrance vient de ce que la conscience se confond avec les opérations de la nature, qu’elle ne fait que regarder ; la délivrance, l’« isolement » (&lt;em&gt;kaivalya&lt;/em&gt;), vient du discernement qui les sépare.&lt;/p&gt; &lt;p&gt;Le Sâmkhya fournit sa métaphysique au Yoga de &lt;a href="https://fr.wikipedia.org/wiki/Patanjali" title=" Wikipedia"&gt;Patañjali&lt;/a&gt;, qui en est comme la pratique, et imprègne la &lt;em&gt;Bhagavad-Gîtâ&lt;/em&gt;, la médecine āyurvédique et une grande partie de la pensée hindoue. Le Vedânta lui reproche de séparer la nature de l’Absolu, mais reprend beaucoup de ses notions.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F31" s="9" t="s">
         <v>159</v>
@@ -3796,8 +3802,10 @@
       <c r="D32" s="12" t="s">
         <v>162</v>
       </c>
-      <c r="E32" s="2" t="s">
-        <v>163</v>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/L%C3%A9gisme" title="Wikipedia"&gt;Le Légisme&lt;/a&gt;, en chinois &lt;em&gt;fajia&lt;/em&gt;, « école de la loi », est une philosophie politique de la Chine des Royaumes combattants (Ve-IIIe siècle av. J.-C.). À une époque de guerres incessantes, ses penseurs, souvent ministres, cherchent comment rendre un État riche et puissant. Contre les confucéens, qui veulent gouverner par la vertu et les rites, ils affirment que seule la loi, écrite, publique et appliquée à tous, peut assurer l’ordre.&lt;/p&gt; &lt;p&gt;Au IVe siècle av. J.-C., &lt;a href="https://fr.wikipedia.org/wiki/Shang_Yang" title=" Wikipedia"&gt;Shang Yang&lt;/a&gt; réforme le royaume de Qin : il encourage l’agriculture et la guerre, supprime les privilèges de la noblesse héréditaire et instaure des récompenses et des châtiments rigoureux, avec une responsabilité collective des familles. Shen Buhai insiste sur l’art de contrôler les fonctionnaires, Shen Dao sur la position de pouvoir. &lt;a href="https://fr.wikipedia.org/wiki/Han_Fei" title=" Wikipedia"&gt;Han Fei&lt;/a&gt; (vers 280-233 av. J.-C.), disciple du confucéen Xunzi, réunit la loi, la technique et la position en une doctrine complète. Puisque les hommes recherchent leur intérêt, inutile d’en appeler à leur bonté : le souverain doit les gouverner par la crainte et l’intérêt, rester secret et impénétrable, et faire fonctionner l’État comme une machine qui marche seule.&lt;/p&gt; &lt;p&gt;Le légisme triomphe quand &lt;a href="https://fr.wikipedia.org/wiki/Qin_Shi_Huang" title=" Wikipedia"&gt;Qin Shi Huang&lt;/a&gt; unifie la Chine en 221 av. J.-C. et fait brûler les livres des autres écoles. Discrédité par la chute rapide des Qin, il survit en pratique dans l’administration impériale, sous un vernis confucéen. Dans les années 1970, la campagne maoïste « contre Lin Biao et Confucius » en fait encore l’éloge.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F32" s="1" t="s">
         <v>164</v>
@@ -3840,8 +3848,10 @@
       <c r="D33" s="12" t="s">
         <v>168</v>
       </c>
-      <c r="E33" s="2" t="s">
-        <v>169</v>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Therav%C4%81da" title="Wikipedia"&gt;Le Bouddhisme Theravada&lt;/a&gt;, « l’enseignement des Anciens », est la plus ancienne forme du bouddhisme encore vivante. Il se réclame des premiers disciples du Bouddha et se transmet en pali. Sous le règne d’&lt;a href="https://fr.wikipedia.org/wiki/Ashoka" title=" Wikipedia"&gt;Ashoka&lt;/a&gt;, au IIIe siècle av. J.-C., le moine Mahinda l’introduit à Sri Lanka, d’où il gagne la Birmanie, la Thaïlande, le Cambodge et le Laos, où il reste majoritaire.&lt;/p&gt; &lt;p&gt;Ses textes forment le Canon pali, ou &lt;em&gt;Tipitaka&lt;/em&gt; (« trois corbeilles ») : la discipline monastique, les discours du Bouddha et l’&lt;em&gt;Abhidhamma&lt;/em&gt;, analyse philosophique des phénomènes, mis par écrit à Sri Lanka au Ier siècle av. J.-C. Au Ve siècle, &lt;a href="https://fr.wikipedia.org/wiki/Buddhaghosa" title=" Wikipedia"&gt;Buddhaghosa&lt;/a&gt; en donne la synthèse dans le &lt;em&gt;Chemin de la pureté&lt;/em&gt;. L’enseignement repose sur les quatre nobles vérités : la souffrance, son origine dans le désir, sa cessation et le Noble Sentier octuple qui y mène. Tout ce qui existe est impermanent, insatisfaisant et dépourvu de soi : la personne n’est qu’un assemblage changeant de cinq agrégats. L’idéal est l’&lt;em&gt;arhat&lt;/em&gt;, qui a éteint par sa propre pratique les feux du désir, de la haine et de l’illusion, alors que le Mahayana met en avant le bodhisattva, qui se consacre au salut de tous les êtres.&lt;/p&gt; &lt;p&gt;La méditation vipassana, « vision pénétrante », qui observe l’apparition et la disparition des phénomènes, a été remise à l’honneur en Birmanie au XXe siècle par des maîtres comme Mahasi Sayadaw ; elle a inspiré la « pleine conscience » répandue en Occident.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F33" s="1" t="s">
         <v>170</v>
@@ -3934,8 +3944,10 @@
       <c r="D35" s="10" t="s">
         <v>180</v>
       </c>
-      <c r="E35" s="18" t="s">
-        <v>181</v>
+      <c r="E35" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Vaisheshika"  title=" Wikipedia"&gt;Le Vaisheshika&lt;/a&gt;, de &lt;em&gt;viśeṣa&lt;/em&gt;, « particularité », est l’une des six écoles orthodoxes de la philosophie indienne. Ses &lt;em&gt;Vaiśeṣika Sūtra&lt;/em&gt; sont attribués au sage Kaṇāda, dont le nom signifierait « mangeur de grains », et datent sans doute des débuts de notre ère. Son but est la délivrance (&lt;em&gt;mokṣa&lt;/em&gt;), que procure la connaissance exacte des catégories du réel. Le système est surtout connu par le traité de Praśastapāda (VIe siècle), qui l’organise et le complète.&lt;/p&gt; &lt;p&gt;Le Vaisheshika classe tout ce qui existe en six catégories (&lt;em&gt;padārtha&lt;/em&gt;), auxquelles on ajoute plus tard la non-existence : la substance, la qualité, l’action, l’universel, la particularité et l’inhérence, relation qui unit par exemple une qualité à sa substance. Il compte neuf substances : la terre, l’eau, le feu et l’air, faits d’atomes éternels et indivisibles (&lt;em&gt;paramāṇu&lt;/em&gt;), puis l’éther, le temps, l’espace, l’âme et le sens interne. Les atomes s’assemblent par deux, puis par trois, pour former les objets visibles, qui eux sont périssables. Leurs mouvements sont guidés par l’&lt;em&gt;adṛṣṭa&lt;/em&gt;, la force invisible des actes passés ; les auteurs plus tardifs y ajoutent un Dieu ordonnateur, Īśvara. L’âme délivrée retrouve un état pur, sans plaisir ni douleur, car toute qualité liée au corps a cessé.&lt;/p&gt; &lt;p&gt;Très tôt associé au Nyâya, qui lui apporte sa logique, il forme avec lui le Nyāya-Vaiśeṣika. Son atomisme a souvent été comparé à celui de &lt;a href="https://fr.wikipedia.org/wiki/D%C3%A9mocrite" title=" Wikipedia"&gt;Démocrite&lt;/a&gt; ; mais là où Démocrite voyait le hasard, le Vaisheshika voit un ordre moral.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F35" s="9" t="s">
         <v>182</v>
@@ -4638,8 +4650,10 @@
       <c r="D50" s="12" t="s">
         <v>269</v>
       </c>
-      <c r="E50" s="2" t="s">
-        <v>270</v>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Ishraqisme"  title="Wikipedia"&gt;L’Ishraqisme&lt;/a&gt;, ou philosophie de l’Illumination (&lt;em&gt;ishrâq&lt;/em&gt;, le lever du soleil), est le courant fondé par le penseur persan &lt;a href="https://fr.wikipedia.org/wiki/Sohrawardi" title=" Wikipedia"&gt;Sohrawardi&lt;/a&gt; (1154-1191). Dans son &lt;em&gt;Livre de la sagesse orientale&lt;/em&gt;, où l’« Orient » désigne la source de la lumière plutôt qu’un lieu, il veut unir la philosophie grecque, en particulier Platon et le néoplatonisme, la sagesse de l’ancienne Perse et la mystique soufie en une vision fondée sur la lumière.&lt;/p&gt; &lt;p&gt;Pour Sohrawardi, toute la réalité est un déploiement de la Lumière des lumières, qui est Dieu. Les êtres s’ordonnent selon leur degré de lumière, des intelligences angéliques jusqu’aux ténèbres de la matière, qui n’est que lumière absente. La connaissance véritable n’est pas d’abord un raisonnement : c’est une « connaissance par présence », immédiate, comme celle que l’âme a d’elle-même. Elle s’acquiert par la purification et l’expérience spirituelle autant que par la logique, et Sohrawardi critique sur ce point Avicenne. Il décrit aussi un monde intermédiaire entre l’esprit et le corps, le monde des images, où se situent les visions des prophètes et des mystiques. Ses récits symboliques, comme &lt;em&gt;Le Bruissement des ailes de Gabriel&lt;/em&gt;, racontent l’exil de l’âme et son retour vers l’Orient de la lumière.&lt;/p&gt; &lt;p&gt;Accusé d’hérésie par les juristes, il est exécuté à Alep avec l’accord de Saladin, d’où son surnom de « maître tué » (&lt;em&gt;al-maqtûl&lt;/em&gt;). Sa pensée nourrit pourtant l’école d’Ispahan et &lt;a href="https://fr.wikipedia.org/wiki/Molla_Sadra_Chirazi" title=" Wikipedia"&gt;Mollâ Sadrâ&lt;/a&gt;. &lt;a href="https://fr.wikipedia.org/wiki/Henry_Corbin" title=" Wikipedia"&gt;Henry Corbin&lt;/a&gt; l’a fait connaître en Occident au XXe siècle, en le traduisant et en le commentant.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F50" s="1" t="s">
         <v>271</v>
@@ -4686,8 +4700,10 @@
       <c r="D51" s="10" t="s">
         <v>275</v>
       </c>
-      <c r="E51" s="22" t="s">
-        <v>276</v>
+      <c r="E51" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/N%C3%A9oconfucianisme"  title=" Wikipedia"&gt;Le Néoconfucianisme&lt;/a&gt; est le renouveau du confucianisme qui s’épanouit en Chine sous la dynastie Song (960-1279). Face au bouddhisme et au taoïsme, qui offraient une métaphysique et une spiritualité plus riches, des lettrés relisent les Classiques pour donner à la morale confucéenne un fondement cosmique. Devenu orthodoxie d’État, il domine la Chine jusqu’en 1905, ainsi que la Corée, le Japon et le Vietnam.&lt;/p&gt; &lt;p&gt;Zhou Dunyi médite sur le « Faîte suprême » d’où naissent le yin et le yang ; les frères Cheng distinguent en toute chose le &lt;em&gt;li&lt;/em&gt;, principe ou ordre rationnel, et le &lt;em&gt;qi&lt;/em&gt;, souffle ou énergie matérielle. &lt;a href="https://fr.wikipedia.org/wiki/Zhu_Xi" title=" Wikipedia"&gt;Zhu Xi&lt;/a&gt; (1130-1200) fait la synthèse de cette « école du Principe » : chaque être porte en lui le principe universel, et la nature humaine est bonne, comme le disait Mencius, mais obscurcie par un souffle impur. On se perfectionne par l’« investigation des choses », l’étude et la méditation assise. Ses commentaires des Quatre Livres servent de base aux examens impériaux de 1313 à 1905. Contre lui, Lu Jiuyuan puis &lt;a href="https://fr.wikipedia.org/wiki/Wang_Yangming" title=" Wikipedia"&gt;Wang Yangming&lt;/a&gt; (1472-1529) fondent l’« école du Cœur » : le principe n’est pas à chercher dans les choses mais dans le cœur, et la connaissance est inséparable de l’action.&lt;/p&gt; &lt;p&gt;Critiqué au XVIIIe siècle par l’école des études critiques, le &lt;em&gt;kaozheng&lt;/em&gt;, puis par la modernisation, il inspire encore au XXe siècle le « nouveau confucianisme ». En Corée, Yi Hwang et Yi I en débattent au XVIe siècle, et au Japon la doctrine de Zhu Xi devient celle du shogunat Tokugawa.&lt;/p&gt;</t>
+        </is>
       </c>
       <c r="F51" s="9" t="s">
         <v>277</v>
@@ -5889,8 +5905,10 @@
       <c r="D76" s="12" t="s">
         <v>396</v>
       </c>
-      <c r="E76" s="2" t="s">
-        <v>397</v>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/%C3%89cole_de_Ky%C5%8Dto"  title=" Wikipedia"&gt;L’école de Kyōto&lt;/a&gt; désigne le premier grand courant de philosophie moderne né au Japon, autour de &lt;a href="https://fr.wikipedia.org/wiki/Kitar%C5%8D_Nishida" title=" Wikipedia"&gt;Kitarō Nishida&lt;/a&gt; (1870-1945) et de ses successeurs à l’université impériale de Kyōto. On en fixe souvent le point de départ à 1911, date de la &lt;em&gt;Recherche sur le bien&lt;/em&gt;, où Nishida part de l’« expérience pure », antérieure à la séparation du sujet et de l’objet.&lt;/p&gt; &lt;p&gt;Ses penseurs, formés à la philosophie allemande, de Kant et Hegel à Husserl et Heidegger, veulent exprimer dans le langage de la philosophie occidentale l’expérience spirituelle de l’Asie, en particulier celle du bouddhisme zen et de la Terre pure. Au centre de leur réflexion se trouve la notion de « néant absolu » : non pas un simple manque, mais le fond ouvert d’où tout surgit, que Nishida pense comme le « lieu » (&lt;em&gt;basho&lt;/em&gt;) de toute réalité. Tanabe Hajime en tire une « philosophie de la repentance », et &lt;a href="https://fr.wikipedia.org/wiki/Keiji_Nishitani" title=" Wikipedia"&gt;Nishitani Keiji&lt;/a&gt; affronte le nihilisme européen : on ne le surmonte qu’en le traversant jusqu’à la vacuité. Watsuji Tetsurō et Kuki Shūzō, proches du groupe, l’ouvrent à l’éthique et à l’esthétique.&lt;/p&gt; &lt;p&gt;Plusieurs de ses membres furent compromis dans la justification idéologique de la guerre du Pacifique, ce qui a longtemps pesé sur sa réception. Depuis les années 1980, l’école est étudiée dans le monde entier comme le lieu d’un dialogue majeur entre la philosophie occidentale et les traditions spirituelles d’Asie. Ueda Shizuteru, mort en 2019, en a prolongé la pensée jusqu’à notre siècle.&lt;/p&gt;  &lt;audio controls title="Philosophie japonaise: l’école de Kyôto par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/10467-15.11.2013-ITEMA_20549374-2013C12410E0320-NET_FC_EE7092B3-7D80-40AA-947D-AFAD338FBA01-21.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;</t>
+        </is>
       </c>
       <c r="F76" s="1" t="s">
         <v>398</v>

</xml_diff>